<commit_message>
docs: plan UT coverage for test baseline
</commit_message>
<xml_diff>
--- a/docs/04-测试文档/手工测试用例/测试用例基线.xlsx
+++ b/docs/04-测试文档/手工测试用例/测试用例基线.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <name val="宋体"/>
       <charset val="134"/>
@@ -180,8 +180,11 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill/>
     </fill>
@@ -384,6 +387,11 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399976"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -667,7 +675,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -682,6 +690,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1275,7 +1289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H106"/>
+  <dimension ref="A1:J106"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14" defaultRowHeight="13.5"/>
   <cols>
     <col width="9.25" customWidth="1" style="1" min="1" max="1"/>
@@ -1286,6 +1300,8 @@
     <col width="51.375" customWidth="1" style="1" min="6" max="6"/>
     <col width="45.75" customWidth="1" style="1" min="7" max="7"/>
     <col width="8.625" customWidth="1" style="1" min="8" max="8"/>
+    <col width="36" customWidth="1" style="1" min="9" max="9"/>
+    <col width="80" customWidth="1" style="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="1">
@@ -1329,6 +1345,16 @@
           <t>实际结果</t>
         </is>
       </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>UT覆盖状态</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>UT覆盖位置/不覆盖原因</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="42.75" customHeight="1" s="1">
       <c r="A2" s="4" t="inlineStr">
@@ -1370,6 +1396,16 @@
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr"/>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>不补UT</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="inlineStr">
+        <is>
+          <t>应用默认页渲染场景，不进入本轮 UT 补充范围。</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="28.5" customHeight="1" s="1">
       <c r="A3" s="4" t="inlineStr">
@@ -1410,6 +1446,16 @@
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr"/>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/dashboard/viewmodel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="28.5" customHeight="1" s="1">
       <c r="A4" s="4" t="inlineStr">
@@ -1450,6 +1496,16 @@
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr"/>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/dashboard/viewmodel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="28.5" customHeight="1" s="1">
       <c r="A5" s="4" t="inlineStr">
@@ -1490,6 +1546,16 @@
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr"/>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/dashboard/viewmodel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="42.75" customHeight="1" s="1">
       <c r="A6" s="4" t="inlineStr">
@@ -1530,6 +1596,16 @@
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr"/>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>不补UT</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>快捷入口真实跳转属于导航/页面交互场景，不进入本轮 UT 补充范围。</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="42.75" customHeight="1" s="1">
       <c r="A7" s="4" t="inlineStr">
@@ -1571,6 +1647,16 @@
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr"/>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/dashboard/viewmodel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="42.75" customHeight="1" s="1">
       <c r="A8" s="4" t="inlineStr">
@@ -1612,6 +1698,16 @@
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr"/>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/service.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="42.75" customHeight="1" s="1">
       <c r="A9" s="4" t="inlineStr">
@@ -1653,6 +1749,16 @@
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr"/>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/service.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="28.5" customHeight="1" s="1">
       <c r="A10" s="4" t="inlineStr">
@@ -1693,6 +1799,16 @@
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr"/>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/service.test.ets；entry/src/test/firewall/mode-strategy.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="28.5" customHeight="1" s="1">
       <c r="A11" s="4" t="inlineStr">
@@ -1733,6 +1849,16 @@
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr"/>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/service.test.ets；entry/src/test/firewall/mode-strategy.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="42.75" customHeight="1" s="1">
       <c r="A12" s="4" t="inlineStr">
@@ -1775,6 +1901,16 @@
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr"/>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>不补UT</t>
+        </is>
+      </c>
+      <c r="J12" s="7" t="inlineStr">
+        <is>
+          <t>模式卡片不可选择属于页面禁用态，不进入本轮 UT 补充范围。</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="42.75" customHeight="1" s="1">
       <c r="A13" s="4" t="inlineStr">
@@ -1816,6 +1952,16 @@
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr"/>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>不补UT</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>模式卡片展示完整属于页面渲染场景，不进入本轮 UT 补充范围。</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="28.5" customHeight="1" s="1">
       <c r="A14" s="4" t="inlineStr">
@@ -1856,6 +2002,16 @@
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr"/>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>不补UT</t>
+        </is>
+      </c>
+      <c r="J14" s="7" t="inlineStr">
+        <is>
+          <t>进入规则详情页属于导航场景，不进入本轮 UT 补充范围。</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="28.5" customHeight="1" s="1">
       <c r="A15" s="4" t="inlineStr">
@@ -1896,6 +2052,16 @@
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr"/>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>不补UT</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>空状态展示属于页面渲染场景；service 层空数组返回已有基础支撑，不再补 UT。</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="71.25" customHeight="1" s="1">
       <c r="A16" s="4" t="inlineStr">
@@ -1944,6 +2110,16 @@
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr"/>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J16" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/rule-utils.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="71.25" customHeight="1" s="1">
       <c r="A17" s="4" t="inlineStr">
@@ -1990,6 +2166,16 @@
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr"/>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/rule-utils.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="42.75" customHeight="1" s="1">
       <c r="A18" s="4" t="inlineStr">
@@ -2036,6 +2222,16 @@
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr"/>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/rule-utils.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="28.5" customHeight="1" s="1">
       <c r="A19" s="4" t="inlineStr">
@@ -2082,6 +2278,16 @@
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr"/>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/rule-utils.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="42.75" customHeight="1" s="1">
       <c r="A20" s="4" t="inlineStr">
@@ -2125,6 +2331,16 @@
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr"/>
+      <c r="I20" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J20" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/service.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="28.5" customHeight="1" s="1">
       <c r="A21" s="4" t="inlineStr">
@@ -2165,6 +2381,16 @@
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr"/>
+      <c r="I21" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/service.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="28.5" customHeight="1" s="1">
       <c r="A22" s="4" t="inlineStr">
@@ -2207,6 +2433,16 @@
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr"/>
+      <c r="I22" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J22" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/rule-utils.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="28.5" customHeight="1" s="1">
       <c r="A23" s="4" t="inlineStr">
@@ -2250,6 +2486,16 @@
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr"/>
+      <c r="I23" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J23" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/rule-utils.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="28.5" customHeight="1" s="1">
       <c r="A24" s="4" t="inlineStr">
@@ -2293,6 +2539,16 @@
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr"/>
+      <c r="I24" s="7" t="inlineStr">
+        <is>
+          <t>待补UT</t>
+        </is>
+      </c>
+      <c r="J24" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/rule-utils.test.ets：补 wildcard 单级域名重叠判定。</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="85.5" customHeight="1" s="1">
       <c r="A25" s="4" t="inlineStr">
@@ -2338,6 +2594,16 @@
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr"/>
+      <c r="I25" s="7" t="inlineStr">
+        <is>
+          <t>待补UT</t>
+        </is>
+      </c>
+      <c r="J25" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/service.test.ets：补用户级白名单策略下发 + PIN 成功/失败。</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="85.5" customHeight="1" s="1">
       <c r="A26" s="4" t="inlineStr">
@@ -2383,6 +2649,16 @@
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr"/>
+      <c r="I26" s="7" t="inlineStr">
+        <is>
+          <t>待补UT</t>
+        </is>
+      </c>
+      <c r="J26" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/service.test.ets：补用户级黑名单策略下发 + PIN 成功/失败。</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="85.5" customHeight="1" s="1">
       <c r="A27" s="4" t="inlineStr">
@@ -2428,6 +2704,16 @@
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr"/>
+      <c r="I27" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J27" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/rule-utils.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="42.75" customHeight="1" s="1">
       <c r="A28" s="4" t="inlineStr">
@@ -2472,6 +2758,16 @@
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr"/>
+      <c r="I28" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J28" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/rule-utils.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="28.5" customHeight="1" s="1">
       <c r="A29" s="4" t="inlineStr">
@@ -2512,6 +2808,16 @@
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr"/>
+      <c r="I29" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/service.test.ets；entry/src/test/firewall/mode-strategy.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="28.5" customHeight="1" s="1">
       <c r="A30" s="4" t="inlineStr">
@@ -2552,6 +2858,16 @@
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr"/>
+      <c r="I30" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J30" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/service.test.ets；entry/src/test/firewall/mode-strategy.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="42.75" customHeight="1" s="1">
       <c r="A31" s="4" t="inlineStr">
@@ -2593,6 +2909,16 @@
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr"/>
+      <c r="I31" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J31" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/service.test.ets；entry/src/test/firewall/mode-strategy.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="42.75" customHeight="1" s="1">
       <c r="A32" s="4" t="inlineStr">
@@ -2634,6 +2960,16 @@
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr"/>
+      <c r="I32" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J32" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/service.test.ets；entry/src/test/firewall/mode-strategy.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="71.25" customHeight="1" s="1">
       <c r="A33" s="4" t="inlineStr">
@@ -2678,6 +3014,16 @@
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr"/>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>待补UT</t>
+        </is>
+      </c>
+      <c r="J33" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/entryability/entryability.test.ets；entry/src/test/firewall/system-user-provider.test.ets：补账户新增/删除事件分发与可用用户列表更新。</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="71.25" customHeight="1" s="1">
       <c r="A34" s="4" t="inlineStr">
@@ -2722,6 +3068,16 @@
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr"/>
+      <c r="I34" s="7" t="inlineStr">
+        <is>
+          <t>待补UT</t>
+        </is>
+      </c>
+      <c r="J34" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/entryability/entryability.test.ets；entry/src/test/firewall/system-user-provider.test.ets：补账户新增/删除事件分发与可用用户列表更新。</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="71.25" customHeight="1" s="1">
       <c r="A35" s="4" t="inlineStr">
@@ -2766,6 +3122,16 @@
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr"/>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>待补UT</t>
+        </is>
+      </c>
+      <c r="J35" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/entryability/entryability.test.ets；entry/src/test/firewall/system-user-provider.test.ets：补账户新增/删除事件分发与可用用户列表更新。</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="71.25" customHeight="1" s="1">
       <c r="A36" s="4" t="inlineStr">
@@ -2810,6 +3176,16 @@
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr"/>
+      <c r="I36" s="7" t="inlineStr">
+        <is>
+          <t>待补UT</t>
+        </is>
+      </c>
+      <c r="J36" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/entryability/entryability.test.ets；entry/src/test/firewall/system-user-provider.test.ets：补账户新增/删除事件分发与可用用户列表更新。</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="28.5" customHeight="1" s="1">
       <c r="A37" s="4" t="inlineStr">
@@ -2850,6 +3226,16 @@
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr"/>
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J37" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/log-manage/list-viewmodel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="42.75" customHeight="1" s="1">
       <c r="A38" s="4" t="inlineStr">
@@ -2892,6 +3278,16 @@
         </is>
       </c>
       <c r="H38" s="5" t="inlineStr"/>
+      <c r="I38" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J38" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/log-manage/audit-source.test.ets；entry/src/test/log-manage/collector-service.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="42.75" customHeight="1" s="1">
       <c r="A39" s="4" t="inlineStr">
@@ -2935,6 +3331,16 @@
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr"/>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J39" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/log-manage/audit-source.test.ets；entry/src/test/log-manage/collector-service.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="28.5" customHeight="1" s="1">
       <c r="A40" s="4" t="inlineStr">
@@ -2977,6 +3383,16 @@
         </is>
       </c>
       <c r="H40" s="5" t="inlineStr"/>
+      <c r="I40" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J40" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/log-manage/audit-source.test.ets；entry/src/test/log-manage/crash-source.test.ets；entry/src/test/log-manage/entry-normalizer.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="28.5" customHeight="1" s="1">
       <c r="A41" s="4" t="inlineStr">
@@ -3018,6 +3434,16 @@
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr"/>
+      <c r="I41" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J41" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/log-manage/list-viewmodel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="28.5" customHeight="1" s="1">
       <c r="A42" s="4" t="inlineStr">
@@ -3059,6 +3485,16 @@
         </is>
       </c>
       <c r="H42" s="5" t="inlineStr"/>
+      <c r="I42" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J42" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/log-manage/list-viewmodel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="28.5" customHeight="1" s="1">
       <c r="A43" s="4" t="inlineStr">
@@ -3100,6 +3536,16 @@
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr"/>
+      <c r="I43" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J43" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/log-manage/list-viewmodel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="42.75" customHeight="1" s="1">
       <c r="A44" s="4" t="inlineStr">
@@ -3142,6 +3588,16 @@
         </is>
       </c>
       <c r="H44" s="5" t="inlineStr"/>
+      <c r="I44" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J44" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/log-manage/list-viewmodel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="28.5" customHeight="1" s="1">
       <c r="A45" s="4" t="inlineStr">
@@ -3182,6 +3638,16 @@
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr"/>
+      <c r="I45" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J45" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/log-manage/list-viewmodel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="42.75" customHeight="1" s="1">
       <c r="A46" s="4" t="inlineStr">
@@ -3223,6 +3689,16 @@
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr"/>
+      <c r="I46" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J46" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/log-manage/list-viewmodel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="42.75" customHeight="1" s="1">
       <c r="A47" s="4" t="inlineStr">
@@ -3264,6 +3740,16 @@
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr"/>
+      <c r="I47" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J47" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/log-manage/list-viewmodel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="42.75" customHeight="1" s="1">
       <c r="A48" s="4" t="inlineStr">
@@ -3305,6 +3791,16 @@
         </is>
       </c>
       <c r="H48" s="5" t="inlineStr"/>
+      <c r="I48" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J48" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/log-manage/export-service.test.ets；entry/src/test/log-manage/list-viewmodel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="28.5" customHeight="1" s="1">
       <c r="A49" s="4" t="inlineStr">
@@ -3344,6 +3840,16 @@
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr"/>
+      <c r="I49" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J49" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/log-manage/export-service.test.ets；entry/src/test/log-manage/list-viewmodel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="42.75" customHeight="1" s="1">
       <c r="A50" s="4" t="inlineStr">
@@ -3385,6 +3891,16 @@
         </is>
       </c>
       <c r="H50" s="5" t="inlineStr"/>
+      <c r="I50" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J50" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/log-manage/settings-viewmodel.test.ets；entry/src/test/log-manage/maintenance-service.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="42.75" customHeight="1" s="1">
       <c r="A51" s="4" t="inlineStr">
@@ -3426,6 +3942,16 @@
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr"/>
+      <c r="I51" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J51" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/log-manage/settings-viewmodel.test.ets；entry/src/test/log-manage/maintenance-service.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="28.5" customHeight="1" s="1">
       <c r="A52" s="4" t="inlineStr">
@@ -3466,6 +3992,16 @@
         </is>
       </c>
       <c r="H52" s="5" t="inlineStr"/>
+      <c r="I52" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J52" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/log-manage/list-viewmodel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="28.5" customHeight="1" s="1">
       <c r="A53" s="4" t="inlineStr">
@@ -3506,6 +4042,16 @@
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr"/>
+      <c r="I53" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J53" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/log-manage/audit-source.test.ets；entry/src/test/log-manage/collector-service.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="28.5" customHeight="1" s="1">
       <c r="A54" s="4" t="inlineStr">
@@ -3547,6 +4093,16 @@
         </is>
       </c>
       <c r="H54" s="5" t="inlineStr"/>
+      <c r="I54" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J54" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/log-manage/crash-source.test.ets；entry/src/test/log-manage/collector-service.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="28.5" customHeight="1" s="1">
       <c r="A55" s="4" t="inlineStr">
@@ -3586,6 +4142,16 @@
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr"/>
+      <c r="I55" s="7" t="inlineStr">
+        <is>
+          <t>不补UT</t>
+        </is>
+      </c>
+      <c r="J55" s="7" t="inlineStr">
+        <is>
+          <t>默认页签展示属于页面渲染场景，不进入本轮 UT 补充范围。</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="28.5" customHeight="1" s="1">
       <c r="A56" s="4" t="inlineStr">
@@ -3626,6 +4192,16 @@
         </is>
       </c>
       <c r="H56" s="5" t="inlineStr"/>
+      <c r="I56" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J56" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/viewmodels/InterfaceControlViewModel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="28.5" customHeight="1" s="1">
       <c r="A57" s="4" t="inlineStr">
@@ -3666,6 +4242,16 @@
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr"/>
+      <c r="I57" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J57" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/viewmodels/InterfaceControlViewModel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="28.5" customHeight="1" s="1">
       <c r="A58" s="4" t="inlineStr">
@@ -3706,6 +4292,16 @@
         </is>
       </c>
       <c r="H58" s="5" t="inlineStr"/>
+      <c r="I58" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J58" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/viewmodels/InterfaceControlViewModel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="28.5" customHeight="1" s="1">
       <c r="A59" s="4" t="inlineStr">
@@ -3746,6 +4342,16 @@
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr"/>
+      <c r="I59" s="7" t="inlineStr">
+        <is>
+          <t>待补UT</t>
+        </is>
+      </c>
+      <c r="J59" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/viewmodels/InterfaceControlViewModel.test.ets：补 USB 存储禁止访问 prohibited/disabled 分支。</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="28.5" customHeight="1" s="1">
       <c r="A60" s="4" t="inlineStr">
@@ -3786,6 +4392,16 @@
         </is>
       </c>
       <c r="H60" s="5" t="inlineStr"/>
+      <c r="I60" s="7" t="inlineStr">
+        <is>
+          <t>待补UT</t>
+        </is>
+      </c>
+      <c r="J60" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/viewmodels/InterfaceControlViewModel.test.ets：补 USB 接口禁用时 USB 存储策略冲突拒绝。</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="42.75" customHeight="1" s="1">
       <c r="A61" s="4" t="inlineStr">
@@ -3826,6 +4442,16 @@
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr"/>
+      <c r="I61" s="7" t="inlineStr">
+        <is>
+          <t>待补UT</t>
+        </is>
+      </c>
+      <c r="J61" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/viewmodels/InterfaceControlViewModel.test.ets：补蓝牙接口策略切换。</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="28.5" customHeight="1" s="1">
       <c r="A62" s="4" t="inlineStr">
@@ -3866,6 +4492,16 @@
         </is>
       </c>
       <c r="H62" s="5" t="inlineStr"/>
+      <c r="I62" s="7" t="inlineStr">
+        <is>
+          <t>待补UT</t>
+        </is>
+      </c>
+      <c r="J62" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/viewmodels/InterfaceControlViewModel.test.ets：补 Wi-Fi 接口策略切换。</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="42" customHeight="1" s="1">
       <c r="A63" s="4" t="inlineStr">
@@ -3907,6 +4543,16 @@
         </is>
       </c>
       <c r="H63" s="5" t="inlineStr"/>
+      <c r="I63" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J63" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/peripheral/connection-record-usb-consumer.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="28.5" customHeight="1" s="1">
       <c r="A64" s="4" t="inlineStr">
@@ -3947,6 +4593,16 @@
         </is>
       </c>
       <c r="H64" s="5" t="inlineStr"/>
+      <c r="I64" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J64" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/peripheral/connection-record-usb-consumer.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="28.5" customHeight="1" s="1">
       <c r="A65" s="4" t="inlineStr">
@@ -3987,6 +4643,16 @@
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr"/>
+      <c r="I65" s="7" t="inlineStr">
+        <is>
+          <t>不补UT</t>
+        </is>
+      </c>
+      <c r="J65" s="7" t="inlineStr">
+        <is>
+          <t>设备详情展示属于 UI 侧场景，不进入本轮 UT 补充范围。</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="28.5" customHeight="1" s="1">
       <c r="A66" s="4" t="inlineStr">
@@ -4027,6 +4693,16 @@
         </is>
       </c>
       <c r="H66" s="5" t="inlineStr"/>
+      <c r="I66" s="7" t="inlineStr">
+        <is>
+          <t>不补UT</t>
+        </is>
+      </c>
+      <c r="J66" s="7" t="inlineStr">
+        <is>
+          <t>黑白名单页签展示属于页面渲染场景，不进入本轮 UT 补充范围。</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="28.5" customHeight="1" s="1">
       <c r="A67" s="4" t="inlineStr">
@@ -4067,6 +4743,16 @@
         </is>
       </c>
       <c r="H67" s="5" t="inlineStr"/>
+      <c r="I67" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J67" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/viewmodels/PeripheralPolicyViewModel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="28.5" customHeight="1" s="1">
       <c r="A68" s="4" t="inlineStr">
@@ -4107,6 +4793,16 @@
         </is>
       </c>
       <c r="H68" s="5" t="inlineStr"/>
+      <c r="I68" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J68" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/viewmodels/PeripheralPolicyViewModel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="42.75" customHeight="1" s="1">
       <c r="A69" s="4" t="inlineStr">
@@ -4147,6 +4843,16 @@
         </is>
       </c>
       <c r="H69" s="5" t="inlineStr"/>
+      <c r="I69" s="7" t="inlineStr">
+        <is>
+          <t>待补UT</t>
+        </is>
+      </c>
+      <c r="J69" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/viewmodels/PeripheralPolicyViewModel.test.ets：补接口禁用时单设备策略冲突拒绝与提示原因。</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="28.5" customHeight="1" s="1">
       <c r="A70" s="4" t="inlineStr">
@@ -4187,6 +4893,16 @@
         </is>
       </c>
       <c r="H70" s="5" t="inlineStr"/>
+      <c r="I70" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J70" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/viewmodels/PeripheralRecordViewModel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="42.75" customHeight="1" s="1">
       <c r="A71" s="4" t="inlineStr">
@@ -4228,6 +4944,16 @@
         </is>
       </c>
       <c r="H71" s="5" t="inlineStr"/>
+      <c r="I71" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J71" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/viewmodels/PeripheralViewModel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="42.75" customHeight="1" s="1">
       <c r="A72" s="4" t="inlineStr">
@@ -4268,6 +4994,16 @@
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr"/>
+      <c r="I72" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J72" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/viewmodels/PeripheralPolicyViewModel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="28.5" customHeight="1" s="1">
       <c r="A73" s="4" t="inlineStr">
@@ -4310,6 +5046,16 @@
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr"/>
+      <c r="I73" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J73" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/viewmodels/PeripheralPolicyViewModel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="28.5" customHeight="1" s="1">
       <c r="A74" s="4" t="inlineStr">
@@ -4352,6 +5098,16 @@
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr"/>
+      <c r="I74" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J74" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/peripheral/connection-record-bluetooth-acl-consumer.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="28.5" customHeight="1" s="1">
       <c r="A75" s="4" t="inlineStr">
@@ -4392,6 +5148,16 @@
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr"/>
+      <c r="I75" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J75" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/peripheral/connection-record-bluetooth-acl-consumer.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="28.5" customHeight="1" s="1">
       <c r="A76" s="4" t="inlineStr">
@@ -4432,6 +5198,16 @@
         </is>
       </c>
       <c r="H76" s="5" t="inlineStr"/>
+      <c r="I76" s="7" t="inlineStr">
+        <is>
+          <t>不补UT</t>
+        </is>
+      </c>
+      <c r="J76" s="7" t="inlineStr">
+        <is>
+          <t>蓝牙详情展示属于 UI 侧场景；蓝牙记录建模已有 UT，不再补展示 UT。</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="42.75" customHeight="1" s="1">
       <c r="A77" s="4" t="inlineStr">
@@ -4472,6 +5248,16 @@
         </is>
       </c>
       <c r="H77" s="5" t="inlineStr"/>
+      <c r="I77" s="7" t="inlineStr">
+        <is>
+          <t>待补UT</t>
+        </is>
+      </c>
+      <c r="J77" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/viewmodels/PeripheralPolicyViewModel.test.ets：补蓝牙设备 allow -&gt; deny，含 deviceId normalize。</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="42.75" customHeight="1" s="1">
       <c r="A78" s="4" t="inlineStr">
@@ -4512,6 +5298,16 @@
         </is>
       </c>
       <c r="H78" s="5" t="inlineStr"/>
+      <c r="I78" s="7" t="inlineStr">
+        <is>
+          <t>待补UT</t>
+        </is>
+      </c>
+      <c r="J78" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/viewmodels/PeripheralPolicyViewModel.test.ets：补蓝牙设备 deny -&gt; allow，含 deviceId normalize。</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="42.75" customHeight="1" s="1">
       <c r="A79" s="4" t="inlineStr">
@@ -4554,6 +5350,16 @@
         </is>
       </c>
       <c r="H79" s="5" t="inlineStr"/>
+      <c r="I79" s="7" t="inlineStr">
+        <is>
+          <t>不补UT</t>
+        </is>
+      </c>
+      <c r="J79" s="7" t="inlineStr">
+        <is>
+          <t>Select 显示回滚属于 AsyncSelectRow 组件本地交互状态，不进入本轮 UT 补充范围。</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="42.75" customHeight="1" s="1">
       <c r="A80" s="4" t="inlineStr">
@@ -4596,6 +5402,16 @@
         </is>
       </c>
       <c r="H80" s="5" t="inlineStr"/>
+      <c r="I80" s="7" t="inlineStr">
+        <is>
+          <t>不补UT</t>
+        </is>
+      </c>
+      <c r="J80" s="7" t="inlineStr">
+        <is>
+          <t>Select 显示回滚属于 AsyncSelectRow 组件本地交互状态，不进入本轮 UT 补充范围。</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="42.75" customHeight="1" s="1">
       <c r="A81" s="4" t="inlineStr">
@@ -4638,6 +5454,16 @@
         </is>
       </c>
       <c r="H81" s="5" t="inlineStr"/>
+      <c r="I81" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J81" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/viewmodels/PeripheralPolicyViewModel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="57" customHeight="1" s="1">
       <c r="A82" s="4" t="inlineStr">
@@ -4681,6 +5507,16 @@
         </is>
       </c>
       <c r="H82" s="5" t="inlineStr"/>
+      <c r="I82" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J82" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/identity/settings-viewmodel.test.ets；entry/src/test/identity/service.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="28.5" customHeight="1" s="1">
       <c r="A83" s="4" t="inlineStr">
@@ -4722,6 +5558,16 @@
         </is>
       </c>
       <c r="H83" s="5" t="inlineStr"/>
+      <c r="I83" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J83" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/identity/settings-viewmodel.test.ets；entry/src/test/identity/service.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="28.5" customHeight="1" s="1">
       <c r="A84" s="4" t="inlineStr">
@@ -4764,6 +5610,16 @@
         </is>
       </c>
       <c r="H84" s="5" t="inlineStr"/>
+      <c r="I84" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J84" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/identity/settings-viewmodel.test.ets；entry/src/test/identity/service.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="42.75" customHeight="1" s="1">
       <c r="A85" s="4" t="inlineStr">
@@ -4804,6 +5660,16 @@
         </is>
       </c>
       <c r="H85" s="5" t="inlineStr"/>
+      <c r="I85" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J85" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/identity/settings-viewmodel.test.ets；entry/src/test/identity/service.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="42.75" customHeight="1" s="1">
       <c r="A86" s="4" t="inlineStr">
@@ -4844,6 +5710,16 @@
         </is>
       </c>
       <c r="H86" s="5" t="inlineStr"/>
+      <c r="I86" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J86" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/identity/settings-viewmodel.test.ets；entry/src/test/identity/service.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="42.75" customHeight="1" s="1">
       <c r="A87" s="4" t="inlineStr">
@@ -4885,6 +5761,16 @@
         </is>
       </c>
       <c r="H87" s="5" t="inlineStr"/>
+      <c r="I87" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J87" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/tool-settings/viewmodel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="42.75" customHeight="1" s="1">
       <c r="A88" s="4" t="inlineStr">
@@ -4926,6 +5812,16 @@
         </is>
       </c>
       <c r="H88" s="5" t="inlineStr"/>
+      <c r="I88" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J88" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/tool-settings/viewmodel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="42.75" customHeight="1" s="1">
       <c r="A89" s="4" t="inlineStr">
@@ -4967,6 +5863,16 @@
         </is>
       </c>
       <c r="H89" s="5" t="inlineStr"/>
+      <c r="I89" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J89" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/tool-settings/viewmodel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="28.5" customHeight="1" s="1">
       <c r="A90" s="4" t="inlineStr">
@@ -5008,6 +5914,16 @@
         </is>
       </c>
       <c r="H90" s="5" t="inlineStr"/>
+      <c r="I90" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J90" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/tool-settings/viewmodel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="28.5" customHeight="1" s="1">
       <c r="A91" s="4" t="inlineStr">
@@ -5049,6 +5965,16 @@
         </is>
       </c>
       <c r="H91" s="5" t="inlineStr"/>
+      <c r="I91" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J91" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/tool-settings/viewmodel.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="42.75" customHeight="1" s="1">
       <c r="A92" s="4" t="inlineStr">
@@ -5089,6 +6015,16 @@
         </is>
       </c>
       <c r="H92" s="5" t="inlineStr"/>
+      <c r="I92" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J92" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/tool-settings/viewmodel.test.ets；entry/src/test/tool-settings/system-settings-service.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="42.75" customHeight="1" s="1">
       <c r="A93" s="4" t="inlineStr">
@@ -5129,6 +6065,16 @@
         </is>
       </c>
       <c r="H93" s="5" t="inlineStr"/>
+      <c r="I93" s="7" t="inlineStr">
+        <is>
+          <t>不补UT</t>
+        </is>
+      </c>
+      <c r="J93" s="7" t="inlineStr">
+        <is>
+          <t>页面打开属于页面渲染/导航场景，不进入本轮 UT 补充范围。</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="28.5" customHeight="1" s="1">
       <c r="A94" s="4" t="inlineStr">
@@ -5168,6 +6114,16 @@
         </is>
       </c>
       <c r="H94" s="5" t="inlineStr"/>
+      <c r="I94" s="7" t="inlineStr">
+        <is>
+          <t>不补UT</t>
+        </is>
+      </c>
+      <c r="J94" s="7" t="inlineStr">
+        <is>
+          <t>使用指南展示属于页面展示场景；文案结构已有基础 UT，不再补。</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="28.5" customHeight="1" s="1">
       <c r="A95" s="4" t="inlineStr">
@@ -5209,6 +6165,16 @@
         </is>
       </c>
       <c r="H95" s="5" t="inlineStr"/>
+      <c r="I95" s="7" t="inlineStr">
+        <is>
+          <t>不补UT</t>
+        </is>
+      </c>
+      <c r="J95" s="7" t="inlineStr">
+        <is>
+          <t>FAQ 展开收起属于页面交互场景，不进入本轮 UT 补充范围。</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="28.5" customHeight="1" s="1">
       <c r="A96" s="4" t="inlineStr">
@@ -5248,6 +6214,16 @@
         </is>
       </c>
       <c r="H96" s="5" t="inlineStr"/>
+      <c r="I96" s="7" t="inlineStr">
+        <is>
+          <t>不补UT</t>
+        </is>
+      </c>
+      <c r="J96" s="7" t="inlineStr">
+        <is>
+          <t>联系方式展示属于页面展示场景；文案结构已有基础 UT，不再补。</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="28.5" customHeight="1" s="1">
       <c r="A97" s="4" t="inlineStr">
@@ -5287,6 +6263,16 @@
         </is>
       </c>
       <c r="H97" s="5" t="inlineStr"/>
+      <c r="I97" s="7" t="inlineStr">
+        <is>
+          <t>不补UT</t>
+        </is>
+      </c>
+      <c r="J97" s="7" t="inlineStr">
+        <is>
+          <t>导航、弹窗或菜单交互属于 UI/ohosTest 范围，不进入本轮 UT 补充范围。</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="28.5" customHeight="1" s="1">
       <c r="A98" s="4" t="inlineStr">
@@ -5326,6 +6312,16 @@
         </is>
       </c>
       <c r="H98" s="5" t="inlineStr"/>
+      <c r="I98" s="7" t="inlineStr">
+        <is>
+          <t>不补UT</t>
+        </is>
+      </c>
+      <c r="J98" s="7" t="inlineStr">
+        <is>
+          <t>导航、弹窗或菜单交互属于 UI/ohosTest 范围，不进入本轮 UT 补充范围。</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="28.5" customHeight="1" s="1">
       <c r="A99" s="4" t="inlineStr">
@@ -5366,6 +6362,16 @@
         </is>
       </c>
       <c r="H99" s="5" t="inlineStr"/>
+      <c r="I99" s="7" t="inlineStr">
+        <is>
+          <t>不补UT</t>
+        </is>
+      </c>
+      <c r="J99" s="7" t="inlineStr">
+        <is>
+          <t>导航、弹窗或菜单交互属于 UI/ohosTest 范围，不进入本轮 UT 补充范围。</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="42.75" customHeight="1" s="1">
       <c r="A100" s="4" t="inlineStr">
@@ -5406,6 +6412,16 @@
         </is>
       </c>
       <c r="H100" s="5" t="inlineStr"/>
+      <c r="I100" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J100" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/theme/theme-manager.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="28.5" customHeight="1" s="1">
       <c r="A101" s="4" t="inlineStr">
@@ -5446,6 +6462,16 @@
         </is>
       </c>
       <c r="H101" s="5" t="inlineStr"/>
+      <c r="I101" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J101" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/theme/theme-manager.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="42.75" customHeight="1" s="1">
       <c r="A102" s="4" t="inlineStr">
@@ -5487,6 +6513,16 @@
         </is>
       </c>
       <c r="H102" s="5" t="inlineStr"/>
+      <c r="I102" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J102" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/theme/theme-manager.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="42.75" customHeight="1" s="1">
       <c r="A103" s="4" t="inlineStr">
@@ -5527,6 +6563,16 @@
         </is>
       </c>
       <c r="H103" s="5" t="inlineStr"/>
+      <c r="I103" s="7" t="inlineStr">
+        <is>
+          <t>不补UT</t>
+        </is>
+      </c>
+      <c r="J103" s="7" t="inlineStr">
+        <is>
+          <t>导航、弹窗或菜单交互属于 UI/ohosTest 范围，不进入本轮 UT 补充范围。</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="42.75" customHeight="1" s="1">
       <c r="A104" s="4" t="inlineStr">
@@ -5568,6 +6614,16 @@
         </is>
       </c>
       <c r="H104" s="5" t="inlineStr"/>
+      <c r="I104" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J104" s="7" t="inlineStr">
+        <is>
+          <t>entry/src/test/common/csv-file-export-service.test.ets；entry/src/test/log-manage/export-service.test.ets</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
@@ -5609,6 +6665,16 @@
         </is>
       </c>
       <c r="H105" s="5" t="inlineStr"/>
+      <c r="I105" s="7" t="inlineStr">
+        <is>
+          <t>不补UT</t>
+        </is>
+      </c>
+      <c r="J105" s="7" t="inlineStr">
+        <is>
+          <t>重启后恢复属于集成语义；存储读写已有基础 UT，不再补。</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
@@ -5651,6 +6717,16 @@
         </is>
       </c>
       <c r="H106" s="5" t="inlineStr"/>
+      <c r="I106" s="7" t="inlineStr">
+        <is>
+          <t>不补UT</t>
+        </is>
+      </c>
+      <c r="J106" s="7" t="inlineStr">
+        <is>
+          <t>前后台切换属于应用生命周期集成场景，不进入本轮 UT 补充范围。</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
test: supplement baseline ut coverage
</commit_message>
<xml_diff>
--- a/docs/04-测试文档/手工测试用例/测试用例基线.xlsx
+++ b/docs/04-测试文档/手工测试用例/测试用例基线.xlsx
@@ -4344,12 +4344,12 @@
       <c r="H59" s="5" t="inlineStr"/>
       <c r="I59" s="7" t="inlineStr">
         <is>
-          <t>待补UT</t>
+          <t>已有UT覆盖</t>
         </is>
       </c>
       <c r="J59" s="7" t="inlineStr">
         <is>
-          <t>entry/src/test/viewmodels/InterfaceControlViewModel.test.ets：补 USB 存储禁止访问 prohibited/disabled 分支。</t>
+          <t>entry/src/test/viewmodels/InterfaceControlViewModel.test.ets</t>
         </is>
       </c>
     </row>
@@ -5250,12 +5250,12 @@
       <c r="H77" s="5" t="inlineStr"/>
       <c r="I77" s="7" t="inlineStr">
         <is>
-          <t>待补UT</t>
+          <t>已有UT覆盖</t>
         </is>
       </c>
       <c r="J77" s="7" t="inlineStr">
         <is>
-          <t>entry/src/test/viewmodels/PeripheralPolicyViewModel.test.ets：补蓝牙设备 allow -&gt; deny，含 deviceId normalize。</t>
+          <t>entry/src/test/viewmodels/PeripheralPolicyViewModel.test.ets</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: clarify local ut coverage boundary
</commit_message>
<xml_diff>
--- a/docs/04-测试文档/手工测试用例/测试用例基线.xlsx
+++ b/docs/04-测试文档/手工测试用例/测试用例基线.xlsx
@@ -3016,12 +3016,12 @@
       <c r="H33" s="5" t="inlineStr"/>
       <c r="I33" s="7" t="inlineStr">
         <is>
-          <t>待补UT</t>
+          <t>UT部分覆盖</t>
         </is>
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>entry/src/test/entryability/entryability.test.ets；entry/src/test/firewall/system-user-provider.test.ets：补账户新增/删除事件分发与可用用户列表更新。</t>
+          <t>entry/src/test/entryability/entryability.test.ets；entry/src/test/firewall/system-user-provider.test.ets：覆盖账户新增事件分发到 SystemUserProvider.trackAddedUser、用户维护方法入口、用户列表结果结构和用户策略结果。Local UT 不覆盖 application.getApplicationContext() 后的 Preferences 真实落盘，不覆盖弹窗重新打开 UI 刷新。</t>
         </is>
       </c>
     </row>
@@ -3070,12 +3070,12 @@
       <c r="H34" s="5" t="inlineStr"/>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>待补UT</t>
+          <t>UT部分覆盖</t>
         </is>
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
-          <t>entry/src/test/entryability/entryability.test.ets；entry/src/test/firewall/system-user-provider.test.ets：补账户新增/删除事件分发与可用用户列表更新。</t>
+          <t>entry/src/test/entryability/entryability.test.ets；entry/src/test/firewall/system-user-provider.test.ets：覆盖账户删除事件分发到 SystemUserProvider.trackRemovedUser、用户维护方法入口、用户列表结果结构和用户策略结果。Local UT 不覆盖 application.getApplicationContext() 后的 Preferences 真实落盘，不覆盖弹窗重新打开 UI 刷新。</t>
         </is>
       </c>
     </row>
@@ -3124,12 +3124,12 @@
       <c r="H35" s="5" t="inlineStr"/>
       <c r="I35" s="7" t="inlineStr">
         <is>
-          <t>待补UT</t>
+          <t>UT部分覆盖</t>
         </is>
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>entry/src/test/entryability/entryability.test.ets；entry/src/test/firewall/system-user-provider.test.ets：补账户新增/删除事件分发与可用用户列表更新。</t>
+          <t>entry/src/test/entryability/entryability.test.ets；entry/src/test/firewall/system-user-provider.test.ets：覆盖账户新增事件分发到 SystemUserProvider.trackAddedUser、用户维护方法入口、用户列表结果结构和用户策略结果。Local UT 不覆盖 application.getApplicationContext() 后的 Preferences 真实落盘，不覆盖弹窗重新打开 UI 刷新。</t>
         </is>
       </c>
     </row>
@@ -3178,12 +3178,12 @@
       <c r="H36" s="5" t="inlineStr"/>
       <c r="I36" s="7" t="inlineStr">
         <is>
-          <t>待补UT</t>
+          <t>UT部分覆盖</t>
         </is>
       </c>
       <c r="J36" s="7" t="inlineStr">
         <is>
-          <t>entry/src/test/entryability/entryability.test.ets；entry/src/test/firewall/system-user-provider.test.ets：补账户新增/删除事件分发与可用用户列表更新。</t>
+          <t>entry/src/test/entryability/entryability.test.ets；entry/src/test/firewall/system-user-provider.test.ets：覆盖账户删除事件分发到 SystemUserProvider.trackRemovedUser、用户维护方法入口、用户列表结果结构和用户策略结果。Local UT 不覆盖 application.getApplicationContext() 后的 Preferences 真实落盘，不覆盖弹窗重新打开 UI 刷新。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: sync completed ut coverage status
</commit_message>
<xml_diff>
--- a/docs/04-测试文档/手工测试用例/测试用例基线.xlsx
+++ b/docs/04-测试文档/手工测试用例/测试用例基线.xlsx
@@ -2541,12 +2541,12 @@
       <c r="H24" s="5" t="inlineStr"/>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>待补UT</t>
+          <t>已有UT覆盖</t>
         </is>
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
-          <t>entry/src/test/firewall/rule-utils.test.ets：补 wildcard 单级域名重叠判定。</t>
+          <t>entry/src/test/firewall/rule-utils.test.ets</t>
         </is>
       </c>
     </row>
@@ -2596,12 +2596,12 @@
       <c r="H25" s="5" t="inlineStr"/>
       <c r="I25" s="7" t="inlineStr">
         <is>
-          <t>待补UT</t>
+          <t>已有UT覆盖</t>
         </is>
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
-          <t>entry/src/test/firewall/service.test.ets：补用户级白名单策略下发 + PIN 成功/失败。</t>
+          <t>entry/src/test/firewall/service.test.ets</t>
         </is>
       </c>
     </row>
@@ -2651,12 +2651,12 @@
       <c r="H26" s="5" t="inlineStr"/>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>待补UT</t>
+          <t>已有UT覆盖</t>
         </is>
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
-          <t>entry/src/test/firewall/service.test.ets：补用户级黑名单策略下发 + PIN 成功/失败。</t>
+          <t>entry/src/test/firewall/service.test.ets</t>
         </is>
       </c>
     </row>
@@ -4394,12 +4394,12 @@
       <c r="H60" s="5" t="inlineStr"/>
       <c r="I60" s="7" t="inlineStr">
         <is>
-          <t>待补UT</t>
+          <t>已有UT覆盖</t>
         </is>
       </c>
       <c r="J60" s="7" t="inlineStr">
         <is>
-          <t>entry/src/test/viewmodels/InterfaceControlViewModel.test.ets：补 USB 接口禁用时 USB 存储策略冲突拒绝。</t>
+          <t>entry/src/test/viewmodels/InterfaceControlViewModel.test.ets</t>
         </is>
       </c>
     </row>
@@ -4444,12 +4444,12 @@
       <c r="H61" s="5" t="inlineStr"/>
       <c r="I61" s="7" t="inlineStr">
         <is>
-          <t>待补UT</t>
+          <t>已有UT覆盖</t>
         </is>
       </c>
       <c r="J61" s="7" t="inlineStr">
         <is>
-          <t>entry/src/test/viewmodels/InterfaceControlViewModel.test.ets：补蓝牙接口策略切换。</t>
+          <t>entry/src/test/viewmodels/InterfaceControlViewModel.test.ets</t>
         </is>
       </c>
     </row>
@@ -4494,12 +4494,12 @@
       <c r="H62" s="5" t="inlineStr"/>
       <c r="I62" s="7" t="inlineStr">
         <is>
-          <t>待补UT</t>
+          <t>已有UT覆盖</t>
         </is>
       </c>
       <c r="J62" s="7" t="inlineStr">
         <is>
-          <t>entry/src/test/viewmodels/InterfaceControlViewModel.test.ets：补 Wi-Fi 接口策略切换。</t>
+          <t>entry/src/test/viewmodels/InterfaceControlViewModel.test.ets</t>
         </is>
       </c>
     </row>
@@ -4845,12 +4845,12 @@
       <c r="H69" s="5" t="inlineStr"/>
       <c r="I69" s="7" t="inlineStr">
         <is>
-          <t>待补UT</t>
+          <t>已有UT覆盖</t>
         </is>
       </c>
       <c r="J69" s="7" t="inlineStr">
         <is>
-          <t>entry/src/test/viewmodels/PeripheralPolicyViewModel.test.ets：补接口禁用时单设备策略冲突拒绝与提示原因。</t>
+          <t>entry/src/test/viewmodels/PeripheralPolicyViewModel.test.ets</t>
         </is>
       </c>
     </row>
@@ -5300,12 +5300,12 @@
       <c r="H78" s="5" t="inlineStr"/>
       <c r="I78" s="7" t="inlineStr">
         <is>
-          <t>待补UT</t>
+          <t>已有UT覆盖</t>
         </is>
       </c>
       <c r="J78" s="7" t="inlineStr">
         <is>
-          <t>entry/src/test/viewmodels/PeripheralPolicyViewModel.test.ets：补蓝牙设备 deny -&gt; allow，含 deviceId normalize。</t>
+          <t>entry/src/test/viewmodels/PeripheralPolicyViewModel.test.ets</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: lock usb storage auto deny exception
</commit_message>
<xml_diff>
--- a/docs/04-测试文档/手工测试用例/测试用例基线.xlsx
+++ b/docs/04-测试文档/手工测试用例/测试用例基线.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例_ai" sheetId="1" r:id="Ra9c56190b0d84acd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例_ai" sheetId="1" r:id="R1e6d9a190c1f4ae1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3939,550 +3939,553 @@
     </x:row>
     <x:row r="87" s="1" customFormat="1" ht="42.75" customHeight="1">
       <x:c r="A87" s="4" t="str">
+        <x:v>PER-033</x:v>
+      </x:c>
+      <x:c r="B87" s="5" t="str">
+        <x:v>外设管理</x:v>
+      </x:c>
+      <x:c r="C87" s="5" t="str">
+        <x:v>首次连接自动拉黑</x:v>
+      </x:c>
+      <x:c r="D87" s="5" t="str">
+        <x:v>验证 USB 存储总策略为禁止访问时，首次接入 USB 存储设备不自动下发设备级黑名单</x:v>
+      </x:c>
+      <x:c r="E87" s="5" t="str">
+        <x:v>应用已激活企业管理员，USB 存储策略当前为 `禁止访问`，目标 U 盘此前未存在本地 allow / deny 策略</x:v>
+      </x:c>
+      <x:c r="F87" s="5" t="str">
+        <x:v>1. 进入接口管控页签，将 USB 存储策略设置为 `禁止访问`
+2. 插入首次接入的 USB 存储设备
+3. 查看设备连接记录和黑白名单页签</x:v>
+      </x:c>
+      <x:c r="G87" s="5" t="str">
+        <x:v>1. 本次连接记录正常落库并展示 USB 存储已禁用
+2. 不下发设备级 deny
+3. 本地黑白名单不新增该 U 盘 deny 策略</x:v>
+      </x:c>
+      <x:c r="H87" s="5"/>
+      <x:c r="I87" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J87" s="7" t="str">
+        <x:v>entry/src/test/peripheral/connection-record-usb-consumer.test.ets</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" s="1" customFormat="1" ht="42.75" customHeight="1">
+      <x:c r="A88" s="4" t="str">
         <x:v>ID-001</x:v>
       </x:c>
-      <x:c r="B87" s="5" t="str">
+      <x:c r="B88" s="5" t="str">
         <x:v>身份鉴别</x:v>
       </x:c>
-      <x:c r="C87" s="5" t="str">
+      <x:c r="C88" s="5" t="str">
         <x:v>口令复杂度策略</x:v>
       </x:c>
-      <x:c r="D87" s="5" t="str">
+      <x:c r="D88" s="5" t="str">
         <x:v>验证保存口令复杂度策略：最小长度 8，大写/小写/数字开启，特殊字符关闭</x:v>
       </x:c>
-      <x:c r="E87" s="5" t="str">
+      <x:c r="E88" s="5" t="str">
         <x:v>应用已激活企业管理员</x:v>
       </x:c>
-      <x:c r="F87" s="5" t="str">
+      <x:c r="F88" s="5" t="str">
         <x:v>1. 进入身份鉴别页
 2. 设置最小长度为 `8`
 3. 开启大写字母、小写字母、数字要求
 4. 关闭特殊字符要求
 5. 点击保存身份鉴别配置</x:v>
       </x:c>
-      <x:c r="G87" s="5" t="str">
+      <x:c r="G88" s="5" t="str">
         <x:v>1. 页面提示身份鉴别配置已保存
 2. 系统设置中策略显示与配置一致</x:v>
       </x:c>
-      <x:c r="H87" s="5"/>
-      <x:c r="I87" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J87" s="7" t="str">
+      <x:c r="H88" s="5"/>
+      <x:c r="I88" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J88" s="7" t="str">
         <x:v>entry/src/test/identity/settings-viewmodel.test.ets；entry/src/test/identity/service.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="88" s="1" customFormat="1" ht="42.75" customHeight="1">
-      <x:c r="A88" s="4" t="str">
+    <x:row r="89" s="1" customFormat="1" ht="42.75" customHeight="1">
+      <x:c r="A89" s="4" t="str">
         <x:v>ID-002</x:v>
       </x:c>
-      <x:c r="B88" s="5" t="str">
+      <x:c r="B89" s="5" t="str">
         <x:v>身份鉴别</x:v>
       </x:c>
-      <x:c r="C88" s="5" t="str">
+      <x:c r="C89" s="5" t="str">
         <x:v>密码有效期策略</x:v>
       </x:c>
-      <x:c r="D88" s="5" t="str">
+      <x:c r="D89" s="5" t="str">
         <x:v>验证将密码有效期设置为 180 天后保存成功</x:v>
       </x:c>
-      <x:c r="E88" s="5" t="str">
+      <x:c r="E89" s="5" t="str">
         <x:v>应用已激活企业管理员</x:v>
       </x:c>
-      <x:c r="F88" s="5" t="str">
+      <x:c r="F89" s="5" t="str">
         <x:v>1. 进入身份鉴别页
 2. 选择密码有效期 `180天`
 3. 点击保存</x:v>
       </x:c>
-      <x:c r="G88" s="5" t="str">
+      <x:c r="G89" s="5" t="str">
         <x:v>1. 页面提示保存成功
 2. 再次进入页面可回显 `180天`</x:v>
       </x:c>
-      <x:c r="H88" s="5"/>
-      <x:c r="I88" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J88" s="7" t="str">
+      <x:c r="H89" s="5"/>
+      <x:c r="I89" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J89" s="7" t="str">
         <x:v>entry/src/test/identity/settings-viewmodel.test.ets；entry/src/test/identity/service.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="89" s="1" customFormat="1" ht="42.75" customHeight="1">
-      <x:c r="A89" s="4" t="str">
+    <x:row r="90" s="1" customFormat="1" ht="28.5" customHeight="1">
+      <x:c r="A90" s="4" t="str">
         <x:v>ID-003</x:v>
       </x:c>
-      <x:c r="B89" s="5" t="str">
+      <x:c r="B90" s="5" t="str">
         <x:v>身份鉴别</x:v>
       </x:c>
-      <x:c r="C89" s="5" t="str">
+      <x:c r="C90" s="5" t="str">
         <x:v>密码有效期策略</x:v>
       </x:c>
-      <x:c r="D89" s="5" t="str">
+      <x:c r="D90" s="5" t="str">
         <x:v>验证将自定义密码有效期设置为 30 天后保存成功</x:v>
       </x:c>
-      <x:c r="E89" s="5" t="str">
+      <x:c r="E90" s="5" t="str">
         <x:v>应用已激活企业管理员</x:v>
       </x:c>
-      <x:c r="F89" s="5" t="str">
+      <x:c r="F90" s="5" t="str">
         <x:v>1. 进入身份鉴别页
 2. 选择自定义有效期
 3. 输入 `30`
 4. 点击保存</x:v>
       </x:c>
-      <x:c r="G89" s="5" t="str">
+      <x:c r="G90" s="5" t="str">
         <x:v>1. 页面提示保存成功
 2. 再次进入页面可回显 `30天`</x:v>
       </x:c>
-      <x:c r="H89" s="5"/>
-      <x:c r="I89" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J89" s="7" t="str">
+      <x:c r="H90" s="5"/>
+      <x:c r="I90" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J90" s="7" t="str">
         <x:v>entry/src/test/identity/settings-viewmodel.test.ets；entry/src/test/identity/service.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="90" s="1" customFormat="1" ht="28.5" customHeight="1">
-      <x:c r="A90" s="4" t="str">
+    <x:row r="91" s="1" customFormat="1" ht="28.5" customHeight="1">
+      <x:c r="A91" s="4" t="str">
         <x:v>ID-004</x:v>
       </x:c>
-      <x:c r="B90" s="5" t="str">
+      <x:c r="B91" s="5" t="str">
         <x:v>身份鉴别</x:v>
       </x:c>
-      <x:c r="C90" s="5" t="str">
+      <x:c r="C91" s="5" t="str">
         <x:v>输入参数校验</x:v>
       </x:c>
-      <x:c r="D90" s="5" t="str">
+      <x:c r="D91" s="5" t="str">
         <x:v>验证自定义密码有效期非法字符被过滤，空值保存时被拦截</x:v>
       </x:c>
-      <x:c r="E90" s="5" t="str">
+      <x:c r="E91" s="5" t="str">
         <x:v>已选择自定义有效期</x:v>
       </x:c>
-      <x:c r="F90" s="5" t="str">
+      <x:c r="F91" s="5" t="str">
         <x:v>1. 选择自定义有效期
 2. 尝试输入 abc、-1 等非法字符
 3. 清空输入框
 4. 点击保存</x:v>
       </x:c>
-      <x:c r="G90" s="5" t="str">
+      <x:c r="G91" s="5" t="str">
         <x:v>1. 非法字符不会保留在输入框中，或仅保留数字字符
 2. 自定义有效期为空时点击保存，页面提示请输入非负整数天数
 3. 未通过校验时不下发策略</x:v>
       </x:c>
-      <x:c r="H90" s="5"/>
-      <x:c r="I90" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J90" s="7" t="str">
+      <x:c r="H91" s="5"/>
+      <x:c r="I91" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J91" s="7" t="str">
         <x:v>entry/src/test/identity/settings-viewmodel.test.ets；entry/src/test/identity/service.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="91" s="1" customFormat="1" ht="28.5" customHeight="1">
-      <x:c r="A91" s="4" t="str">
+    <x:row r="92" s="1" customFormat="1" ht="42.75" customHeight="1">
+      <x:c r="A92" s="4" t="str">
         <x:v>ID-007</x:v>
       </x:c>
-      <x:c r="B91" s="5" t="str">
+      <x:c r="B92" s="5" t="str">
         <x:v>身份鉴别</x:v>
       </x:c>
-      <x:c r="C91" s="5" t="str">
+      <x:c r="C92" s="5" t="str">
         <x:v>策略保存</x:v>
       </x:c>
-      <x:c r="D91" s="5" t="str">
+      <x:c r="D92" s="5" t="str">
         <x:v>验证自定义密码有效期输入 0 天时触发风险提示</x:v>
       </x:c>
-      <x:c r="E91" s="5" t="str">
+      <x:c r="E92" s="5" t="str">
         <x:v>应用已激活企业管理员，已选择自定义有效期</x:v>
       </x:c>
-      <x:c r="F91" s="5" t="str">
+      <x:c r="F92" s="5" t="str">
         <x:v>1. 输入 `0`
 2. 点击保存</x:v>
       </x:c>
-      <x:c r="G91" s="5" t="str">
+      <x:c r="G92" s="5" t="str">
         <x:v>1. 页面弹出风险提示
 2. 用户确认前不直接保存策略</x:v>
       </x:c>
-      <x:c r="H91" s="5"/>
-      <x:c r="I91" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J91" s="7" t="str">
+      <x:c r="H92" s="5"/>
+      <x:c r="I92" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J92" s="7" t="str">
         <x:v>entry/src/test/identity/settings-viewmodel.test.ets；entry/src/test/identity/service.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="92" s="1" customFormat="1" ht="42.75" customHeight="1">
-      <x:c r="A92" s="4" t="str">
+    <x:row r="93" s="1" customFormat="1" ht="42.75" customHeight="1">
+      <x:c r="A93" s="4" t="str">
         <x:v>SET-002</x:v>
       </x:c>
-      <x:c r="B92" s="5" t="str">
+      <x:c r="B93" s="5" t="str">
         <x:v>工具设置</x:v>
       </x:c>
-      <x:c r="C92" s="5" t="str">
+      <x:c r="C93" s="5" t="str">
         <x:v>启动认证开关</x:v>
       </x:c>
-      <x:c r="D92" s="5" t="str">
+      <x:c r="D93" s="5" t="str">
         <x:v>验证关闭启动时身份校验后保存成功</x:v>
       </x:c>
-      <x:c r="E92" s="5" t="str">
+      <x:c r="E93" s="5" t="str">
         <x:v>启动时身份校验当前已开启</x:v>
       </x:c>
-      <x:c r="F92" s="5" t="str">
+      <x:c r="F93" s="5" t="str">
         <x:v>1. 进入工具设置页
 2. 关闭启动时身份校验
 3. 点击保存设置</x:v>
       </x:c>
-      <x:c r="G92" s="5" t="str">
+      <x:c r="G93" s="5" t="str">
         <x:v>1. 页面提示工具设置已保存
 2. 重启应用后不再要求启动认证</x:v>
       </x:c>
-      <x:c r="H92" s="5"/>
-      <x:c r="I92" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J92" s="7" t="str">
+      <x:c r="H93" s="5"/>
+      <x:c r="I93" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J93" s="7" t="str">
         <x:v>entry/src/test/tool-settings/viewmodel.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="93" s="1" customFormat="1" ht="42.75" customHeight="1">
-      <x:c r="A93" s="4" t="str">
+    <x:row r="94" s="1" customFormat="1" ht="28.5" customHeight="1">
+      <x:c r="A94" s="4" t="str">
         <x:v>SET-003</x:v>
       </x:c>
-      <x:c r="B93" s="5" t="str">
+      <x:c r="B94" s="5" t="str">
         <x:v>工具设置</x:v>
       </x:c>
-      <x:c r="C93" s="5" t="str">
+      <x:c r="C94" s="5" t="str">
         <x:v>认证方式选择</x:v>
       </x:c>
-      <x:c r="D93" s="5" t="str">
+      <x:c r="D94" s="5" t="str">
         <x:v>验证选择 PIN 认证方式后保存成功</x:v>
       </x:c>
-      <x:c r="E93" s="5" t="str">
+      <x:c r="E94" s="5" t="str">
         <x:v>启动时身份校验已开启，系统 PIN 可用</x:v>
       </x:c>
-      <x:c r="F93" s="5" t="str">
+      <x:c r="F94" s="5" t="str">
         <x:v>1. 进入工具设置页
 2. 选择 `PIN` 认证方式
 3. 点击保存设置</x:v>
       </x:c>
-      <x:c r="G93" s="5" t="str">
+      <x:c r="G94" s="5" t="str">
         <x:v>1. 页面提示保存成功
 2. 重启应用后按 PIN 方式进行校验</x:v>
       </x:c>
-      <x:c r="H93" s="5"/>
-      <x:c r="I93" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J93" s="7" t="str">
+      <x:c r="H94" s="5"/>
+      <x:c r="I94" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J94" s="7" t="str">
         <x:v>entry/src/test/tool-settings/viewmodel.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="94" s="1" customFormat="1" ht="28.5" customHeight="1">
-      <x:c r="A94" s="4" t="str">
+    <x:row r="95" s="1" customFormat="1" ht="28.5" customHeight="1">
+      <x:c r="A95" s="4" t="str">
         <x:v>SET-004</x:v>
       </x:c>
-      <x:c r="B94" s="5" t="str">
+      <x:c r="B95" s="5" t="str">
         <x:v>工具设置</x:v>
       </x:c>
-      <x:c r="C94" s="5" t="str">
+      <x:c r="C95" s="5" t="str">
         <x:v>认证方式选择</x:v>
       </x:c>
-      <x:c r="D94" s="5" t="str">
+      <x:c r="D95" s="5" t="str">
         <x:v>验证选择指纹认证方式后保存成功</x:v>
       </x:c>
-      <x:c r="E94" s="5" t="str">
+      <x:c r="E95" s="5" t="str">
         <x:v>设备已录入指纹且系统指纹认证可用</x:v>
       </x:c>
-      <x:c r="F94" s="5" t="str">
+      <x:c r="F95" s="5" t="str">
         <x:v>1. 进入工具设置页
 2. 选择 `指纹` 认证方式
 3. 点击保存设置</x:v>
       </x:c>
-      <x:c r="G94" s="5" t="str">
+      <x:c r="G95" s="5" t="str">
         <x:v>1. 页面提示保存成功
 2. 重启应用后按指纹方式进行校验</x:v>
       </x:c>
-      <x:c r="H94" s="5"/>
-      <x:c r="I94" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J94" s="7" t="str">
+      <x:c r="H95" s="5"/>
+      <x:c r="I95" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J95" s="7" t="str">
         <x:v>entry/src/test/tool-settings/viewmodel.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="95" s="1" customFormat="1" ht="28.5" customHeight="1">
-      <x:c r="A95" s="4" t="str">
+    <x:row r="96" s="1" customFormat="1" ht="28.5" customHeight="1">
+      <x:c r="A96" s="4" t="str">
         <x:v>SET-005</x:v>
       </x:c>
-      <x:c r="B95" s="5" t="str">
+      <x:c r="B96" s="5" t="str">
         <x:v>工具设置</x:v>
       </x:c>
-      <x:c r="C95" s="5" t="str">
+      <x:c r="C96" s="5" t="str">
         <x:v>无变更保存</x:v>
       </x:c>
-      <x:c r="D95" s="5" t="str">
+      <x:c r="D96" s="5" t="str">
         <x:v>验证未修改设置时保存按钮不可点击</x:v>
       </x:c>
-      <x:c r="E95" s="5" t="str">
+      <x:c r="E96" s="5" t="str">
         <x:v>进入工具设置页且不修改任何配置</x:v>
       </x:c>
-      <x:c r="F95" s="5" t="str">
+      <x:c r="F96" s="5" t="str">
         <x:v>1. 进入工具设置页
 2. 不做任何修改
 3. 观察保存按钮状态</x:v>
       </x:c>
-      <x:c r="G95" s="5" t="str">
+      <x:c r="G96" s="5" t="str">
         <x:v>1. 保存按钮保持不可点击状态
 2. 页面不触发保存动作</x:v>
       </x:c>
-      <x:c r="H95" s="5"/>
-      <x:c r="I95" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J95" s="7" t="str">
+      <x:c r="H96" s="5"/>
+      <x:c r="I96" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J96" s="7" t="str">
         <x:v>entry/src/test/tool-settings/viewmodel.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="96" s="1" customFormat="1" ht="28.5" customHeight="1">
-      <x:c r="A96" s="4" t="str">
+    <x:row r="97" s="1" customFormat="1" ht="28.5" customHeight="1">
+      <x:c r="A97" s="4" t="str">
         <x:v>SET-006</x:v>
       </x:c>
-      <x:c r="B96" s="5" t="str">
+      <x:c r="B97" s="5" t="str">
         <x:v>工具设置</x:v>
       </x:c>
-      <x:c r="C96" s="5" t="str">
+      <x:c r="C97" s="5" t="str">
         <x:v>认证方式不可用提示</x:v>
       </x:c>
-      <x:c r="D96" s="5" t="str">
+      <x:c r="D97" s="5" t="str">
         <x:v>验证选择当前设备不可用的认证方式时出现不可用确认提示</x:v>
       </x:c>
-      <x:c r="E96" s="5" t="str">
+      <x:c r="E97" s="5" t="str">
         <x:v>当前设备存在一种不可用认证方式</x:v>
       </x:c>
-      <x:c r="F96" s="5" t="str">
+      <x:c r="F97" s="5" t="str">
         <x:v>1. 进入工具设置页
 2. 选择当前设备不可用的认证方式
 3. 点击保存设置</x:v>
       </x:c>
-      <x:c r="G96" s="5" t="str">
+      <x:c r="G97" s="5" t="str">
         <x:v>1. 页面弹出认证方式不可用提示
 2. 用户确认前不直接保存</x:v>
       </x:c>
-      <x:c r="H96" s="5"/>
-      <x:c r="I96" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J96" s="7" t="str">
+      <x:c r="H97" s="5"/>
+      <x:c r="I97" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J97" s="7" t="str">
         <x:v>entry/src/test/tool-settings/viewmodel.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="97" s="1" customFormat="1" ht="28.5" customHeight="1">
-      <x:c r="A97" s="4" t="str">
+    <x:row r="98" s="1" customFormat="1" ht="28.5" customHeight="1">
+      <x:c r="A98" s="4" t="str">
         <x:v>SET-007</x:v>
       </x:c>
-      <x:c r="B97" s="5" t="str">
+      <x:c r="B98" s="5" t="str">
         <x:v>工具设置</x:v>
       </x:c>
-      <x:c r="C97" s="5" t="str">
+      <x:c r="C98" s="5" t="str">
         <x:v>修改密码入口</x:v>
       </x:c>
-      <x:c r="D97" s="5" t="str">
+      <x:c r="D98" s="5" t="str">
         <x:v>验证点击修改密码后拉起系统“生物识别和密码”页面</x:v>
       </x:c>
-      <x:c r="E97" s="5" t="str">
+      <x:c r="E98" s="5" t="str">
         <x:v>系统设置能力可用</x:v>
       </x:c>
-      <x:c r="F97" s="5" t="str">
+      <x:c r="F98" s="5" t="str">
         <x:v>1. 进入工具设置页
 2. 点击 `修改密码`</x:v>
       </x:c>
-      <x:c r="G97" s="5" t="str">
+      <x:c r="G98" s="5" t="str">
         <x:v>1. 成功拉起系统 `生物识别和密码` 页面
 2. 拉起失败时展示明确失败提示</x:v>
       </x:c>
-      <x:c r="H97" s="5"/>
-      <x:c r="I97" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J97" s="7" t="str">
+      <x:c r="H98" s="5"/>
+      <x:c r="I98" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J98" s="7" t="str">
         <x:v>entry/src/test/tool-settings/viewmodel.test.ets；entry/src/test/tool-settings/system-settings-service.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="98" s="1" customFormat="1" ht="28.5" customHeight="1">
-      <x:c r="A98" s="4" t="str">
+    <x:row r="99" s="1" customFormat="1" ht="28.5" customHeight="1">
+      <x:c r="A99" s="4" t="str">
         <x:v>HELP-001</x:v>
       </x:c>
-      <x:c r="B98" s="5" t="str">
+      <x:c r="B99" s="5" t="str">
         <x:v>帮助与反馈</x:v>
       </x:c>
-      <x:c r="C98" s="5" t="str">
+      <x:c r="C99" s="5" t="str">
         <x:v>页面展示</x:v>
       </x:c>
-      <x:c r="D98" s="5" t="str">
+      <x:c r="D99" s="5" t="str">
         <x:v>验证帮助与反馈页可正常打开</x:v>
       </x:c>
-      <x:c r="E98" s="5" t="str">
+      <x:c r="E99" s="5" t="str">
         <x:v>应用处于任一主页面</x:v>
       </x:c>
-      <x:c r="F98" s="5" t="str">
+      <x:c r="F99" s="5" t="str">
         <x:v>1. 打开右上角菜单
 2. 点击帮助与反馈</x:v>
       </x:c>
-      <x:c r="G98" s="5" t="str">
+      <x:c r="G99" s="5" t="str">
         <x:v>1. 成功进入帮助与反馈页
 2. 页面标题、说明正常展示</x:v>
-      </x:c>
-      <x:c r="H98" s="5"/>
-      <x:c r="I98" s="7" t="str">
-        <x:v>不补UT</x:v>
-      </x:c>
-      <x:c r="J98" s="7" t="str">
-        <x:v>页面打开属于页面渲染/导航场景，不进入本轮 UT 补充范围。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="99" s="1" customFormat="1" ht="28.5" customHeight="1">
-      <x:c r="A99" s="4" t="str">
-        <x:v>HELP-002</x:v>
-      </x:c>
-      <x:c r="B99" s="5" t="str">
-        <x:v>帮助与反馈</x:v>
-      </x:c>
-      <x:c r="C99" s="5" t="str">
-        <x:v>使用指南展示</x:v>
-      </x:c>
-      <x:c r="D99" s="5" t="str">
-        <x:v>验证使用指南内容展示完整</x:v>
-      </x:c>
-      <x:c r="E99" s="5" t="str">
-        <x:v>已进入帮助与反馈页</x:v>
-      </x:c>
-      <x:c r="F99" s="5" t="str">
-        <x:v>1. 查看使用指南区域</x:v>
-      </x:c>
-      <x:c r="G99" s="5" t="str">
-        <x:v>1. 展示防火墙、外设、身份鉴别、工具设置、主题模式等指南项
-2. 文案无截断</x:v>
       </x:c>
       <x:c r="H99" s="5"/>
       <x:c r="I99" s="7" t="str">
         <x:v>不补UT</x:v>
       </x:c>
       <x:c r="J99" s="7" t="str">
-        <x:v>使用指南展示属于页面展示场景；文案结构已有基础 UT，不再补。</x:v>
+        <x:v>页面打开属于页面渲染/导航场景，不进入本轮 UT 补充范围。</x:v>
       </x:c>
     </x:row>
     <x:row r="100" s="1" customFormat="1" ht="42.75" customHeight="1">
       <x:c r="A100" s="4" t="str">
-        <x:v>HELP-003</x:v>
+        <x:v>HELP-002</x:v>
       </x:c>
       <x:c r="B100" s="5" t="str">
         <x:v>帮助与反馈</x:v>
       </x:c>
       <x:c r="C100" s="5" t="str">
-        <x:v>FAQ展开收起</x:v>
+        <x:v>使用指南展示</x:v>
       </x:c>
       <x:c r="D100" s="5" t="str">
-        <x:v>验证 FAQ 可以展开和收起</x:v>
+        <x:v>验证使用指南内容展示完整</x:v>
       </x:c>
       <x:c r="E100" s="5" t="str">
         <x:v>已进入帮助与反馈页</x:v>
       </x:c>
       <x:c r="F100" s="5" t="str">
+        <x:v>1. 查看使用指南区域</x:v>
+      </x:c>
+      <x:c r="G100" s="5" t="str">
+        <x:v>1. 展示防火墙、外设、身份鉴别、工具设置、主题模式等指南项
+2. 文案无截断</x:v>
+      </x:c>
+      <x:c r="H100" s="5"/>
+      <x:c r="I100" s="7" t="str">
+        <x:v>不补UT</x:v>
+      </x:c>
+      <x:c r="J100" s="7" t="str">
+        <x:v>使用指南展示属于页面展示场景；文案结构已有基础 UT，不再补。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" s="1" customFormat="1" ht="28.5" customHeight="1">
+      <x:c r="A101" s="4" t="str">
+        <x:v>HELP-003</x:v>
+      </x:c>
+      <x:c r="B101" s="5" t="str">
+        <x:v>帮助与反馈</x:v>
+      </x:c>
+      <x:c r="C101" s="5" t="str">
+        <x:v>FAQ展开收起</x:v>
+      </x:c>
+      <x:c r="D101" s="5" t="str">
+        <x:v>验证 FAQ 可以展开和收起</x:v>
+      </x:c>
+      <x:c r="E101" s="5" t="str">
+        <x:v>已进入帮助与反馈页</x:v>
+      </x:c>
+      <x:c r="F101" s="5" t="str">
         <x:v>1. 点击任一 FAQ 展开按钮
 2. 再次点击收起按钮</x:v>
       </x:c>
-      <x:c r="G100" s="5" t="str">
+      <x:c r="G101" s="5" t="str">
         <x:v>1. 首次点击展示答案
 2. 再次点击隐藏答案
 3. 按钮文案在展开和收起间切换</x:v>
       </x:c>
-      <x:c r="H100" s="5"/>
-      <x:c r="I100" s="7" t="str">
-        <x:v>不补UT</x:v>
-      </x:c>
-      <x:c r="J100" s="7" t="str">
-        <x:v>FAQ 展开收起属于页面交互场景，不进入本轮 UT 补充范围。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="101" s="1" customFormat="1" ht="28.5" customHeight="1">
-      <x:c r="A101" s="4" t="str">
-        <x:v>HELP-004</x:v>
-      </x:c>
-      <x:c r="B101" s="5" t="str">
-        <x:v>帮助与反馈</x:v>
-      </x:c>
-      <x:c r="C101" s="5" t="str">
-        <x:v>联系方式展示</x:v>
-      </x:c>
-      <x:c r="D101" s="5" t="str">
-        <x:v>验证联系与反馈信息展示正确</x:v>
-      </x:c>
-      <x:c r="E101" s="5" t="str">
-        <x:v>已进入帮助与反馈页</x:v>
-      </x:c>
-      <x:c r="F101" s="5" t="str">
-        <x:v>1. 查看联系与反馈区域</x:v>
-      </x:c>
-      <x:c r="G101" s="5" t="str">
-        <x:v>1. 展示反馈邮箱
-2. 邮箱内容为 `consumer@huawei.com`</x:v>
-      </x:c>
       <x:c r="H101" s="5"/>
       <x:c r="I101" s="7" t="str">
         <x:v>不补UT</x:v>
       </x:c>
       <x:c r="J101" s="7" t="str">
-        <x:v>联系方式展示属于页面展示场景；文案结构已有基础 UT，不再补。</x:v>
+        <x:v>FAQ 展开收起属于页面交互场景，不进入本轮 UT 补充范围。</x:v>
       </x:c>
     </x:row>
     <x:row r="102" s="1" customFormat="1" ht="42.75" customHeight="1">
       <x:c r="A102" s="4" t="str">
-        <x:v>NAV-001</x:v>
+        <x:v>HELP-004</x:v>
       </x:c>
       <x:c r="B102" s="5" t="str">
-        <x:v>全局导航与主题</x:v>
+        <x:v>帮助与反馈</x:v>
       </x:c>
       <x:c r="C102" s="5" t="str">
-        <x:v>侧边栏导航</x:v>
+        <x:v>联系方式展示</x:v>
       </x:c>
       <x:c r="D102" s="5" t="str">
-        <x:v>验证侧边栏可以进入所有主模块</x:v>
+        <x:v>验证联系与反馈信息展示正确</x:v>
       </x:c>
       <x:c r="E102" s="5" t="str">
-        <x:v>应用处于安全总览页</x:v>
+        <x:v>已进入帮助与反馈页</x:v>
       </x:c>
       <x:c r="F102" s="5" t="str">
-        <x:v>1. 依次点击侧边栏防火墙、日志、外设、身份鉴别、工具设置</x:v>
+        <x:v>1. 查看联系与反馈区域</x:v>
       </x:c>
       <x:c r="G102" s="5" t="str">
-        <x:v>1. 每次均进入对应页面
-2. 侧边栏选中态同步更新</x:v>
+        <x:v>1. 展示反馈邮箱
+2. 邮箱内容为 `consumer@huawei.com`</x:v>
       </x:c>
       <x:c r="H102" s="5"/>
       <x:c r="I102" s="7" t="str">
         <x:v>不补UT</x:v>
       </x:c>
       <x:c r="J102" s="7" t="str">
-        <x:v>导航、弹窗或菜单交互属于 UI/ohosTest 范围，不进入本轮 UT 补充范围。</x:v>
+        <x:v>联系方式展示属于页面展示场景；文案结构已有基础 UT，不再补。</x:v>
       </x:c>
     </x:row>
     <x:row r="103" s="1" customFormat="1" ht="42.75" customHeight="1">
       <x:c r="A103" s="4" t="str">
-        <x:v>NAV-002</x:v>
+        <x:v>NAV-001</x:v>
       </x:c>
       <x:c r="B103" s="5" t="str">
         <x:v>全局导航与主题</x:v>
       </x:c>
       <x:c r="C103" s="5" t="str">
-        <x:v>返回按钮</x:v>
+        <x:v>侧边栏导航</x:v>
       </x:c>
       <x:c r="D103" s="5" t="str">
-        <x:v>验证子页面返回按钮回到安全总览或上级页面</x:v>
+        <x:v>验证侧边栏可以进入所有主模块</x:v>
       </x:c>
       <x:c r="E103" s="5" t="str">
-        <x:v>已进入任一子页面</x:v>
+        <x:v>应用处于安全总览页</x:v>
       </x:c>
       <x:c r="F103" s="5" t="str">
-        <x:v>1. 点击页面左上角返回按钮</x:v>
+        <x:v>1. 依次点击侧边栏防火墙、日志、外设、身份鉴别、工具设置</x:v>
       </x:c>
       <x:c r="G103" s="5" t="str">
-        <x:v>1. 返回到预期上级页面
-2. 页面不闪退、不空白</x:v>
+        <x:v>1. 每次均进入对应页面
+2. 侧边栏选中态同步更新</x:v>
       </x:c>
       <x:c r="H103" s="5"/>
       <x:c r="I103" s="7" t="str">
@@ -4494,27 +4497,26 @@
     </x:row>
     <x:row r="104" s="1" customFormat="1" ht="42.75" customHeight="1">
       <x:c r="A104" s="4" t="str">
-        <x:v>NAV-003</x:v>
+        <x:v>NAV-002</x:v>
       </x:c>
       <x:c r="B104" s="5" t="str">
         <x:v>全局导航与主题</x:v>
       </x:c>
       <x:c r="C104" s="5" t="str">
-        <x:v>主题菜单</x:v>
+        <x:v>返回按钮</x:v>
       </x:c>
       <x:c r="D104" s="5" t="str">
-        <x:v>验证右上角主题菜单可以打开和关闭</x:v>
+        <x:v>验证子页面返回按钮回到安全总览或上级页面</x:v>
       </x:c>
       <x:c r="E104" s="5" t="str">
-        <x:v>应用处于任一页面</x:v>
+        <x:v>已进入任一子页面</x:v>
       </x:c>
       <x:c r="F104" s="5" t="str">
-        <x:v>1. 点击右上角菜单按钮
-2. 点击页面空白区域</x:v>
+        <x:v>1. 点击页面左上角返回按钮</x:v>
       </x:c>
       <x:c r="G104" s="5" t="str">
-        <x:v>1. 菜单打开后展示主题、帮助、关于等入口
-2. 点击空白区域后菜单关闭</x:v>
+        <x:v>1. 返回到预期上级页面
+2. 页面不闪退、不空白</x:v>
       </x:c>
       <x:c r="H104" s="5"/>
       <x:c r="I104" s="7" t="str">
@@ -4526,230 +4528,262 @@
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="4" t="str">
-        <x:v>NAV-004</x:v>
+        <x:v>NAV-003</x:v>
       </x:c>
       <x:c r="B105" s="5" t="str">
         <x:v>全局导航与主题</x:v>
       </x:c>
       <x:c r="C105" s="5" t="str">
+        <x:v>主题菜单</x:v>
+      </x:c>
+      <x:c r="D105" s="5" t="str">
+        <x:v>验证右上角主题菜单可以打开和关闭</x:v>
+      </x:c>
+      <x:c r="E105" s="5" t="str">
+        <x:v>应用处于任一页面</x:v>
+      </x:c>
+      <x:c r="F105" s="5" t="str">
+        <x:v>1. 点击右上角菜单按钮
+2. 点击页面空白区域</x:v>
+      </x:c>
+      <x:c r="G105" s="5" t="str">
+        <x:v>1. 菜单打开后展示主题、帮助、关于等入口
+2. 点击空白区域后菜单关闭</x:v>
+      </x:c>
+      <x:c r="H105" s="5"/>
+      <x:c r="I105" s="7" t="str">
+        <x:v>不补UT</x:v>
+      </x:c>
+      <x:c r="J105" s="7" t="str">
+        <x:v>导航、弹窗或菜单交互属于 UI/ohosTest 范围，不进入本轮 UT 补充范围。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" s="4" t="str">
+        <x:v>NAV-004</x:v>
+      </x:c>
+      <x:c r="B106" s="5" t="str">
+        <x:v>全局导航与主题</x:v>
+      </x:c>
+      <x:c r="C106" s="5" t="str">
         <x:v>深浅色切换</x:v>
       </x:c>
-      <x:c r="D105" s="5" t="str">
+      <x:c r="D106" s="5" t="str">
         <x:v>验证浅色模式切换生效</x:v>
       </x:c>
-      <x:c r="E105" s="5" t="str">
+      <x:c r="E106" s="5" t="str">
         <x:v>应用可正常打开</x:v>
       </x:c>
-      <x:c r="F105" s="5" t="str">
+      <x:c r="F106" s="5" t="str">
         <x:v>1. 打开右上角菜单
 2. 选择浅色模式</x:v>
       </x:c>
-      <x:c r="G105" s="5" t="str">
+      <x:c r="G106" s="5" t="str">
         <x:v>1. 页面切换为浅色主题
 2. 顶部窗口按钮样式同步浅色配置</x:v>
       </x:c>
-      <x:c r="H105" s="5"/>
-      <x:c r="I105" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J105" s="7" t="str">
+      <x:c r="H106" s="5"/>
+      <x:c r="I106" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J106" s="7" t="str">
         <x:v>entry/src/test/theme/theme-manager.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="106">
-      <x:c r="A106" s="4" t="str">
+    <x:row r="107">
+      <x:c r="A107" t="str">
         <x:v>NAV-005</x:v>
       </x:c>
-      <x:c r="B106" s="5" t="str">
+      <x:c r="B107" t="str">
         <x:v>全局导航与主题</x:v>
       </x:c>
-      <x:c r="C106" s="5" t="str">
+      <x:c r="C107" t="str">
         <x:v>深浅色切换</x:v>
       </x:c>
-      <x:c r="D106" s="5" t="str">
+      <x:c r="D107" t="str">
         <x:v>验证深色模式切换生效</x:v>
       </x:c>
-      <x:c r="E106" s="5" t="str">
+      <x:c r="E107" t="str">
         <x:v>应用可正常打开</x:v>
       </x:c>
-      <x:c r="F106" s="5" t="str">
+      <x:c r="F107" t="str">
         <x:v>1. 打开右上角菜单
 2. 选择深色模式</x:v>
       </x:c>
-      <x:c r="G106" s="5" t="str">
+      <x:c r="G107" t="str">
         <x:v>1. 页面切换为深色主题
 2. 页面文字、背景、图标对比度正常</x:v>
       </x:c>
-      <x:c r="H106" s="5"/>
-      <x:c r="I106" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J106" s="7" t="str">
+      <x:c r="H107"/>
+      <x:c r="I107" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J107" t="str">
         <x:v>entry/src/test/theme/theme-manager.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="107">
-      <x:c r="A107" t="str">
+    <x:row r="108">
+      <x:c r="A108" t="str">
         <x:v>NAV-006</x:v>
       </x:c>
-      <x:c r="B107" t="str">
+      <x:c r="B108" t="str">
         <x:v>全局导航与主题</x:v>
       </x:c>
-      <x:c r="C107" t="str">
+      <x:c r="C108" t="str">
         <x:v>深浅色切换</x:v>
       </x:c>
-      <x:c r="D107" t="str">
+      <x:c r="D108" t="str">
         <x:v>验证跟随系统模式保存和回显</x:v>
       </x:c>
-      <x:c r="E107" t="str">
+      <x:c r="E108" t="str">
         <x:v>系统主题可切换</x:v>
       </x:c>
-      <x:c r="F107" t="str">
+      <x:c r="F108" t="str">
         <x:v>1. 打开右上角菜单
 2. 选择跟随系统
 3. 重启应用</x:v>
       </x:c>
-      <x:c r="G107" t="str">
+      <x:c r="G108" t="str">
         <x:v>1. 应用主题跟随系统当前主题
 2. 菜单中当前选项回显正确</x:v>
       </x:c>
-      <x:c r="H107"/>
-      <x:c r="I107" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J107" t="str">
+      <x:c r="H108"/>
+      <x:c r="I108" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J108" t="str">
         <x:v>entry/src/test/theme/theme-manager.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="108">
-      <x:c r="A108" t="str">
+    <x:row r="109">
+      <x:c r="A109" t="str">
         <x:v>NAV-007</x:v>
       </x:c>
-      <x:c r="B108" t="str">
+      <x:c r="B109" t="str">
         <x:v>全局导航与主题</x:v>
       </x:c>
-      <x:c r="C108" t="str">
+      <x:c r="C109" t="str">
         <x:v>关于弹窗</x:v>
       </x:c>
-      <x:c r="D108" t="str">
+      <x:c r="D109" t="str">
         <x:v>验证关于弹窗展示应用信息</x:v>
       </x:c>
-      <x:c r="E108" t="str">
+      <x:c r="E109" t="str">
         <x:v>应用处于任一页面</x:v>
       </x:c>
-      <x:c r="F108" t="str">
+      <x:c r="F109" t="str">
         <x:v>1. 打开右上角菜单
 2. 点击关于</x:v>
       </x:c>
-      <x:c r="G108" t="str">
+      <x:c r="G109" t="str">
         <x:v>1. 弹窗展示应用名称、版本和版权信息
 2. 点击确定后弹窗关闭</x:v>
       </x:c>
-      <x:c r="H108"/>
-      <x:c r="I108" t="str">
+      <x:c r="H109"/>
+      <x:c r="I109" t="str">
         <x:v>不补UT</x:v>
       </x:c>
-      <x:c r="J108" t="str">
+      <x:c r="J109" t="str">
         <x:v>导航、弹窗或菜单交互属于 UI/ohosTest 范围，不进入本轮 UT 补充范围。</x:v>
       </x:c>
     </x:row>
-    <x:row r="109">
-      <x:c r="A109" t="str">
+    <x:row r="110">
+      <x:c r="A110" t="str">
         <x:v>SYS-005</x:v>
       </x:c>
-      <x:c r="B109" t="str">
+      <x:c r="B110" t="str">
         <x:v>系统集成基础</x:v>
       </x:c>
-      <x:c r="C109" t="str">
+      <x:c r="C110" t="str">
         <x:v>导出文件能力</x:v>
       </x:c>
-      <x:c r="D109" t="str">
+      <x:c r="D110" t="str">
         <x:v>验证通用 CSV 导出能力正常</x:v>
       </x:c>
-      <x:c r="E109" t="str">
+      <x:c r="E110" t="str">
         <x:v>日志或外设存在可导出数据</x:v>
       </x:c>
-      <x:c r="F109" t="str">
+      <x:c r="F110" t="str">
         <x:v>1. 在任一支持导出的页面点击导出
 2. 打开导出文件</x:v>
       </x:c>
-      <x:c r="G109" t="str">
+      <x:c r="G110" t="str">
         <x:v>1. 文件保存成功
 2. 文件编码和表头正确
 3. 中文内容不乱码</x:v>
       </x:c>
-      <x:c r="H109"/>
-      <x:c r="I109" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J109" t="str">
+      <x:c r="H110"/>
+      <x:c r="I110" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J110" t="str">
         <x:v>entry/src/test/common/csv-file-export-service.test.ets；entry/src/test/log-manage/export-service.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="110">
-      <x:c r="A110" t="str">
+    <x:row r="111">
+      <x:c r="A111" t="str">
         <x:v>SYS-006</x:v>
       </x:c>
-      <x:c r="B110" t="str">
+      <x:c r="B111" t="str">
         <x:v>系统集成基础</x:v>
       </x:c>
-      <x:c r="C110" t="str">
+      <x:c r="C111" t="str">
         <x:v>本地存储能力</x:v>
       </x:c>
-      <x:c r="D110" t="str">
+      <x:c r="D111" t="str">
         <x:v>验证设置类配置重启后可恢复</x:v>
       </x:c>
-      <x:c r="E110" t="str">
+      <x:c r="E111" t="str">
         <x:v>已修改工具设置或日志存储设置</x:v>
       </x:c>
-      <x:c r="F110" t="str">
+      <x:c r="F111" t="str">
         <x:v>1. 保存配置
 2. 关闭并重启应用
 3. 重新进入对应页面</x:v>
       </x:c>
-      <x:c r="G110" t="str">
+      <x:c r="G111" t="str">
         <x:v>1. 页面回显上次保存配置
 2. 无默认值覆盖已保存配置</x:v>
       </x:c>
-      <x:c r="H110"/>
-      <x:c r="I110" t="str">
+      <x:c r="H111"/>
+      <x:c r="I111" t="str">
         <x:v>不补UT</x:v>
       </x:c>
-      <x:c r="J110" t="str">
+      <x:c r="J111" t="str">
         <x:v>重启后恢复属于集成语义；存储读写已有基础 UT，不再补。</x:v>
       </x:c>
     </x:row>
-    <x:row r="111">
-      <x:c r="A111" t="str">
+    <x:row r="112">
+      <x:c r="A112" t="str">
         <x:v>SYS-007</x:v>
       </x:c>
-      <x:c r="B111" t="str">
+      <x:c r="B112" t="str">
         <x:v>系统集成基础</x:v>
       </x:c>
-      <x:c r="C111" t="str">
+      <x:c r="C112" t="str">
         <x:v>应用恢复</x:v>
       </x:c>
-      <x:c r="D111" t="str">
+      <x:c r="D112" t="str">
         <x:v>验证应用前后台切换后当前页面状态正常</x:v>
       </x:c>
-      <x:c r="E111" t="str">
+      <x:c r="E112" t="str">
         <x:v>应用已打开任一业务页面</x:v>
       </x:c>
-      <x:c r="F111" t="str">
+      <x:c r="F112" t="str">
         <x:v>1. 将应用切到后台
 2. 等待 5 秒
 3. 恢复到前台</x:v>
       </x:c>
-      <x:c r="G111" t="str">
+      <x:c r="G112" t="str">
         <x:v>1. 当前页面仍可操作
 2. 关键数据自动刷新或保持一致
 3. 无崩溃</x:v>
       </x:c>
-      <x:c r="H111"/>
-      <x:c r="I111" t="str">
+      <x:c r="H112"/>
+      <x:c r="I112" t="str">
         <x:v>不补UT</x:v>
       </x:c>
-      <x:c r="J111" t="str">
+      <x:c r="J112" t="str">
         <x:v>前后台切换属于应用生命周期集成场景，不进入本轮 UT 补充范围。</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
docs: lock usb storage policy conflict fixes
</commit_message>
<xml_diff>
--- a/docs/04-测试文档/手工测试用例/测试用例基线.xlsx
+++ b/docs/04-测试文档/手工测试用例/测试用例基线.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例_ai" sheetId="1" r:id="R1e6d9a190c1f4ae1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例_ai" sheetId="1" r:id="R8110e46ef7734661"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3973,582 +3973,587 @@
     </x:row>
     <x:row r="88" s="1" customFormat="1" ht="42.75" customHeight="1">
       <x:c r="A88" s="4" t="str">
+        <x:v>PER-034</x:v>
+      </x:c>
+      <x:c r="B88" s="5" t="str">
+        <x:v>外设管理</x:v>
+      </x:c>
+      <x:c r="C88" s="5" t="str">
+        <x:v>设备连接记录</x:v>
+      </x:c>
+      <x:c r="D88" s="5" t="str">
+        <x:v>验证 USB 存储只读且本地存在禁止接入策略时，连接记录优先展示禁止接入</x:v>
+      </x:c>
+      <x:c r="E88" s="5" t="str">
+        <x:v>USB 存储策略当前为 `只读`，目标 U 盘已存在本地 deny 策略</x:v>
+      </x:c>
+      <x:c r="F88" s="5" t="str">
+        <x:v>1. 进入接口管控页签，确认 USB 存储策略为 `只读`
+2. 保持目标 U 盘在黑白名单中为 `禁止接入`
+3. 插入目标 U 盘并查看设备连接记录</x:v>
+      </x:c>
+      <x:c r="G88" s="5" t="str">
+        <x:v>1. 本次连接记录正常落库
+2. 记录策略展示为已禁用或禁止接入
+3. 命中类型优先体现单设备禁止接入，不被 USB 存储只读覆盖</x:v>
+      </x:c>
+      <x:c r="H88" s="5"/>
+      <x:c r="I88" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J88" s="7" t="str">
+        <x:v>entry/src/test/peripheral/connection-record-usb-consumer.test.ets</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" s="1" customFormat="1" ht="42.75" customHeight="1">
+      <x:c r="A89" s="4" t="str">
+        <x:v>PER-035</x:v>
+      </x:c>
+      <x:c r="B89" s="5" t="str">
+        <x:v>外设管理</x:v>
+      </x:c>
+      <x:c r="C89" s="5" t="str">
+        <x:v>单设备策略切换</x:v>
+      </x:c>
+      <x:c r="D89" s="5" t="str">
+        <x:v>验证 USB 存储总策略为禁止访问时，黑白名单不允许将 USB 存储设备切换为禁止接入</x:v>
+      </x:c>
+      <x:c r="E89" s="5" t="str">
+        <x:v>USB 存储策略当前为 `禁止访问`，黑白名单中存在目标 USB 存储设备</x:v>
+      </x:c>
+      <x:c r="F89" s="5" t="str">
+        <x:v>1. 进入接口管控页签，确认 USB 存储策略为 `禁止访问`
+2. 进入黑白名单页签
+3. 将目标 USB 存储设备从 `允许接入` 切换为 `禁止接入`</x:v>
+      </x:c>
+      <x:c r="G89" s="5" t="str">
+        <x:v>1. 系统下发被拦截并返回 USB 存储账户级冲突
+2. 本地黑白名单不写入 deny 策略
+3. 页面保持原本单设备策略状态并展示失败提示</x:v>
+      </x:c>
+      <x:c r="H89" s="5"/>
+      <x:c r="I89" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J89" s="7" t="str">
+        <x:v>entry/src/test/peripheral/device-policy-dispatch-service.test.ets</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" s="1" customFormat="1" ht="28.5" customHeight="1">
+      <x:c r="A90" s="4" t="str">
         <x:v>ID-001</x:v>
       </x:c>
-      <x:c r="B88" s="5" t="str">
+      <x:c r="B90" s="5" t="str">
         <x:v>身份鉴别</x:v>
       </x:c>
-      <x:c r="C88" s="5" t="str">
+      <x:c r="C90" s="5" t="str">
         <x:v>口令复杂度策略</x:v>
       </x:c>
-      <x:c r="D88" s="5" t="str">
+      <x:c r="D90" s="5" t="str">
         <x:v>验证保存口令复杂度策略：最小长度 8，大写/小写/数字开启，特殊字符关闭</x:v>
       </x:c>
-      <x:c r="E88" s="5" t="str">
+      <x:c r="E90" s="5" t="str">
         <x:v>应用已激活企业管理员</x:v>
       </x:c>
-      <x:c r="F88" s="5" t="str">
+      <x:c r="F90" s="5" t="str">
         <x:v>1. 进入身份鉴别页
 2. 设置最小长度为 `8`
 3. 开启大写字母、小写字母、数字要求
 4. 关闭特殊字符要求
 5. 点击保存身份鉴别配置</x:v>
       </x:c>
-      <x:c r="G88" s="5" t="str">
+      <x:c r="G90" s="5" t="str">
         <x:v>1. 页面提示身份鉴别配置已保存
 2. 系统设置中策略显示与配置一致</x:v>
       </x:c>
-      <x:c r="H88" s="5"/>
-      <x:c r="I88" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J88" s="7" t="str">
+      <x:c r="H90" s="5"/>
+      <x:c r="I90" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J90" s="7" t="str">
         <x:v>entry/src/test/identity/settings-viewmodel.test.ets；entry/src/test/identity/service.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="89" s="1" customFormat="1" ht="42.75" customHeight="1">
-      <x:c r="A89" s="4" t="str">
+    <x:row r="91" s="1" customFormat="1" ht="28.5" customHeight="1">
+      <x:c r="A91" s="4" t="str">
         <x:v>ID-002</x:v>
       </x:c>
-      <x:c r="B89" s="5" t="str">
+      <x:c r="B91" s="5" t="str">
         <x:v>身份鉴别</x:v>
       </x:c>
-      <x:c r="C89" s="5" t="str">
+      <x:c r="C91" s="5" t="str">
         <x:v>密码有效期策略</x:v>
       </x:c>
-      <x:c r="D89" s="5" t="str">
+      <x:c r="D91" s="5" t="str">
         <x:v>验证将密码有效期设置为 180 天后保存成功</x:v>
       </x:c>
-      <x:c r="E89" s="5" t="str">
+      <x:c r="E91" s="5" t="str">
         <x:v>应用已激活企业管理员</x:v>
       </x:c>
-      <x:c r="F89" s="5" t="str">
+      <x:c r="F91" s="5" t="str">
         <x:v>1. 进入身份鉴别页
 2. 选择密码有效期 `180天`
 3. 点击保存</x:v>
       </x:c>
-      <x:c r="G89" s="5" t="str">
+      <x:c r="G91" s="5" t="str">
         <x:v>1. 页面提示保存成功
 2. 再次进入页面可回显 `180天`</x:v>
       </x:c>
-      <x:c r="H89" s="5"/>
-      <x:c r="I89" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J89" s="7" t="str">
+      <x:c r="H91" s="5"/>
+      <x:c r="I91" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J91" s="7" t="str">
         <x:v>entry/src/test/identity/settings-viewmodel.test.ets；entry/src/test/identity/service.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="90" s="1" customFormat="1" ht="28.5" customHeight="1">
-      <x:c r="A90" s="4" t="str">
+    <x:row r="92" s="1" customFormat="1" ht="42.75" customHeight="1">
+      <x:c r="A92" s="4" t="str">
         <x:v>ID-003</x:v>
       </x:c>
-      <x:c r="B90" s="5" t="str">
+      <x:c r="B92" s="5" t="str">
         <x:v>身份鉴别</x:v>
       </x:c>
-      <x:c r="C90" s="5" t="str">
+      <x:c r="C92" s="5" t="str">
         <x:v>密码有效期策略</x:v>
       </x:c>
-      <x:c r="D90" s="5" t="str">
+      <x:c r="D92" s="5" t="str">
         <x:v>验证将自定义密码有效期设置为 30 天后保存成功</x:v>
       </x:c>
-      <x:c r="E90" s="5" t="str">
+      <x:c r="E92" s="5" t="str">
         <x:v>应用已激活企业管理员</x:v>
       </x:c>
-      <x:c r="F90" s="5" t="str">
+      <x:c r="F92" s="5" t="str">
         <x:v>1. 进入身份鉴别页
 2. 选择自定义有效期
 3. 输入 `30`
 4. 点击保存</x:v>
       </x:c>
-      <x:c r="G90" s="5" t="str">
+      <x:c r="G92" s="5" t="str">
         <x:v>1. 页面提示保存成功
 2. 再次进入页面可回显 `30天`</x:v>
       </x:c>
-      <x:c r="H90" s="5"/>
-      <x:c r="I90" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J90" s="7" t="str">
+      <x:c r="H92" s="5"/>
+      <x:c r="I92" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J92" s="7" t="str">
         <x:v>entry/src/test/identity/settings-viewmodel.test.ets；entry/src/test/identity/service.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="91" s="1" customFormat="1" ht="28.5" customHeight="1">
-      <x:c r="A91" s="4" t="str">
+    <x:row r="93" s="1" customFormat="1" ht="42.75" customHeight="1">
+      <x:c r="A93" s="4" t="str">
         <x:v>ID-004</x:v>
       </x:c>
-      <x:c r="B91" s="5" t="str">
+      <x:c r="B93" s="5" t="str">
         <x:v>身份鉴别</x:v>
       </x:c>
-      <x:c r="C91" s="5" t="str">
+      <x:c r="C93" s="5" t="str">
         <x:v>输入参数校验</x:v>
       </x:c>
-      <x:c r="D91" s="5" t="str">
+      <x:c r="D93" s="5" t="str">
         <x:v>验证自定义密码有效期非法字符被过滤，空值保存时被拦截</x:v>
       </x:c>
-      <x:c r="E91" s="5" t="str">
+      <x:c r="E93" s="5" t="str">
         <x:v>已选择自定义有效期</x:v>
       </x:c>
-      <x:c r="F91" s="5" t="str">
+      <x:c r="F93" s="5" t="str">
         <x:v>1. 选择自定义有效期
 2. 尝试输入 abc、-1 等非法字符
 3. 清空输入框
 4. 点击保存</x:v>
       </x:c>
-      <x:c r="G91" s="5" t="str">
+      <x:c r="G93" s="5" t="str">
         <x:v>1. 非法字符不会保留在输入框中，或仅保留数字字符
 2. 自定义有效期为空时点击保存，页面提示请输入非负整数天数
 3. 未通过校验时不下发策略</x:v>
       </x:c>
-      <x:c r="H91" s="5"/>
-      <x:c r="I91" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J91" s="7" t="str">
+      <x:c r="H93" s="5"/>
+      <x:c r="I93" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J93" s="7" t="str">
         <x:v>entry/src/test/identity/settings-viewmodel.test.ets；entry/src/test/identity/service.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="92" s="1" customFormat="1" ht="42.75" customHeight="1">
-      <x:c r="A92" s="4" t="str">
+    <x:row r="94" s="1" customFormat="1" ht="28.5" customHeight="1">
+      <x:c r="A94" s="4" t="str">
         <x:v>ID-007</x:v>
       </x:c>
-      <x:c r="B92" s="5" t="str">
+      <x:c r="B94" s="5" t="str">
         <x:v>身份鉴别</x:v>
       </x:c>
-      <x:c r="C92" s="5" t="str">
+      <x:c r="C94" s="5" t="str">
         <x:v>策略保存</x:v>
       </x:c>
-      <x:c r="D92" s="5" t="str">
+      <x:c r="D94" s="5" t="str">
         <x:v>验证自定义密码有效期输入 0 天时触发风险提示</x:v>
       </x:c>
-      <x:c r="E92" s="5" t="str">
+      <x:c r="E94" s="5" t="str">
         <x:v>应用已激活企业管理员，已选择自定义有效期</x:v>
       </x:c>
-      <x:c r="F92" s="5" t="str">
+      <x:c r="F94" s="5" t="str">
         <x:v>1. 输入 `0`
 2. 点击保存</x:v>
       </x:c>
-      <x:c r="G92" s="5" t="str">
+      <x:c r="G94" s="5" t="str">
         <x:v>1. 页面弹出风险提示
 2. 用户确认前不直接保存策略</x:v>
       </x:c>
-      <x:c r="H92" s="5"/>
-      <x:c r="I92" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J92" s="7" t="str">
+      <x:c r="H94" s="5"/>
+      <x:c r="I94" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J94" s="7" t="str">
         <x:v>entry/src/test/identity/settings-viewmodel.test.ets；entry/src/test/identity/service.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="93" s="1" customFormat="1" ht="42.75" customHeight="1">
-      <x:c r="A93" s="4" t="str">
+    <x:row r="95" s="1" customFormat="1" ht="28.5" customHeight="1">
+      <x:c r="A95" s="4" t="str">
         <x:v>SET-002</x:v>
       </x:c>
-      <x:c r="B93" s="5" t="str">
+      <x:c r="B95" s="5" t="str">
         <x:v>工具设置</x:v>
       </x:c>
-      <x:c r="C93" s="5" t="str">
+      <x:c r="C95" s="5" t="str">
         <x:v>启动认证开关</x:v>
       </x:c>
-      <x:c r="D93" s="5" t="str">
+      <x:c r="D95" s="5" t="str">
         <x:v>验证关闭启动时身份校验后保存成功</x:v>
       </x:c>
-      <x:c r="E93" s="5" t="str">
+      <x:c r="E95" s="5" t="str">
         <x:v>启动时身份校验当前已开启</x:v>
       </x:c>
-      <x:c r="F93" s="5" t="str">
+      <x:c r="F95" s="5" t="str">
         <x:v>1. 进入工具设置页
 2. 关闭启动时身份校验
 3. 点击保存设置</x:v>
       </x:c>
-      <x:c r="G93" s="5" t="str">
+      <x:c r="G95" s="5" t="str">
         <x:v>1. 页面提示工具设置已保存
 2. 重启应用后不再要求启动认证</x:v>
       </x:c>
-      <x:c r="H93" s="5"/>
-      <x:c r="I93" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J93" s="7" t="str">
+      <x:c r="H95" s="5"/>
+      <x:c r="I95" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J95" s="7" t="str">
         <x:v>entry/src/test/tool-settings/viewmodel.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="94" s="1" customFormat="1" ht="28.5" customHeight="1">
-      <x:c r="A94" s="4" t="str">
+    <x:row r="96" s="1" customFormat="1" ht="28.5" customHeight="1">
+      <x:c r="A96" s="4" t="str">
         <x:v>SET-003</x:v>
       </x:c>
-      <x:c r="B94" s="5" t="str">
+      <x:c r="B96" s="5" t="str">
         <x:v>工具设置</x:v>
       </x:c>
-      <x:c r="C94" s="5" t="str">
+      <x:c r="C96" s="5" t="str">
         <x:v>认证方式选择</x:v>
       </x:c>
-      <x:c r="D94" s="5" t="str">
+      <x:c r="D96" s="5" t="str">
         <x:v>验证选择 PIN 认证方式后保存成功</x:v>
       </x:c>
-      <x:c r="E94" s="5" t="str">
+      <x:c r="E96" s="5" t="str">
         <x:v>启动时身份校验已开启，系统 PIN 可用</x:v>
       </x:c>
-      <x:c r="F94" s="5" t="str">
+      <x:c r="F96" s="5" t="str">
         <x:v>1. 进入工具设置页
 2. 选择 `PIN` 认证方式
 3. 点击保存设置</x:v>
       </x:c>
-      <x:c r="G94" s="5" t="str">
+      <x:c r="G96" s="5" t="str">
         <x:v>1. 页面提示保存成功
 2. 重启应用后按 PIN 方式进行校验</x:v>
       </x:c>
-      <x:c r="H94" s="5"/>
-      <x:c r="I94" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J94" s="7" t="str">
+      <x:c r="H96" s="5"/>
+      <x:c r="I96" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J96" s="7" t="str">
         <x:v>entry/src/test/tool-settings/viewmodel.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="95" s="1" customFormat="1" ht="28.5" customHeight="1">
-      <x:c r="A95" s="4" t="str">
+    <x:row r="97" s="1" customFormat="1" ht="28.5" customHeight="1">
+      <x:c r="A97" s="4" t="str">
         <x:v>SET-004</x:v>
       </x:c>
-      <x:c r="B95" s="5" t="str">
+      <x:c r="B97" s="5" t="str">
         <x:v>工具设置</x:v>
       </x:c>
-      <x:c r="C95" s="5" t="str">
+      <x:c r="C97" s="5" t="str">
         <x:v>认证方式选择</x:v>
       </x:c>
-      <x:c r="D95" s="5" t="str">
+      <x:c r="D97" s="5" t="str">
         <x:v>验证选择指纹认证方式后保存成功</x:v>
       </x:c>
-      <x:c r="E95" s="5" t="str">
+      <x:c r="E97" s="5" t="str">
         <x:v>设备已录入指纹且系统指纹认证可用</x:v>
       </x:c>
-      <x:c r="F95" s="5" t="str">
+      <x:c r="F97" s="5" t="str">
         <x:v>1. 进入工具设置页
 2. 选择 `指纹` 认证方式
 3. 点击保存设置</x:v>
       </x:c>
-      <x:c r="G95" s="5" t="str">
+      <x:c r="G97" s="5" t="str">
         <x:v>1. 页面提示保存成功
 2. 重启应用后按指纹方式进行校验</x:v>
       </x:c>
-      <x:c r="H95" s="5"/>
-      <x:c r="I95" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J95" s="7" t="str">
+      <x:c r="H97" s="5"/>
+      <x:c r="I97" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J97" s="7" t="str">
         <x:v>entry/src/test/tool-settings/viewmodel.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="96" s="1" customFormat="1" ht="28.5" customHeight="1">
-      <x:c r="A96" s="4" t="str">
+    <x:row r="98" s="1" customFormat="1" ht="28.5" customHeight="1">
+      <x:c r="A98" s="4" t="str">
         <x:v>SET-005</x:v>
       </x:c>
-      <x:c r="B96" s="5" t="str">
+      <x:c r="B98" s="5" t="str">
         <x:v>工具设置</x:v>
       </x:c>
-      <x:c r="C96" s="5" t="str">
+      <x:c r="C98" s="5" t="str">
         <x:v>无变更保存</x:v>
       </x:c>
-      <x:c r="D96" s="5" t="str">
+      <x:c r="D98" s="5" t="str">
         <x:v>验证未修改设置时保存按钮不可点击</x:v>
       </x:c>
-      <x:c r="E96" s="5" t="str">
+      <x:c r="E98" s="5" t="str">
         <x:v>进入工具设置页且不修改任何配置</x:v>
       </x:c>
-      <x:c r="F96" s="5" t="str">
+      <x:c r="F98" s="5" t="str">
         <x:v>1. 进入工具设置页
 2. 不做任何修改
 3. 观察保存按钮状态</x:v>
       </x:c>
-      <x:c r="G96" s="5" t="str">
+      <x:c r="G98" s="5" t="str">
         <x:v>1. 保存按钮保持不可点击状态
 2. 页面不触发保存动作</x:v>
       </x:c>
-      <x:c r="H96" s="5"/>
-      <x:c r="I96" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J96" s="7" t="str">
+      <x:c r="H98" s="5"/>
+      <x:c r="I98" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J98" s="7" t="str">
         <x:v>entry/src/test/tool-settings/viewmodel.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="97" s="1" customFormat="1" ht="28.5" customHeight="1">
-      <x:c r="A97" s="4" t="str">
+    <x:row r="99" s="1" customFormat="1" ht="28.5" customHeight="1">
+      <x:c r="A99" s="4" t="str">
         <x:v>SET-006</x:v>
       </x:c>
-      <x:c r="B97" s="5" t="str">
+      <x:c r="B99" s="5" t="str">
         <x:v>工具设置</x:v>
       </x:c>
-      <x:c r="C97" s="5" t="str">
+      <x:c r="C99" s="5" t="str">
         <x:v>认证方式不可用提示</x:v>
       </x:c>
-      <x:c r="D97" s="5" t="str">
+      <x:c r="D99" s="5" t="str">
         <x:v>验证选择当前设备不可用的认证方式时出现不可用确认提示</x:v>
       </x:c>
-      <x:c r="E97" s="5" t="str">
+      <x:c r="E99" s="5" t="str">
         <x:v>当前设备存在一种不可用认证方式</x:v>
       </x:c>
-      <x:c r="F97" s="5" t="str">
+      <x:c r="F99" s="5" t="str">
         <x:v>1. 进入工具设置页
 2. 选择当前设备不可用的认证方式
 3. 点击保存设置</x:v>
       </x:c>
-      <x:c r="G97" s="5" t="str">
+      <x:c r="G99" s="5" t="str">
         <x:v>1. 页面弹出认证方式不可用提示
 2. 用户确认前不直接保存</x:v>
       </x:c>
-      <x:c r="H97" s="5"/>
-      <x:c r="I97" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J97" s="7" t="str">
+      <x:c r="H99" s="5"/>
+      <x:c r="I99" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J99" s="7" t="str">
         <x:v>entry/src/test/tool-settings/viewmodel.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="98" s="1" customFormat="1" ht="28.5" customHeight="1">
-      <x:c r="A98" s="4" t="str">
+    <x:row r="100" s="1" customFormat="1" ht="42.75" customHeight="1">
+      <x:c r="A100" s="4" t="str">
         <x:v>SET-007</x:v>
       </x:c>
-      <x:c r="B98" s="5" t="str">
+      <x:c r="B100" s="5" t="str">
         <x:v>工具设置</x:v>
       </x:c>
-      <x:c r="C98" s="5" t="str">
+      <x:c r="C100" s="5" t="str">
         <x:v>修改密码入口</x:v>
       </x:c>
-      <x:c r="D98" s="5" t="str">
+      <x:c r="D100" s="5" t="str">
         <x:v>验证点击修改密码后拉起系统“生物识别和密码”页面</x:v>
       </x:c>
-      <x:c r="E98" s="5" t="str">
+      <x:c r="E100" s="5" t="str">
         <x:v>系统设置能力可用</x:v>
       </x:c>
-      <x:c r="F98" s="5" t="str">
+      <x:c r="F100" s="5" t="str">
         <x:v>1. 进入工具设置页
 2. 点击 `修改密码`</x:v>
       </x:c>
-      <x:c r="G98" s="5" t="str">
+      <x:c r="G100" s="5" t="str">
         <x:v>1. 成功拉起系统 `生物识别和密码` 页面
 2. 拉起失败时展示明确失败提示</x:v>
       </x:c>
-      <x:c r="H98" s="5"/>
-      <x:c r="I98" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J98" s="7" t="str">
+      <x:c r="H100" s="5"/>
+      <x:c r="I100" s="7" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J100" s="7" t="str">
         <x:v>entry/src/test/tool-settings/viewmodel.test.ets；entry/src/test/tool-settings/system-settings-service.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="99" s="1" customFormat="1" ht="28.5" customHeight="1">
-      <x:c r="A99" s="4" t="str">
+    <x:row r="101" s="1" customFormat="1" ht="28.5" customHeight="1">
+      <x:c r="A101" s="4" t="str">
         <x:v>HELP-001</x:v>
       </x:c>
-      <x:c r="B99" s="5" t="str">
+      <x:c r="B101" s="5" t="str">
         <x:v>帮助与反馈</x:v>
       </x:c>
-      <x:c r="C99" s="5" t="str">
+      <x:c r="C101" s="5" t="str">
         <x:v>页面展示</x:v>
       </x:c>
-      <x:c r="D99" s="5" t="str">
+      <x:c r="D101" s="5" t="str">
         <x:v>验证帮助与反馈页可正常打开</x:v>
       </x:c>
-      <x:c r="E99" s="5" t="str">
+      <x:c r="E101" s="5" t="str">
         <x:v>应用处于任一主页面</x:v>
       </x:c>
-      <x:c r="F99" s="5" t="str">
+      <x:c r="F101" s="5" t="str">
         <x:v>1. 打开右上角菜单
 2. 点击帮助与反馈</x:v>
       </x:c>
-      <x:c r="G99" s="5" t="str">
+      <x:c r="G101" s="5" t="str">
         <x:v>1. 成功进入帮助与反馈页
 2. 页面标题、说明正常展示</x:v>
       </x:c>
-      <x:c r="H99" s="5"/>
-      <x:c r="I99" s="7" t="str">
+      <x:c r="H101" s="5"/>
+      <x:c r="I101" s="7" t="str">
         <x:v>不补UT</x:v>
       </x:c>
-      <x:c r="J99" s="7" t="str">
+      <x:c r="J101" s="7" t="str">
         <x:v>页面打开属于页面渲染/导航场景，不进入本轮 UT 补充范围。</x:v>
       </x:c>
     </x:row>
-    <x:row r="100" s="1" customFormat="1" ht="42.75" customHeight="1">
-      <x:c r="A100" s="4" t="str">
+    <x:row r="102" s="1" customFormat="1" ht="42.75" customHeight="1">
+      <x:c r="A102" s="4" t="str">
         <x:v>HELP-002</x:v>
       </x:c>
-      <x:c r="B100" s="5" t="str">
+      <x:c r="B102" s="5" t="str">
         <x:v>帮助与反馈</x:v>
       </x:c>
-      <x:c r="C100" s="5" t="str">
+      <x:c r="C102" s="5" t="str">
         <x:v>使用指南展示</x:v>
       </x:c>
-      <x:c r="D100" s="5" t="str">
+      <x:c r="D102" s="5" t="str">
         <x:v>验证使用指南内容展示完整</x:v>
       </x:c>
-      <x:c r="E100" s="5" t="str">
+      <x:c r="E102" s="5" t="str">
         <x:v>已进入帮助与反馈页</x:v>
       </x:c>
-      <x:c r="F100" s="5" t="str">
+      <x:c r="F102" s="5" t="str">
         <x:v>1. 查看使用指南区域</x:v>
       </x:c>
-      <x:c r="G100" s="5" t="str">
+      <x:c r="G102" s="5" t="str">
         <x:v>1. 展示防火墙、外设、身份鉴别、工具设置、主题模式等指南项
 2. 文案无截断</x:v>
       </x:c>
-      <x:c r="H100" s="5"/>
-      <x:c r="I100" s="7" t="str">
+      <x:c r="H102" s="5"/>
+      <x:c r="I102" s="7" t="str">
         <x:v>不补UT</x:v>
       </x:c>
-      <x:c r="J100" s="7" t="str">
+      <x:c r="J102" s="7" t="str">
         <x:v>使用指南展示属于页面展示场景；文案结构已有基础 UT，不再补。</x:v>
       </x:c>
     </x:row>
-    <x:row r="101" s="1" customFormat="1" ht="28.5" customHeight="1">
-      <x:c r="A101" s="4" t="str">
+    <x:row r="103" s="1" customFormat="1" ht="42.75" customHeight="1">
+      <x:c r="A103" s="4" t="str">
         <x:v>HELP-003</x:v>
       </x:c>
-      <x:c r="B101" s="5" t="str">
+      <x:c r="B103" s="5" t="str">
         <x:v>帮助与反馈</x:v>
       </x:c>
-      <x:c r="C101" s="5" t="str">
+      <x:c r="C103" s="5" t="str">
         <x:v>FAQ展开收起</x:v>
       </x:c>
-      <x:c r="D101" s="5" t="str">
+      <x:c r="D103" s="5" t="str">
         <x:v>验证 FAQ 可以展开和收起</x:v>
       </x:c>
-      <x:c r="E101" s="5" t="str">
+      <x:c r="E103" s="5" t="str">
         <x:v>已进入帮助与反馈页</x:v>
       </x:c>
-      <x:c r="F101" s="5" t="str">
+      <x:c r="F103" s="5" t="str">
         <x:v>1. 点击任一 FAQ 展开按钮
 2. 再次点击收起按钮</x:v>
       </x:c>
-      <x:c r="G101" s="5" t="str">
+      <x:c r="G103" s="5" t="str">
         <x:v>1. 首次点击展示答案
 2. 再次点击隐藏答案
 3. 按钮文案在展开和收起间切换</x:v>
       </x:c>
-      <x:c r="H101" s="5"/>
-      <x:c r="I101" s="7" t="str">
-        <x:v>不补UT</x:v>
-      </x:c>
-      <x:c r="J101" s="7" t="str">
-        <x:v>FAQ 展开收起属于页面交互场景，不进入本轮 UT 补充范围。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="102" s="1" customFormat="1" ht="42.75" customHeight="1">
-      <x:c r="A102" s="4" t="str">
-        <x:v>HELP-004</x:v>
-      </x:c>
-      <x:c r="B102" s="5" t="str">
-        <x:v>帮助与反馈</x:v>
-      </x:c>
-      <x:c r="C102" s="5" t="str">
-        <x:v>联系方式展示</x:v>
-      </x:c>
-      <x:c r="D102" s="5" t="str">
-        <x:v>验证联系与反馈信息展示正确</x:v>
-      </x:c>
-      <x:c r="E102" s="5" t="str">
-        <x:v>已进入帮助与反馈页</x:v>
-      </x:c>
-      <x:c r="F102" s="5" t="str">
-        <x:v>1. 查看联系与反馈区域</x:v>
-      </x:c>
-      <x:c r="G102" s="5" t="str">
-        <x:v>1. 展示反馈邮箱
-2. 邮箱内容为 `consumer@huawei.com`</x:v>
-      </x:c>
-      <x:c r="H102" s="5"/>
-      <x:c r="I102" s="7" t="str">
-        <x:v>不补UT</x:v>
-      </x:c>
-      <x:c r="J102" s="7" t="str">
-        <x:v>联系方式展示属于页面展示场景；文案结构已有基础 UT，不再补。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="103" s="1" customFormat="1" ht="42.75" customHeight="1">
-      <x:c r="A103" s="4" t="str">
-        <x:v>NAV-001</x:v>
-      </x:c>
-      <x:c r="B103" s="5" t="str">
-        <x:v>全局导航与主题</x:v>
-      </x:c>
-      <x:c r="C103" s="5" t="str">
-        <x:v>侧边栏导航</x:v>
-      </x:c>
-      <x:c r="D103" s="5" t="str">
-        <x:v>验证侧边栏可以进入所有主模块</x:v>
-      </x:c>
-      <x:c r="E103" s="5" t="str">
-        <x:v>应用处于安全总览页</x:v>
-      </x:c>
-      <x:c r="F103" s="5" t="str">
-        <x:v>1. 依次点击侧边栏防火墙、日志、外设、身份鉴别、工具设置</x:v>
-      </x:c>
-      <x:c r="G103" s="5" t="str">
-        <x:v>1. 每次均进入对应页面
-2. 侧边栏选中态同步更新</x:v>
-      </x:c>
       <x:c r="H103" s="5"/>
       <x:c r="I103" s="7" t="str">
         <x:v>不补UT</x:v>
       </x:c>
       <x:c r="J103" s="7" t="str">
-        <x:v>导航、弹窗或菜单交互属于 UI/ohosTest 范围，不进入本轮 UT 补充范围。</x:v>
+        <x:v>FAQ 展开收起属于页面交互场景，不进入本轮 UT 补充范围。</x:v>
       </x:c>
     </x:row>
     <x:row r="104" s="1" customFormat="1" ht="42.75" customHeight="1">
       <x:c r="A104" s="4" t="str">
-        <x:v>NAV-002</x:v>
+        <x:v>HELP-004</x:v>
       </x:c>
       <x:c r="B104" s="5" t="str">
-        <x:v>全局导航与主题</x:v>
+        <x:v>帮助与反馈</x:v>
       </x:c>
       <x:c r="C104" s="5" t="str">
-        <x:v>返回按钮</x:v>
+        <x:v>联系方式展示</x:v>
       </x:c>
       <x:c r="D104" s="5" t="str">
-        <x:v>验证子页面返回按钮回到安全总览或上级页面</x:v>
+        <x:v>验证联系与反馈信息展示正确</x:v>
       </x:c>
       <x:c r="E104" s="5" t="str">
-        <x:v>已进入任一子页面</x:v>
+        <x:v>已进入帮助与反馈页</x:v>
       </x:c>
       <x:c r="F104" s="5" t="str">
-        <x:v>1. 点击页面左上角返回按钮</x:v>
+        <x:v>1. 查看联系与反馈区域</x:v>
       </x:c>
       <x:c r="G104" s="5" t="str">
-        <x:v>1. 返回到预期上级页面
-2. 页面不闪退、不空白</x:v>
+        <x:v>1. 展示反馈邮箱
+2. 邮箱内容为 `consumer@huawei.com`</x:v>
       </x:c>
       <x:c r="H104" s="5"/>
       <x:c r="I104" s="7" t="str">
         <x:v>不补UT</x:v>
       </x:c>
       <x:c r="J104" s="7" t="str">
-        <x:v>导航、弹窗或菜单交互属于 UI/ohosTest 范围，不进入本轮 UT 补充范围。</x:v>
+        <x:v>联系方式展示属于页面展示场景；文案结构已有基础 UT，不再补。</x:v>
       </x:c>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="4" t="str">
-        <x:v>NAV-003</x:v>
+        <x:v>NAV-001</x:v>
       </x:c>
       <x:c r="B105" s="5" t="str">
         <x:v>全局导航与主题</x:v>
       </x:c>
       <x:c r="C105" s="5" t="str">
-        <x:v>主题菜单</x:v>
+        <x:v>侧边栏导航</x:v>
       </x:c>
       <x:c r="D105" s="5" t="str">
-        <x:v>验证右上角主题菜单可以打开和关闭</x:v>
+        <x:v>验证侧边栏可以进入所有主模块</x:v>
       </x:c>
       <x:c r="E105" s="5" t="str">
-        <x:v>应用处于任一页面</x:v>
+        <x:v>应用处于安全总览页</x:v>
       </x:c>
       <x:c r="F105" s="5" t="str">
-        <x:v>1. 点击右上角菜单按钮
-2. 点击页面空白区域</x:v>
+        <x:v>1. 依次点击侧边栏防火墙、日志、外设、身份鉴别、工具设置</x:v>
       </x:c>
       <x:c r="G105" s="5" t="str">
-        <x:v>1. 菜单打开后展示主题、帮助、关于等入口
-2. 点击空白区域后菜单关闭</x:v>
+        <x:v>1. 每次均进入对应页面
+2. 侧边栏选中态同步更新</x:v>
       </x:c>
       <x:c r="H105" s="5"/>
       <x:c r="I105" s="7" t="str">
@@ -4560,230 +4565,293 @@
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="4" t="str">
-        <x:v>NAV-004</x:v>
+        <x:v>NAV-002</x:v>
       </x:c>
       <x:c r="B106" s="5" t="str">
         <x:v>全局导航与主题</x:v>
       </x:c>
       <x:c r="C106" s="5" t="str">
+        <x:v>返回按钮</x:v>
+      </x:c>
+      <x:c r="D106" s="5" t="str">
+        <x:v>验证子页面返回按钮回到安全总览或上级页面</x:v>
+      </x:c>
+      <x:c r="E106" s="5" t="str">
+        <x:v>已进入任一子页面</x:v>
+      </x:c>
+      <x:c r="F106" s="5" t="str">
+        <x:v>1. 点击页面左上角返回按钮</x:v>
+      </x:c>
+      <x:c r="G106" s="5" t="str">
+        <x:v>1. 返回到预期上级页面
+2. 页面不闪退、不空白</x:v>
+      </x:c>
+      <x:c r="H106" s="5"/>
+      <x:c r="I106" s="7" t="str">
+        <x:v>不补UT</x:v>
+      </x:c>
+      <x:c r="J106" s="7" t="str">
+        <x:v>导航、弹窗或菜单交互属于 UI/ohosTest 范围，不进入本轮 UT 补充范围。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" t="str">
+        <x:v>NAV-003</x:v>
+      </x:c>
+      <x:c r="B107" t="str">
+        <x:v>全局导航与主题</x:v>
+      </x:c>
+      <x:c r="C107" t="str">
+        <x:v>主题菜单</x:v>
+      </x:c>
+      <x:c r="D107" t="str">
+        <x:v>验证右上角主题菜单可以打开和关闭</x:v>
+      </x:c>
+      <x:c r="E107" t="str">
+        <x:v>应用处于任一页面</x:v>
+      </x:c>
+      <x:c r="F107" t="str">
+        <x:v>1. 点击右上角菜单按钮
+2. 点击页面空白区域</x:v>
+      </x:c>
+      <x:c r="G107" t="str">
+        <x:v>1. 菜单打开后展示主题、帮助、关于等入口
+2. 点击空白区域后菜单关闭</x:v>
+      </x:c>
+      <x:c r="H107"/>
+      <x:c r="I107" t="str">
+        <x:v>不补UT</x:v>
+      </x:c>
+      <x:c r="J107" t="str">
+        <x:v>导航、弹窗或菜单交互属于 UI/ohosTest 范围，不进入本轮 UT 补充范围。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" t="str">
+        <x:v>NAV-004</x:v>
+      </x:c>
+      <x:c r="B108" t="str">
+        <x:v>全局导航与主题</x:v>
+      </x:c>
+      <x:c r="C108" t="str">
         <x:v>深浅色切换</x:v>
       </x:c>
-      <x:c r="D106" s="5" t="str">
+      <x:c r="D108" t="str">
         <x:v>验证浅色模式切换生效</x:v>
       </x:c>
-      <x:c r="E106" s="5" t="str">
+      <x:c r="E108" t="str">
         <x:v>应用可正常打开</x:v>
       </x:c>
-      <x:c r="F106" s="5" t="str">
+      <x:c r="F108" t="str">
         <x:v>1. 打开右上角菜单
 2. 选择浅色模式</x:v>
       </x:c>
-      <x:c r="G106" s="5" t="str">
+      <x:c r="G108" t="str">
         <x:v>1. 页面切换为浅色主题
 2. 顶部窗口按钮样式同步浅色配置</x:v>
       </x:c>
-      <x:c r="H106" s="5"/>
-      <x:c r="I106" s="7" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J106" s="7" t="str">
+      <x:c r="H108"/>
+      <x:c r="I108" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J108" t="str">
         <x:v>entry/src/test/theme/theme-manager.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="107">
-      <x:c r="A107" t="str">
+    <x:row r="109">
+      <x:c r="A109" t="str">
         <x:v>NAV-005</x:v>
       </x:c>
-      <x:c r="B107" t="str">
+      <x:c r="B109" t="str">
         <x:v>全局导航与主题</x:v>
       </x:c>
-      <x:c r="C107" t="str">
+      <x:c r="C109" t="str">
         <x:v>深浅色切换</x:v>
       </x:c>
-      <x:c r="D107" t="str">
+      <x:c r="D109" t="str">
         <x:v>验证深色模式切换生效</x:v>
       </x:c>
-      <x:c r="E107" t="str">
+      <x:c r="E109" t="str">
         <x:v>应用可正常打开</x:v>
       </x:c>
-      <x:c r="F107" t="str">
+      <x:c r="F109" t="str">
         <x:v>1. 打开右上角菜单
 2. 选择深色模式</x:v>
       </x:c>
-      <x:c r="G107" t="str">
+      <x:c r="G109" t="str">
         <x:v>1. 页面切换为深色主题
 2. 页面文字、背景、图标对比度正常</x:v>
       </x:c>
-      <x:c r="H107"/>
-      <x:c r="I107" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J107" t="str">
+      <x:c r="H109"/>
+      <x:c r="I109" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J109" t="str">
         <x:v>entry/src/test/theme/theme-manager.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="108">
-      <x:c r="A108" t="str">
+    <x:row r="110">
+      <x:c r="A110" t="str">
         <x:v>NAV-006</x:v>
       </x:c>
-      <x:c r="B108" t="str">
+      <x:c r="B110" t="str">
         <x:v>全局导航与主题</x:v>
       </x:c>
-      <x:c r="C108" t="str">
+      <x:c r="C110" t="str">
         <x:v>深浅色切换</x:v>
       </x:c>
-      <x:c r="D108" t="str">
+      <x:c r="D110" t="str">
         <x:v>验证跟随系统模式保存和回显</x:v>
       </x:c>
-      <x:c r="E108" t="str">
+      <x:c r="E110" t="str">
         <x:v>系统主题可切换</x:v>
       </x:c>
-      <x:c r="F108" t="str">
+      <x:c r="F110" t="str">
         <x:v>1. 打开右上角菜单
 2. 选择跟随系统
 3. 重启应用</x:v>
       </x:c>
-      <x:c r="G108" t="str">
+      <x:c r="G110" t="str">
         <x:v>1. 应用主题跟随系统当前主题
 2. 菜单中当前选项回显正确</x:v>
       </x:c>
-      <x:c r="H108"/>
-      <x:c r="I108" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J108" t="str">
+      <x:c r="H110"/>
+      <x:c r="I110" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J110" t="str">
         <x:v>entry/src/test/theme/theme-manager.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="109">
-      <x:c r="A109" t="str">
+    <x:row r="111">
+      <x:c r="A111" t="str">
         <x:v>NAV-007</x:v>
       </x:c>
-      <x:c r="B109" t="str">
+      <x:c r="B111" t="str">
         <x:v>全局导航与主题</x:v>
       </x:c>
-      <x:c r="C109" t="str">
+      <x:c r="C111" t="str">
         <x:v>关于弹窗</x:v>
       </x:c>
-      <x:c r="D109" t="str">
+      <x:c r="D111" t="str">
         <x:v>验证关于弹窗展示应用信息</x:v>
       </x:c>
-      <x:c r="E109" t="str">
+      <x:c r="E111" t="str">
         <x:v>应用处于任一页面</x:v>
       </x:c>
-      <x:c r="F109" t="str">
+      <x:c r="F111" t="str">
         <x:v>1. 打开右上角菜单
 2. 点击关于</x:v>
       </x:c>
-      <x:c r="G109" t="str">
+      <x:c r="G111" t="str">
         <x:v>1. 弹窗展示应用名称、版本和版权信息
 2. 点击确定后弹窗关闭</x:v>
       </x:c>
-      <x:c r="H109"/>
-      <x:c r="I109" t="str">
+      <x:c r="H111"/>
+      <x:c r="I111" t="str">
         <x:v>不补UT</x:v>
       </x:c>
-      <x:c r="J109" t="str">
+      <x:c r="J111" t="str">
         <x:v>导航、弹窗或菜单交互属于 UI/ohosTest 范围，不进入本轮 UT 补充范围。</x:v>
       </x:c>
     </x:row>
-    <x:row r="110">
-      <x:c r="A110" t="str">
+    <x:row r="112">
+      <x:c r="A112" t="str">
         <x:v>SYS-005</x:v>
       </x:c>
-      <x:c r="B110" t="str">
+      <x:c r="B112" t="str">
         <x:v>系统集成基础</x:v>
       </x:c>
-      <x:c r="C110" t="str">
+      <x:c r="C112" t="str">
         <x:v>导出文件能力</x:v>
       </x:c>
-      <x:c r="D110" t="str">
+      <x:c r="D112" t="str">
         <x:v>验证通用 CSV 导出能力正常</x:v>
       </x:c>
-      <x:c r="E110" t="str">
+      <x:c r="E112" t="str">
         <x:v>日志或外设存在可导出数据</x:v>
       </x:c>
-      <x:c r="F110" t="str">
+      <x:c r="F112" t="str">
         <x:v>1. 在任一支持导出的页面点击导出
 2. 打开导出文件</x:v>
       </x:c>
-      <x:c r="G110" t="str">
+      <x:c r="G112" t="str">
         <x:v>1. 文件保存成功
 2. 文件编码和表头正确
 3. 中文内容不乱码</x:v>
       </x:c>
-      <x:c r="H110"/>
-      <x:c r="I110" t="str">
-        <x:v>已有UT覆盖</x:v>
-      </x:c>
-      <x:c r="J110" t="str">
+      <x:c r="H112"/>
+      <x:c r="I112" t="str">
+        <x:v>已有UT覆盖</x:v>
+      </x:c>
+      <x:c r="J112" t="str">
         <x:v>entry/src/test/common/csv-file-export-service.test.ets；entry/src/test/log-manage/export-service.test.ets</x:v>
       </x:c>
     </x:row>
-    <x:row r="111">
-      <x:c r="A111" t="str">
+    <x:row r="113">
+      <x:c r="A113" t="str">
         <x:v>SYS-006</x:v>
       </x:c>
-      <x:c r="B111" t="str">
+      <x:c r="B113" t="str">
         <x:v>系统集成基础</x:v>
       </x:c>
-      <x:c r="C111" t="str">
+      <x:c r="C113" t="str">
         <x:v>本地存储能力</x:v>
       </x:c>
-      <x:c r="D111" t="str">
+      <x:c r="D113" t="str">
         <x:v>验证设置类配置重启后可恢复</x:v>
       </x:c>
-      <x:c r="E111" t="str">
+      <x:c r="E113" t="str">
         <x:v>已修改工具设置或日志存储设置</x:v>
       </x:c>
-      <x:c r="F111" t="str">
+      <x:c r="F113" t="str">
         <x:v>1. 保存配置
 2. 关闭并重启应用
 3. 重新进入对应页面</x:v>
       </x:c>
-      <x:c r="G111" t="str">
+      <x:c r="G113" t="str">
         <x:v>1. 页面回显上次保存配置
 2. 无默认值覆盖已保存配置</x:v>
       </x:c>
-      <x:c r="H111"/>
-      <x:c r="I111" t="str">
+      <x:c r="H113"/>
+      <x:c r="I113" t="str">
         <x:v>不补UT</x:v>
       </x:c>
-      <x:c r="J111" t="str">
+      <x:c r="J113" t="str">
         <x:v>重启后恢复属于集成语义；存储读写已有基础 UT，不再补。</x:v>
       </x:c>
     </x:row>
-    <x:row r="112">
-      <x:c r="A112" t="str">
+    <x:row r="114">
+      <x:c r="A114" t="str">
         <x:v>SYS-007</x:v>
       </x:c>
-      <x:c r="B112" t="str">
+      <x:c r="B114" t="str">
         <x:v>系统集成基础</x:v>
       </x:c>
-      <x:c r="C112" t="str">
+      <x:c r="C114" t="str">
         <x:v>应用恢复</x:v>
       </x:c>
-      <x:c r="D112" t="str">
+      <x:c r="D114" t="str">
         <x:v>验证应用前后台切换后当前页面状态正常</x:v>
       </x:c>
-      <x:c r="E112" t="str">
+      <x:c r="E114" t="str">
         <x:v>应用已打开任一业务页面</x:v>
       </x:c>
-      <x:c r="F112" t="str">
+      <x:c r="F114" t="str">
         <x:v>1. 将应用切到后台
 2. 等待 5 秒
 3. 恢复到前台</x:v>
       </x:c>
-      <x:c r="G112" t="str">
+      <x:c r="G114" t="str">
         <x:v>1. 当前页面仍可操作
 2. 关键数据自动刷新或保持一致
 3. 无崩溃</x:v>
       </x:c>
-      <x:c r="H112"/>
-      <x:c r="I112" t="str">
+      <x:c r="H114"/>
+      <x:c r="I114" t="str">
         <x:v>不补UT</x:v>
       </x:c>
-      <x:c r="J112" t="str">
+      <x:c r="J114" t="str">
         <x:v>前后台切换属于应用生命周期集成场景，不进入本轮 UT 补充范围。</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
docs: add log import exception test baseline
</commit_message>
<xml_diff>
--- a/docs/04-测试文档/手工测试用例/测试用例基线.xlsx
+++ b/docs/04-测试文档/手工测试用例/测试用例基线.xlsx
@@ -564,7 +564,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -585,6 +585,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1057,7 +1060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J114"/>
+  <dimension ref="A1:J118"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14" defaultRowHeight="13.5"/>
   <cols>
     <col width="9.25" customWidth="1" style="1" min="1" max="1"/>
@@ -3875,1805 +3878,2009 @@
     <row r="55" ht="28.5" customHeight="1" s="1">
       <c r="A55" s="4" t="inlineStr">
         <is>
+          <t>LOG-026</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>日志管理</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>导入异常</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>验证选择非 zip 文件作为离线日志包时被拦截</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>日志管理页可正常打开</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>1. 点击添加日志
+2. 选择非 zip 格式文件</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>1. 导入流程返回非法压缩包结果
+2. 不解压、不扫描、不写入日志数据库
+3. 页面展示明确失败提示</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="n"/>
+      <c r="I55" s="8" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J55" s="8" t="inlineStr">
+        <is>
+          <t>entry/src/test/log-manage/archive-extractor.test.ets</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="28.5" customHeight="1" s="1">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>LOG-027</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>日志管理</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>导入异常</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>验证用户取消选择日志包或解压目录时导入流程取消且不入库</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>日志管理页可正常打开</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>1. 点击添加日志
+2. 在文件选择或目录选择阶段取消</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>1. 导入流程返回用户取消结果
+2. 不扫描文件、不写入日志数据库
+3. 当前日志列表状态保持不变</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="n"/>
+      <c r="I56" s="8" t="inlineStr">
+        <is>
+          <t>待补UT</t>
+        </is>
+      </c>
+      <c r="J56" s="8" t="inlineStr">
+        <is>
+          <t>待补 entry/src/test/log-manage/import-service.test.ets：覆盖 pickZip() 返回 null 与 pickDirectory() 返回 null。</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="28.5" customHeight="1" s="1">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>LOG-028</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>日志管理</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>导入异常</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>验证单个导入规则解析异常不会中断整批导入</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>存在至少一个可被导入规则处理的候选日志文件</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>1. 执行离线日志导入
+2. 某个导入规则解析候选文件时失败</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>1. 失败文件计入失败数量
+2. 其它候选文件继续处理
+3. 导入结果展示失败计数，不误报整批崩溃</t>
+        </is>
+      </c>
+      <c r="H57" s="5" t="n"/>
+      <c r="I57" s="8" t="inlineStr">
+        <is>
+          <t>待补UT</t>
+        </is>
+      </c>
+      <c r="J57" s="8" t="inlineStr">
+        <is>
+          <t>待补 entry/src/test/log-manage/import-service.test.ets：覆盖规则 parse() 抛异常时 failedEntryCount 增加且流程不中断。</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="28.5" customHeight="1" s="1">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>LOG-029</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>日志管理</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>导入异常</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>验证导入结果入库失败时返回明确失败结果</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>离线日志已成功解析出新增记录</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>1. 执行离线日志导入
+2. 入库阶段返回失败</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>1. 导入流程返回入库失败结果
+2. 不展示导入成功提示
+3. 结果中保留已解析、丢弃和失败计数</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="n"/>
+      <c r="I58" s="8" t="inlineStr">
+        <is>
+          <t>待补UT</t>
+        </is>
+      </c>
+      <c r="J58" s="8" t="inlineStr">
+        <is>
+          <t>待补 entry/src/test/log-manage/import-service.test.ets：覆盖 appendEntries() 返回失败时结果为 save_failed。</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="28.5" customHeight="1" s="1">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
           <t>PER-001</t>
         </is>
       </c>
-      <c r="B55" s="5" t="inlineStr">
+      <c r="B59" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C55" s="5" t="inlineStr">
+      <c r="C59" s="5" t="inlineStr">
         <is>
           <t>接口管控</t>
         </is>
       </c>
-      <c r="D55" s="5" t="inlineStr">
+      <c r="D59" s="5" t="inlineStr">
         <is>
           <t>验证外设管理页默认展示接口管控页签</t>
         </is>
       </c>
-      <c r="E55" s="5" t="inlineStr">
+      <c r="E59" s="5" t="inlineStr">
         <is>
           <t>应用可正常启动</t>
         </is>
       </c>
-      <c r="F55" s="5" t="inlineStr">
+      <c r="F59" s="5" t="inlineStr">
         <is>
           <t>1. 进入外设管理页</t>
         </is>
       </c>
-      <c r="G55" s="5" t="inlineStr">
+      <c r="G59" s="5" t="inlineStr">
         <is>
           <t>1. 默认展示接口管控页签
 2. USB、蓝牙、Wi-Fi 等接口项展示完整</t>
         </is>
       </c>
-      <c r="H55" s="5" t="n"/>
-      <c r="I55" s="7" t="inlineStr">
+      <c r="H59" s="5" t="n"/>
+      <c r="I59" s="7" t="inlineStr">
         <is>
           <t>不补UT</t>
         </is>
       </c>
-      <c r="J55" s="7" t="inlineStr">
+      <c r="J59" s="7" t="inlineStr">
         <is>
           <t>默认页签展示属于页面渲染场景，不进入本轮 UT 补充范围。</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="28.5" customHeight="1" s="1">
-      <c r="A56" s="4" t="inlineStr">
+    <row r="60" ht="28.5" customHeight="1" s="1">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>PER-002</t>
         </is>
       </c>
-      <c r="B56" s="5" t="inlineStr">
+      <c r="B60" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C56" s="5" t="inlineStr">
+      <c r="C60" s="5" t="inlineStr">
         <is>
           <t>USB接口策略</t>
         </is>
       </c>
-      <c r="D56" s="5" t="inlineStr">
+      <c r="D60" s="5" t="inlineStr">
         <is>
           <t>验证 USB 接口策略可从启用切换为禁用</t>
         </is>
       </c>
-      <c r="E56" s="5" t="inlineStr">
+      <c r="E60" s="5" t="inlineStr">
         <is>
           <t>应用已激活企业管理员，USB 接口当前为启用</t>
         </is>
       </c>
-      <c r="F56" s="5" t="inlineStr">
+      <c r="F60" s="5" t="inlineStr">
         <is>
           <t>1. 进入接口管控页签
 2. 将 USB 接口策略从 `启用` 改为 `禁用`</t>
         </is>
       </c>
-      <c r="G56" s="5" t="inlineStr">
+      <c r="G60" s="5" t="inlineStr">
         <is>
           <t>1. 页面显示处理中状态
 2. 操作完成后 USB 接口状态为 `禁用`</t>
         </is>
       </c>
-      <c r="H56" s="5" t="n"/>
-      <c r="I56" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J56" s="7" t="inlineStr">
+      <c r="H60" s="5" t="n"/>
+      <c r="I60" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J60" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/viewmodels/InterfaceControlViewModel.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="28.5" customHeight="1" s="1">
-      <c r="A57" s="4" t="inlineStr">
+    <row r="61" ht="42.75" customHeight="1" s="1">
+      <c r="A61" s="4" t="inlineStr">
         <is>
           <t>PER-003</t>
         </is>
       </c>
-      <c r="B57" s="5" t="inlineStr">
+      <c r="B61" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C57" s="5" t="inlineStr">
+      <c r="C61" s="5" t="inlineStr">
         <is>
           <t>USB接口策略</t>
         </is>
       </c>
-      <c r="D57" s="5" t="inlineStr">
+      <c r="D61" s="5" t="inlineStr">
         <is>
           <t>验证 USB 接口策略可从禁用切换为启用</t>
         </is>
       </c>
-      <c r="E57" s="5" t="inlineStr">
+      <c r="E61" s="5" t="inlineStr">
         <is>
           <t>应用已激活企业管理员，USB 接口当前为禁用</t>
         </is>
       </c>
-      <c r="F57" s="5" t="inlineStr">
+      <c r="F61" s="5" t="inlineStr">
         <is>
           <t>1. 进入接口管控页签
 2. 将 USB 接口策略从 `禁用` 改为 `启用`</t>
         </is>
       </c>
-      <c r="G57" s="5" t="inlineStr">
+      <c r="G61" s="5" t="inlineStr">
         <is>
           <t>1. 页面显示处理中状态
 2. 操作完成后 USB 接口状态为 `启用`</t>
         </is>
       </c>
-      <c r="H57" s="5" t="n"/>
-      <c r="I57" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J57" s="7" t="inlineStr">
+      <c r="H61" s="5" t="n"/>
+      <c r="I61" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J61" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/viewmodels/InterfaceControlViewModel.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="28.5" customHeight="1" s="1">
-      <c r="A58" s="4" t="inlineStr">
+    <row r="62" ht="28.5" customHeight="1" s="1">
+      <c r="A62" s="4" t="inlineStr">
         <is>
           <t>PER-004</t>
         </is>
       </c>
-      <c r="B58" s="5" t="inlineStr">
+      <c r="B62" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C58" s="5" t="inlineStr">
+      <c r="C62" s="5" t="inlineStr">
         <is>
           <t>USB存储策略</t>
         </is>
       </c>
-      <c r="D58" s="5" t="inlineStr">
+      <c r="D62" s="5" t="inlineStr">
         <is>
           <t>验证 USB 存储策略可从读写切换为只读</t>
         </is>
       </c>
-      <c r="E58" s="5" t="inlineStr">
+      <c r="E62" s="5" t="inlineStr">
         <is>
           <t>应用已激活企业管理员，USB 存储当前策略为 `读写`</t>
         </is>
       </c>
-      <c r="F58" s="5" t="inlineStr">
+      <c r="F62" s="5" t="inlineStr">
         <is>
           <t>1. 进入接口管控页签
 2. 将 USB 存储策略从 `读写` 改为 `只读`</t>
         </is>
       </c>
-      <c r="G58" s="5" t="inlineStr">
+      <c r="G62" s="5" t="inlineStr">
         <is>
           <t>1. 页面提示设置成功或状态更新
 2. USB 存储策略显示为 `只读`</t>
         </is>
       </c>
-      <c r="H58" s="5" t="n"/>
-      <c r="I58" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J58" s="7" t="inlineStr">
+      <c r="H62" s="5" t="n"/>
+      <c r="I62" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J62" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/viewmodels/InterfaceControlViewModel.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="28.5" customHeight="1" s="1">
-      <c r="A59" s="4" t="inlineStr">
+    <row r="63" ht="42" customHeight="1" s="1">
+      <c r="A63" s="4" t="inlineStr">
         <is>
           <t>PER-005</t>
         </is>
       </c>
-      <c r="B59" s="5" t="inlineStr">
+      <c r="B63" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C59" s="5" t="inlineStr">
+      <c r="C63" s="5" t="inlineStr">
         <is>
           <t>USB存储策略</t>
         </is>
       </c>
-      <c r="D59" s="5" t="inlineStr">
+      <c r="D63" s="5" t="inlineStr">
         <is>
           <t>验证 USB 存储策略可从读写切换为禁止访问</t>
         </is>
       </c>
-      <c r="E59" s="5" t="inlineStr">
+      <c r="E63" s="5" t="inlineStr">
         <is>
           <t>应用已激活企业管理员，USB 存储当前策略为 `读写`</t>
         </is>
       </c>
-      <c r="F59" s="5" t="inlineStr">
+      <c r="F63" s="5" t="inlineStr">
         <is>
           <t>1. 进入接口管控页签
 2. 将 USB 存储策略从 `读写` 改为 `禁止访问`</t>
         </is>
       </c>
-      <c r="G59" s="5" t="inlineStr">
+      <c r="G63" s="5" t="inlineStr">
         <is>
           <t>1. 页面提示设置成功或状态更新
 2. USB 存储策略显示为 `禁止访问`</t>
         </is>
       </c>
-      <c r="H59" s="5" t="n"/>
-      <c r="I59" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J59" s="7" t="inlineStr">
+      <c r="H63" s="5" t="n"/>
+      <c r="I63" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J63" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/viewmodels/InterfaceControlViewModel.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="28.5" customHeight="1" s="1">
-      <c r="A60" s="4" t="inlineStr">
+    <row r="64" ht="28.5" customHeight="1" s="1">
+      <c r="A64" s="4" t="inlineStr">
         <is>
           <t>PER-006</t>
         </is>
       </c>
-      <c r="B60" s="5" t="inlineStr">
+      <c r="B64" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C60" s="5" t="inlineStr">
+      <c r="C64" s="5" t="inlineStr">
         <is>
           <t>策略冲突处理</t>
         </is>
       </c>
-      <c r="D60" s="5" t="inlineStr">
+      <c r="D64" s="5" t="inlineStr">
         <is>
           <t>验证 USB 接口禁用时切换 USB 存储策略提示冲突</t>
         </is>
       </c>
-      <c r="E60" s="5" t="inlineStr">
+      <c r="E64" s="5" t="inlineStr">
         <is>
           <t>USB 接口当前为禁用状态</t>
         </is>
       </c>
-      <c r="F60" s="5" t="inlineStr">
+      <c r="F64" s="5" t="inlineStr">
         <is>
           <t>1. 进入接口管控页签
 2. 尝试修改 USB 存储策略</t>
         </is>
       </c>
-      <c r="G60" s="5" t="inlineStr">
+      <c r="G64" s="5" t="inlineStr">
         <is>
           <t>1. 页面提示 USB 接口处于更高层禁用或冲突状态
 2. 存储策略不被错误更新</t>
         </is>
       </c>
-      <c r="H60" s="5" t="n"/>
-      <c r="I60" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J60" s="7" t="inlineStr">
+      <c r="H64" s="5" t="n"/>
+      <c r="I64" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J64" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/viewmodels/InterfaceControlViewModel.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="42.75" customHeight="1" s="1">
-      <c r="A61" s="4" t="inlineStr">
+    <row r="65" ht="28.5" customHeight="1" s="1">
+      <c r="A65" s="4" t="inlineStr">
         <is>
           <t>PER-007</t>
         </is>
       </c>
-      <c r="B61" s="5" t="inlineStr">
+      <c r="B65" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C61" s="5" t="inlineStr">
+      <c r="C65" s="5" t="inlineStr">
         <is>
           <t>蓝牙策略</t>
         </is>
       </c>
-      <c r="D61" s="5" t="inlineStr">
+      <c r="D65" s="5" t="inlineStr">
         <is>
           <t>验证蓝牙接口策略可从启用切换为禁用</t>
         </is>
       </c>
-      <c r="E61" s="5" t="inlineStr">
+      <c r="E65" s="5" t="inlineStr">
         <is>
           <t>应用已激活企业管理员，蓝牙接口当前为启用</t>
         </is>
       </c>
-      <c r="F61" s="5" t="inlineStr">
+      <c r="F65" s="5" t="inlineStr">
         <is>
           <t>1. 进入接口管控页签
 2. 将蓝牙策略从 `启用` 改为 `禁用`</t>
         </is>
       </c>
-      <c r="G61" s="5" t="inlineStr">
+      <c r="G65" s="5" t="inlineStr">
         <is>
           <t>1. 页面提示设置成功或状态更新
 2. 蓝牙策略显示为 `禁用`</t>
         </is>
       </c>
-      <c r="H61" s="5" t="n"/>
-      <c r="I61" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J61" s="7" t="inlineStr">
+      <c r="H65" s="5" t="n"/>
+      <c r="I65" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J65" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/viewmodels/InterfaceControlViewModel.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="28.5" customHeight="1" s="1">
-      <c r="A62" s="4" t="inlineStr">
+    <row r="66" ht="28.5" customHeight="1" s="1">
+      <c r="A66" s="4" t="inlineStr">
         <is>
           <t>PER-008</t>
         </is>
       </c>
-      <c r="B62" s="5" t="inlineStr">
+      <c r="B66" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C62" s="5" t="inlineStr">
+      <c r="C66" s="5" t="inlineStr">
         <is>
           <t>Wi-Fi策略</t>
         </is>
       </c>
-      <c r="D62" s="5" t="inlineStr">
+      <c r="D66" s="5" t="inlineStr">
         <is>
           <t>验证 Wi-Fi 接口策略可从启用切换为禁用</t>
         </is>
       </c>
-      <c r="E62" s="5" t="inlineStr">
+      <c r="E66" s="5" t="inlineStr">
         <is>
           <t>应用已激活企业管理员，Wi-Fi 接口当前为启用</t>
         </is>
       </c>
-      <c r="F62" s="5" t="inlineStr">
+      <c r="F66" s="5" t="inlineStr">
         <is>
           <t>1. 进入接口管控页签
 2. 将 Wi-Fi 策略从 `启用` 改为 `禁用`</t>
         </is>
       </c>
-      <c r="G62" s="5" t="inlineStr">
+      <c r="G66" s="5" t="inlineStr">
         <is>
           <t>1. 页面提示设置成功或状态更新
 2. Wi-Fi 策略显示为 `禁用`</t>
         </is>
       </c>
-      <c r="H62" s="5" t="n"/>
-      <c r="I62" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J62" s="7" t="inlineStr">
+      <c r="H66" s="5" t="n"/>
+      <c r="I66" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J66" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/viewmodels/InterfaceControlViewModel.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="42" customHeight="1" s="1">
-      <c r="A63" s="4" t="inlineStr">
+    <row r="67" ht="28.5" customHeight="1" s="1">
+      <c r="A67" s="4" t="inlineStr">
         <is>
           <t>PER-009</t>
         </is>
       </c>
-      <c r="B63" s="5" t="inlineStr">
+      <c r="B67" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C63" s="5" t="inlineStr">
+      <c r="C67" s="5" t="inlineStr">
         <is>
           <t>设备连接记录</t>
         </is>
       </c>
-      <c r="D63" s="5" t="inlineStr">
+      <c r="D67" s="5" t="inlineStr">
         <is>
           <t>验证 USB 设备接入后生成连接记录</t>
         </is>
       </c>
-      <c r="E63" s="5" t="inlineStr">
+      <c r="E67" s="5" t="inlineStr">
         <is>
           <t>应用已激活企业管理员，准备一个 USB 设备</t>
         </is>
       </c>
-      <c r="F63" s="5" t="inlineStr">
+      <c r="F67" s="5" t="inlineStr">
         <is>
           <t>1. 进入外设管理页
 2. 插入 USB 设备
 3. 切换到设备连接记录页签</t>
         </is>
       </c>
-      <c r="G63" s="5" t="inlineStr">
+      <c r="G67" s="5" t="inlineStr">
         <is>
           <t>1. 列表出现该 USB 设备连接记录
 2. 展示设备名称、设备类型、连接时间和策略结论</t>
         </is>
       </c>
-      <c r="H63" s="5" t="n"/>
-      <c r="I63" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J63" s="7" t="inlineStr">
+      <c r="H67" s="5" t="n"/>
+      <c r="I67" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J67" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/peripheral/connection-record-usb-consumer.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="28.5" customHeight="1" s="1">
-      <c r="A64" s="4" t="inlineStr">
+    <row r="68" ht="28.5" customHeight="1" s="1">
+      <c r="A68" s="4" t="inlineStr">
         <is>
           <t>PER-010</t>
         </is>
       </c>
-      <c r="B64" s="5" t="inlineStr">
+      <c r="B68" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C64" s="5" t="inlineStr">
+      <c r="C68" s="5" t="inlineStr">
         <is>
           <t>设备连接记录</t>
         </is>
       </c>
-      <c r="D64" s="5" t="inlineStr">
+      <c r="D68" s="5" t="inlineStr">
         <is>
           <t>验证 USB 设备断开后生成断开记录</t>
         </is>
       </c>
-      <c r="E64" s="5" t="inlineStr">
+      <c r="E68" s="5" t="inlineStr">
         <is>
           <t>已存在 USB 设备连接记录</t>
         </is>
       </c>
-      <c r="F64" s="5" t="inlineStr">
+      <c r="F68" s="5" t="inlineStr">
         <is>
           <t>1. 拔出 USB 设备
 2. 查看设备连接记录页签</t>
         </is>
       </c>
-      <c r="G64" s="5" t="inlineStr">
+      <c r="G68" s="5" t="inlineStr">
         <is>
           <t>1. 列表出现断开事件或最近记录更新
 2. 断开前生效策略展示正确</t>
         </is>
       </c>
-      <c r="H64" s="5" t="n"/>
-      <c r="I64" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J64" s="7" t="inlineStr">
+      <c r="H68" s="5" t="n"/>
+      <c r="I68" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J68" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/peripheral/connection-record-usb-consumer.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="28.5" customHeight="1" s="1">
-      <c r="A65" s="4" t="inlineStr">
+    <row r="69" ht="42.75" customHeight="1" s="1">
+      <c r="A69" s="4" t="inlineStr">
         <is>
           <t>PER-011</t>
         </is>
       </c>
-      <c r="B65" s="5" t="inlineStr">
+      <c r="B69" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C65" s="5" t="inlineStr">
+      <c r="C69" s="5" t="inlineStr">
         <is>
           <t>设备详情</t>
         </is>
       </c>
-      <c r="D65" s="5" t="inlineStr">
+      <c r="D69" s="5" t="inlineStr">
         <is>
           <t>验证点击设备记录后展示设备详情</t>
         </is>
       </c>
-      <c r="E65" s="5" t="inlineStr">
+      <c r="E69" s="5" t="inlineStr">
         <is>
           <t>设备连接记录列表至少有一条记录</t>
         </is>
       </c>
-      <c r="F65" s="5" t="inlineStr">
+      <c r="F69" s="5" t="inlineStr">
         <is>
           <t>1. 进入设备连接记录页签
 2. 点击一条设备记录</t>
         </is>
       </c>
-      <c r="G65" s="5" t="inlineStr">
+      <c r="G69" s="5" t="inlineStr">
         <is>
           <t>1. 弹出设备详情
 2. 展示设备标识、最近时间、连接事件、策略结论等字段</t>
         </is>
       </c>
-      <c r="H65" s="5" t="n"/>
-      <c r="I65" s="7" t="inlineStr">
+      <c r="H69" s="5" t="n"/>
+      <c r="I69" s="7" t="inlineStr">
         <is>
           <t>不补UT</t>
         </is>
       </c>
-      <c r="J65" s="7" t="inlineStr">
+      <c r="J69" s="7" t="inlineStr">
         <is>
           <t>设备详情展示属于 UI 侧场景，不进入本轮 UT 补充范围。</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="28.5" customHeight="1" s="1">
-      <c r="A66" s="4" t="inlineStr">
+    <row r="70" ht="28.5" customHeight="1" s="1">
+      <c r="A70" s="4" t="inlineStr">
         <is>
           <t>PER-012</t>
         </is>
       </c>
-      <c r="B66" s="5" t="inlineStr">
+      <c r="B70" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C66" s="5" t="inlineStr">
+      <c r="C70" s="5" t="inlineStr">
         <is>
           <t>黑白名单策略</t>
         </is>
       </c>
-      <c r="D66" s="5" t="inlineStr">
+      <c r="D70" s="5" t="inlineStr">
         <is>
           <t>验证黑白名单页签展示可管理设备</t>
         </is>
       </c>
-      <c r="E66" s="5" t="inlineStr">
+      <c r="E70" s="5" t="inlineStr">
         <is>
           <t>设备连接记录中已有可识别设备</t>
         </is>
       </c>
-      <c r="F66" s="5" t="inlineStr">
+      <c r="F70" s="5" t="inlineStr">
         <is>
           <t>1. 进入外设管理页
 2. 切换到黑白名单页签</t>
         </is>
       </c>
-      <c r="G66" s="5" t="inlineStr">
+      <c r="G70" s="5" t="inlineStr">
         <is>
           <t>1. 列表展示设备名称、设备类型、设备标识和当前策略
 2. 无设备时展示空状态</t>
         </is>
       </c>
-      <c r="H66" s="5" t="n"/>
-      <c r="I66" s="7" t="inlineStr">
+      <c r="H70" s="5" t="n"/>
+      <c r="I70" s="7" t="inlineStr">
         <is>
           <t>不补UT</t>
         </is>
       </c>
-      <c r="J66" s="7" t="inlineStr">
+      <c r="J70" s="7" t="inlineStr">
         <is>
           <t>黑白名单页签展示属于页面渲染场景，不进入本轮 UT 补充范围。</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="28.5" customHeight="1" s="1">
-      <c r="A67" s="4" t="inlineStr">
+    <row r="71" ht="42.75" customHeight="1" s="1">
+      <c r="A71" s="4" t="inlineStr">
         <is>
           <t>PER-013</t>
         </is>
       </c>
-      <c r="B67" s="5" t="inlineStr">
+      <c r="B71" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C67" s="5" t="inlineStr">
+      <c r="C71" s="5" t="inlineStr">
         <is>
           <t>单设备策略切换</t>
         </is>
       </c>
-      <c r="D67" s="5" t="inlineStr">
+      <c r="D71" s="5" t="inlineStr">
         <is>
           <t>验证单设备策略可从允许接入切换为禁止接入</t>
         </is>
       </c>
-      <c r="E67" s="5" t="inlineStr">
+      <c r="E71" s="5" t="inlineStr">
         <is>
           <t>黑白名单中存在可管理设备，当前策略为 `允许接入`</t>
         </is>
       </c>
-      <c r="F67" s="5" t="inlineStr">
+      <c r="F71" s="5" t="inlineStr">
         <is>
           <t>1. 进入黑白名单页签
 2. 将目标设备策略从 `允许接入` 改为 `禁止接入`</t>
         </is>
       </c>
-      <c r="G67" s="5" t="inlineStr">
+      <c r="G71" s="5" t="inlineStr">
         <is>
           <t>1. 页面提示策略修改成功或状态更新
 2. 目标设备当前策略为 `禁止接入`</t>
         </is>
       </c>
-      <c r="H67" s="5" t="n"/>
-      <c r="I67" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J67" s="7" t="inlineStr">
+      <c r="H71" s="5" t="n"/>
+      <c r="I71" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J71" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/viewmodels/PeripheralPolicyViewModel.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="28.5" customHeight="1" s="1">
-      <c r="A68" s="4" t="inlineStr">
+    <row r="72" ht="42.75" customHeight="1" s="1">
+      <c r="A72" s="4" t="inlineStr">
         <is>
           <t>PER-014</t>
         </is>
       </c>
-      <c r="B68" s="5" t="inlineStr">
+      <c r="B72" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C68" s="5" t="inlineStr">
+      <c r="C72" s="5" t="inlineStr">
         <is>
           <t>单设备策略切换</t>
         </is>
       </c>
-      <c r="D68" s="5" t="inlineStr">
+      <c r="D72" s="5" t="inlineStr">
         <is>
           <t>验证单设备策略可从禁止接入切换为允许接入</t>
         </is>
       </c>
-      <c r="E68" s="5" t="inlineStr">
+      <c r="E72" s="5" t="inlineStr">
         <is>
           <t>黑白名单中存在可管理设备，当前策略为 `禁止接入`</t>
         </is>
       </c>
-      <c r="F68" s="5" t="inlineStr">
+      <c r="F72" s="5" t="inlineStr">
         <is>
           <t>1. 进入黑白名单页签
 2. 将目标设备策略从 `禁止接入` 改为 `允许接入`</t>
         </is>
       </c>
-      <c r="G68" s="5" t="inlineStr">
+      <c r="G72" s="5" t="inlineStr">
         <is>
           <t>1. 页面提示策略修改成功或状态更新
 2. 目标设备当前策略为 `允许接入`</t>
         </is>
       </c>
-      <c r="H68" s="5" t="n"/>
-      <c r="I68" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J68" s="7" t="inlineStr">
+      <c r="H72" s="5" t="n"/>
+      <c r="I72" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J72" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/viewmodels/PeripheralPolicyViewModel.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="42.75" customHeight="1" s="1">
-      <c r="A69" s="4" t="inlineStr">
+    <row r="73" ht="28.5" customHeight="1" s="1">
+      <c r="A73" s="4" t="inlineStr">
         <is>
           <t>PER-015</t>
         </is>
       </c>
-      <c r="B69" s="5" t="inlineStr">
+      <c r="B73" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C69" s="5" t="inlineStr">
+      <c r="C73" s="5" t="inlineStr">
         <is>
           <t>策略冲突处理</t>
         </is>
       </c>
-      <c r="D69" s="5" t="inlineStr">
+      <c r="D73" s="5" t="inlineStr">
         <is>
           <t>验证 USB 接口禁用时单设备策略切换提示冲突</t>
         </is>
       </c>
-      <c r="E69" s="5" t="inlineStr">
+      <c r="E73" s="5" t="inlineStr">
         <is>
           <t>USB 接口当前禁用，黑白名单中存在 USB 设备</t>
         </is>
       </c>
-      <c r="F69" s="5" t="inlineStr">
+      <c r="F73" s="5" t="inlineStr">
         <is>
           <t>1. 进入黑白名单页签
 2. 修改 USB 设备策略</t>
         </is>
       </c>
-      <c r="G69" s="5" t="inlineStr">
+      <c r="G73" s="5" t="inlineStr">
         <is>
           <t>1. 页面提示 USB 接口更高层禁用或冲突
 2. 单设备策略不被错误下发</t>
         </is>
       </c>
-      <c r="H69" s="5" t="n"/>
-      <c r="I69" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J69" s="7" t="inlineStr">
+      <c r="H73" s="5" t="n"/>
+      <c r="I73" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J73" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/viewmodels/PeripheralPolicyViewModel.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="70" ht="28.5" customHeight="1" s="1">
-      <c r="A70" s="4" t="inlineStr">
+    <row r="74" ht="28.5" customHeight="1" s="1">
+      <c r="A74" s="4" t="inlineStr">
         <is>
           <t>PER-016</t>
         </is>
       </c>
-      <c r="B70" s="5" t="inlineStr">
+      <c r="B74" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C70" s="5" t="inlineStr">
+      <c r="C74" s="5" t="inlineStr">
         <is>
           <t>记录导出</t>
         </is>
       </c>
-      <c r="D70" s="5" t="inlineStr">
+      <c r="D74" s="5" t="inlineStr">
         <is>
           <t>验证设备连接记录可以导出</t>
         </is>
       </c>
-      <c r="E70" s="5" t="inlineStr">
+      <c r="E74" s="5" t="inlineStr">
         <is>
           <t>设备连接记录至少存在一条记录</t>
         </is>
       </c>
-      <c r="F70" s="5" t="inlineStr">
+      <c r="F74" s="5" t="inlineStr">
         <is>
           <t>1. 进入设备连接记录页签
 2. 点击导出记录</t>
         </is>
       </c>
-      <c r="G70" s="5" t="inlineStr">
+      <c r="G74" s="5" t="inlineStr">
         <is>
           <t>1. 页面提示导出成功
 2. 导出文件包含连接记录表头和数据</t>
         </is>
       </c>
-      <c r="H70" s="5" t="n"/>
-      <c r="I70" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J70" s="7" t="inlineStr">
+      <c r="H74" s="5" t="n"/>
+      <c r="I74" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J74" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/viewmodels/PeripheralRecordViewModel.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="42.75" customHeight="1" s="1">
-      <c r="A71" s="4" t="inlineStr">
+    <row r="75" ht="28.5" customHeight="1" s="1">
+      <c r="A75" s="4" t="inlineStr">
         <is>
           <t>PER-017</t>
         </is>
       </c>
-      <c r="B71" s="5" t="inlineStr">
+      <c r="B75" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C71" s="5" t="inlineStr">
+      <c r="C75" s="5" t="inlineStr">
         <is>
           <t>记录清理</t>
         </is>
       </c>
-      <c r="D71" s="5" t="inlineStr">
+      <c r="D75" s="5" t="inlineStr">
         <is>
           <t>验证设备连接记录可以清理</t>
         </is>
       </c>
-      <c r="E71" s="5" t="inlineStr">
+      <c r="E75" s="5" t="inlineStr">
         <is>
           <t>设备连接记录至少存在一条记录</t>
         </is>
       </c>
-      <c r="F71" s="5" t="inlineStr">
+      <c r="F75" s="5" t="inlineStr">
         <is>
           <t>1. 进入设备连接记录页签
 2. 点击清理记录
 3. 在确认弹窗中确认</t>
         </is>
       </c>
-      <c r="G71" s="5" t="inlineStr">
+      <c r="G75" s="5" t="inlineStr">
         <is>
           <t>1. 页面提示记录已清理
 2. 列表展示空状态</t>
         </is>
       </c>
-      <c r="H71" s="5" t="n"/>
-      <c r="I71" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J71" s="7" t="inlineStr">
+      <c r="H75" s="5" t="n"/>
+      <c r="I75" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J75" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/viewmodels/PeripheralViewModel.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="42.75" customHeight="1" s="1">
-      <c r="A72" s="4" t="inlineStr">
+    <row r="76" ht="28.5" customHeight="1" s="1">
+      <c r="A76" s="4" t="inlineStr">
         <is>
           <t>PER-018</t>
         </is>
       </c>
-      <c r="B72" s="5" t="inlineStr">
+      <c r="B76" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C72" s="5" t="inlineStr">
+      <c r="C76" s="5" t="inlineStr">
         <is>
           <t>策略导出</t>
         </is>
       </c>
-      <c r="D72" s="5" t="inlineStr">
+      <c r="D76" s="5" t="inlineStr">
         <is>
           <t>验证黑白名单策略可以导出</t>
         </is>
       </c>
-      <c r="E72" s="5" t="inlineStr">
+      <c r="E76" s="5" t="inlineStr">
         <is>
           <t>黑白名单中至少存在一条策略记录</t>
         </is>
       </c>
-      <c r="F72" s="5" t="inlineStr">
+      <c r="F76" s="5" t="inlineStr">
         <is>
           <t>1. 进入黑白名单页签
 2. 点击导出名单</t>
         </is>
       </c>
-      <c r="G72" s="5" t="inlineStr">
+      <c r="G76" s="5" t="inlineStr">
         <is>
           <t>1. 页面提示导出成功
 2. 导出文件包含策略表头和数据</t>
         </is>
       </c>
-      <c r="H72" s="5" t="n"/>
-      <c r="I72" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J72" s="7" t="inlineStr">
+      <c r="H76" s="5" t="n"/>
+      <c r="I76" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J76" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/viewmodels/PeripheralPolicyViewModel.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="73" ht="28.5" customHeight="1" s="1">
-      <c r="A73" s="4" t="inlineStr">
+    <row r="77" ht="42.75" customHeight="1" s="1">
+      <c r="A77" s="4" t="inlineStr">
         <is>
           <t>PER-019</t>
         </is>
       </c>
-      <c r="B73" s="5" t="inlineStr">
+      <c r="B77" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C73" s="5" t="inlineStr">
+      <c r="C77" s="5" t="inlineStr">
         <is>
           <t>策略还原</t>
         </is>
       </c>
-      <c r="D73" s="5" t="inlineStr">
+      <c r="D77" s="5" t="inlineStr">
         <is>
           <t>验证黑白名单策略还原后列表状态同步恢复默认值</t>
         </is>
       </c>
-      <c r="E73" s="5" t="inlineStr">
+      <c r="E77" s="5" t="inlineStr">
         <is>
           <t>黑白名单中至少存在一条禁止接入或非默认策略记录</t>
         </is>
       </c>
-      <c r="F73" s="5" t="inlineStr">
+      <c r="F77" s="5" t="inlineStr">
         <is>
           <t>1. 进入黑白名单页签
 2. 点击还原策略
 3. 在确认弹窗中确认</t>
         </is>
       </c>
-      <c r="G73" s="5" t="inlineStr">
+      <c r="G77" s="5" t="inlineStr">
         <is>
           <t>1. 页面提示黑白名单已还原
 2. 已记录设备恢复默认允许接入
 3. 列表中的当前策略和下拉选项同步回到默认状态</t>
         </is>
       </c>
-      <c r="H73" s="5" t="n"/>
-      <c r="I73" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J73" s="7" t="inlineStr">
+      <c r="H77" s="5" t="n"/>
+      <c r="I77" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J77" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/viewmodels/PeripheralPolicyViewModel.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="74" ht="28.5" customHeight="1" s="1">
-      <c r="A74" s="4" t="inlineStr">
+    <row r="78" ht="42.75" customHeight="1" s="1">
+      <c r="A78" s="4" t="inlineStr">
         <is>
           <t>PER-020</t>
         </is>
       </c>
-      <c r="B74" s="5" t="inlineStr">
+      <c r="B78" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C74" s="5" t="inlineStr">
+      <c r="C78" s="5" t="inlineStr">
         <is>
           <t>设备连接记录</t>
         </is>
       </c>
-      <c r="D74" s="5" t="inlineStr">
+      <c r="D78" s="5" t="inlineStr">
         <is>
           <t>验证蓝牙设备连接后生成连接记录</t>
         </is>
       </c>
-      <c r="E74" s="5" t="inlineStr">
+      <c r="E78" s="5" t="inlineStr">
         <is>
           <t>设备支持蓝牙运行期事件，准备一台可连接的蓝牙设备</t>
         </is>
       </c>
-      <c r="F74" s="5" t="inlineStr">
+      <c r="F78" s="5" t="inlineStr">
         <is>
           <t>1. 进入外设管理页
 2. 连接目标蓝牙设备
 3. 切换到设备连接记录页签</t>
         </is>
       </c>
-      <c r="G74" s="5" t="inlineStr">
+      <c r="G78" s="5" t="inlineStr">
         <is>
           <t>1. 列表新增该蓝牙设备连接记录
 2. 设备类型显示为蓝牙设备
 3. 记录展示连接时间和策略结论</t>
         </is>
       </c>
-      <c r="H74" s="5" t="n"/>
-      <c r="I74" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J74" s="7" t="inlineStr">
+      <c r="H78" s="5" t="n"/>
+      <c r="I78" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J78" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/peripheral/connection-record-bluetooth-acl-consumer.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="28.5" customHeight="1" s="1">
-      <c r="A75" s="4" t="inlineStr">
+    <row r="79" ht="42.75" customHeight="1" s="1">
+      <c r="A79" s="4" t="inlineStr">
         <is>
           <t>PER-021</t>
         </is>
       </c>
-      <c r="B75" s="5" t="inlineStr">
+      <c r="B79" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C75" s="5" t="inlineStr">
+      <c r="C79" s="5" t="inlineStr">
         <is>
           <t>设备连接记录</t>
         </is>
       </c>
-      <c r="D75" s="5" t="inlineStr">
+      <c r="D79" s="5" t="inlineStr">
         <is>
           <t>验证蓝牙设备断开后生成断开记录</t>
         </is>
       </c>
-      <c r="E75" s="5" t="inlineStr">
+      <c r="E79" s="5" t="inlineStr">
         <is>
           <t>目标蓝牙设备已连接并已生成连接记录</t>
         </is>
       </c>
-      <c r="F75" s="5" t="inlineStr">
+      <c r="F79" s="5" t="inlineStr">
         <is>
           <t>1. 断开目标蓝牙设备
 2. 查看设备连接记录页签</t>
         </is>
       </c>
-      <c r="G75" s="5" t="inlineStr">
+      <c r="G79" s="5" t="inlineStr">
         <is>
           <t>1. 列表新增蓝牙设备断开记录或最近记录状态更新
 2. 断开记录展示断开前生效策略</t>
         </is>
       </c>
-      <c r="H75" s="5" t="n"/>
-      <c r="I75" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J75" s="7" t="inlineStr">
+      <c r="H79" s="5" t="n"/>
+      <c r="I79" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J79" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/peripheral/connection-record-bluetooth-acl-consumer.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="28.5" customHeight="1" s="1">
-      <c r="A76" s="4" t="inlineStr">
+    <row r="80" ht="42.75" customHeight="1" s="1">
+      <c r="A80" s="4" t="inlineStr">
         <is>
           <t>PER-022</t>
         </is>
       </c>
-      <c r="B76" s="5" t="inlineStr">
+      <c r="B80" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C76" s="5" t="inlineStr">
+      <c r="C80" s="5" t="inlineStr">
         <is>
           <t>设备详情</t>
         </is>
       </c>
-      <c r="D76" s="5" t="inlineStr">
+      <c r="D80" s="5" t="inlineStr">
         <is>
           <t>验证点击蓝牙设备记录后展示设备详情</t>
         </is>
       </c>
-      <c r="E76" s="5" t="inlineStr">
+      <c r="E80" s="5" t="inlineStr">
         <is>
           <t>设备连接记录中至少存在一条蓝牙设备记录</t>
         </is>
       </c>
-      <c r="F76" s="5" t="inlineStr">
+      <c r="F80" s="5" t="inlineStr">
         <is>
           <t>1. 进入设备连接记录页签
 2. 点击蓝牙设备记录</t>
         </is>
       </c>
-      <c r="G76" s="5" t="inlineStr">
+      <c r="G80" s="5" t="inlineStr">
         <is>
           <t>1. 弹出设备详情弹窗
 2. 展示设备标识、连接事件、事件来源和策略结论</t>
         </is>
       </c>
-      <c r="H76" s="5" t="n"/>
-      <c r="I76" s="7" t="inlineStr">
+      <c r="H80" s="5" t="n"/>
+      <c r="I80" s="7" t="inlineStr">
         <is>
           <t>不补UT</t>
         </is>
       </c>
-      <c r="J76" s="7" t="inlineStr">
+      <c r="J80" s="7" t="inlineStr">
         <is>
           <t>蓝牙详情展示属于 UI 侧场景；蓝牙记录建模已有 UT，不再补展示 UT。</t>
         </is>
       </c>
     </row>
-    <row r="77" ht="42.75" customHeight="1" s="1">
-      <c r="A77" s="4" t="inlineStr">
+    <row r="81" ht="42.75" customHeight="1" s="1">
+      <c r="A81" s="4" t="inlineStr">
         <is>
           <t>PER-023</t>
         </is>
       </c>
-      <c r="B77" s="5" t="inlineStr">
+      <c r="B81" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C77" s="5" t="inlineStr">
+      <c r="C81" s="5" t="inlineStr">
         <is>
           <t>单设备策略切换</t>
         </is>
       </c>
-      <c r="D77" s="5" t="inlineStr">
+      <c r="D81" s="5" t="inlineStr">
         <is>
           <t>验证蓝牙设备可切换为禁止接入策略</t>
         </is>
       </c>
-      <c r="E77" s="5" t="inlineStr">
+      <c r="E81" s="5" t="inlineStr">
         <is>
           <t>黑白名单中已出现目标蓝牙设备，应用已激活企业管理员</t>
         </is>
       </c>
-      <c r="F77" s="5" t="inlineStr">
+      <c r="F81" s="5" t="inlineStr">
         <is>
           <t>1. 进入黑白名单页签
 2. 将目标蓝牙设备策略切换为禁止接入</t>
         </is>
       </c>
-      <c r="G77" s="5" t="inlineStr">
+      <c r="G81" s="5" t="inlineStr">
         <is>
           <t>1. 页面提示策略修改成功或状态更新
 2. 目标蓝牙设备当前策略显示为禁止接入</t>
         </is>
       </c>
-      <c r="H77" s="5" t="n"/>
-      <c r="I77" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J77" s="7" t="inlineStr">
+      <c r="H81" s="5" t="n"/>
+      <c r="I81" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J81" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/viewmodels/PeripheralPolicyViewModel.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="78" ht="42.75" customHeight="1" s="1">
-      <c r="A78" s="4" t="inlineStr">
+    <row r="82" ht="57" customHeight="1" s="1">
+      <c r="A82" s="4" t="inlineStr">
         <is>
           <t>PER-024</t>
         </is>
       </c>
-      <c r="B78" s="5" t="inlineStr">
+      <c r="B82" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C78" s="5" t="inlineStr">
+      <c r="C82" s="5" t="inlineStr">
         <is>
           <t>单设备策略切换</t>
         </is>
       </c>
-      <c r="D78" s="5" t="inlineStr">
+      <c r="D82" s="5" t="inlineStr">
         <is>
           <t>验证蓝牙设备可从禁止接入恢复为允许接入</t>
         </is>
       </c>
-      <c r="E78" s="5" t="inlineStr">
+      <c r="E82" s="5" t="inlineStr">
         <is>
           <t>目标蓝牙设备当前策略为禁止接入</t>
         </is>
       </c>
-      <c r="F78" s="5" t="inlineStr">
+      <c r="F82" s="5" t="inlineStr">
         <is>
           <t>1. 进入黑白名单页签
 2. 将目标蓝牙设备策略切换为允许接入</t>
         </is>
       </c>
-      <c r="G78" s="5" t="inlineStr">
+      <c r="G82" s="5" t="inlineStr">
         <is>
           <t>1. 页面提示策略修改成功或状态更新
 2. 目标蓝牙设备当前策略显示为允许接入</t>
         </is>
       </c>
-      <c r="H78" s="5" t="n"/>
-      <c r="I78" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J78" s="7" t="inlineStr">
+      <c r="H82" s="5" t="n"/>
+      <c r="I82" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J82" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/viewmodels/PeripheralPolicyViewModel.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="79" ht="42.75" customHeight="1" s="1">
-      <c r="A79" s="4" t="inlineStr">
+    <row r="83" ht="28.5" customHeight="1" s="1">
+      <c r="A83" s="4" t="inlineStr">
         <is>
           <t>PER-025</t>
         </is>
       </c>
-      <c r="B79" s="5" t="inlineStr">
+      <c r="B83" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C79" s="5" t="inlineStr">
+      <c r="C83" s="5" t="inlineStr">
         <is>
           <t>USB接口策略</t>
         </is>
       </c>
-      <c r="D79" s="5" t="inlineStr">
+      <c r="D83" s="5" t="inlineStr">
         <is>
           <t>验证 USB 接口策略下发失败时 Select 从禁用回滚到启用</t>
         </is>
       </c>
-      <c r="E79" s="5" t="inlineStr">
+      <c r="E83" s="5" t="inlineStr">
         <is>
           <t>USB 接口当前状态为 `启用`，已构造接口策略下发失败场景</t>
         </is>
       </c>
-      <c r="F79" s="5" t="inlineStr">
+      <c r="F83" s="5" t="inlineStr">
         <is>
           <t>1. 进入接口管控页签
 2. 将 USB 接口策略从 `启用` 改为 `禁用`
 3. 触发下发失败</t>
         </is>
       </c>
-      <c r="G79" s="5" t="inlineStr">
+      <c r="G83" s="5" t="inlineStr">
         <is>
           <t>1. 页面展示失败提示
 2. Select 选项回滚到 `启用`
 3. 界面状态与真实系统状态保持一致</t>
         </is>
       </c>
-      <c r="H79" s="5" t="n"/>
-      <c r="I79" s="7" t="inlineStr">
+      <c r="H83" s="5" t="n"/>
+      <c r="I83" s="7" t="inlineStr">
         <is>
           <t>不补UT</t>
         </is>
       </c>
-      <c r="J79" s="7" t="inlineStr">
+      <c r="J83" s="7" t="inlineStr">
         <is>
           <t>Select 显示回滚属于 AsyncSelectRow 组件本地交互状态，不进入本轮 UT 补充范围。</t>
         </is>
       </c>
     </row>
-    <row r="80" ht="42.75" customHeight="1" s="1">
-      <c r="A80" s="4" t="inlineStr">
+    <row r="84" ht="28.5" customHeight="1" s="1">
+      <c r="A84" s="4" t="inlineStr">
         <is>
           <t>PER-026</t>
         </is>
       </c>
-      <c r="B80" s="5" t="inlineStr">
+      <c r="B84" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C80" s="5" t="inlineStr">
+      <c r="C84" s="5" t="inlineStr">
         <is>
           <t>USB存储策略</t>
         </is>
       </c>
-      <c r="D80" s="5" t="inlineStr">
+      <c r="D84" s="5" t="inlineStr">
         <is>
           <t>验证 USB 存储策略下发失败时 Select 从只读回滚到读写</t>
         </is>
       </c>
-      <c r="E80" s="5" t="inlineStr">
+      <c r="E84" s="5" t="inlineStr">
         <is>
           <t>USB 存储当前策略为 `读写`，已构造存储策略下发失败场景</t>
         </is>
       </c>
-      <c r="F80" s="5" t="inlineStr">
+      <c r="F84" s="5" t="inlineStr">
         <is>
           <t>1. 进入接口管控页签
 2. 将 USB 存储策略从 `读写` 改为 `只读`
 3. 触发下发失败</t>
         </is>
       </c>
-      <c r="G80" s="5" t="inlineStr">
+      <c r="G84" s="5" t="inlineStr">
         <is>
           <t>1. 页面展示失败提示
 2. Select 选项回滚到 `读写`
 3. 界面状态与真实系统状态保持一致</t>
         </is>
       </c>
-      <c r="H80" s="5" t="n"/>
-      <c r="I80" s="7" t="inlineStr">
+      <c r="H84" s="5" t="n"/>
+      <c r="I84" s="7" t="inlineStr">
         <is>
           <t>不补UT</t>
         </is>
       </c>
-      <c r="J80" s="7" t="inlineStr">
+      <c r="J84" s="7" t="inlineStr">
         <is>
           <t>Select 显示回滚属于 AsyncSelectRow 组件本地交互状态，不进入本轮 UT 补充范围。</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="42.75" customHeight="1" s="1">
-      <c r="A81" s="4" t="inlineStr">
+    <row r="85" ht="42.75" customHeight="1" s="1">
+      <c r="A85" s="4" t="inlineStr">
         <is>
           <t>PER-027</t>
         </is>
       </c>
-      <c r="B81" s="5" t="inlineStr">
+      <c r="B85" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C81" s="5" t="inlineStr">
+      <c r="C85" s="5" t="inlineStr">
         <is>
           <t>单设备策略切换</t>
         </is>
       </c>
-      <c r="D81" s="5" t="inlineStr">
+      <c r="D85" s="5" t="inlineStr">
         <is>
           <t>验证黑白名单策略下发失败时 Select 从禁止接入回滚到允许接入</t>
         </is>
       </c>
-      <c r="E81" s="5" t="inlineStr">
+      <c r="E85" s="5" t="inlineStr">
         <is>
           <t>黑白名单中存在可管理设备，当前策略为 `允许接入`，已构造策略下发失败场景</t>
         </is>
       </c>
-      <c r="F81" s="5" t="inlineStr">
+      <c r="F85" s="5" t="inlineStr">
         <is>
           <t>1. 进入黑白名单页签
 2. 将目标设备策略从 `允许接入` 改为 `禁止接入`
 3. 触发下发失败</t>
         </is>
       </c>
-      <c r="G81" s="5" t="inlineStr">
+      <c r="G85" s="5" t="inlineStr">
         <is>
           <t>1. 页面展示失败提示
 2. Select 选项回滚到 `允许接入`
 3. 列表中的当前策略与真实系统状态保持一致</t>
         </is>
       </c>
-      <c r="H81" s="5" t="n"/>
-      <c r="I81" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J81" s="7" t="inlineStr">
+      <c r="H85" s="5" t="n"/>
+      <c r="I85" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J85" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/viewmodels/PeripheralPolicyViewModel.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="82" ht="57" customHeight="1" s="1">
-      <c r="A82" s="4" t="inlineStr">
+    <row r="86" ht="42.75" customHeight="1" s="1">
+      <c r="A86" s="4" t="inlineStr">
         <is>
           <t>PER-028</t>
         </is>
       </c>
-      <c r="B82" s="5" t="inlineStr">
+      <c r="B86" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C82" s="5" t="inlineStr">
+      <c r="C86" s="5" t="inlineStr">
         <is>
           <t>首次连接自动拉黑</t>
         </is>
       </c>
-      <c r="D82" s="5" t="inlineStr">
+      <c r="D86" s="5" t="inlineStr">
         <is>
           <t>验证 USB 设备首次连接且本地无策略时自动下发禁止接入并写入黑名单</t>
         </is>
       </c>
-      <c r="E82" s="5" t="inlineStr">
+      <c r="E86" s="5" t="inlineStr">
         <is>
           <t>应用已激活企业管理员，USB 设备此前未存在本地 allow / deny 策略</t>
         </is>
       </c>
-      <c r="F82" s="5" t="inlineStr">
+      <c r="F86" s="5" t="inlineStr">
         <is>
           <t>1. 进入外设管理页
 2. 插入首次接入的 USB 设备
 3. 切换到设备连接记录和黑白名单页签</t>
         </is>
       </c>
-      <c r="G82" s="5" t="inlineStr">
+      <c r="G86" s="5" t="inlineStr">
         <is>
           <t>1. 系统同步下发 USB 禁止接入策略
 2. 下发成功后本地黑白名单新增该设备 deny 策略
 3. 本次连接记录展示禁止接入及首次自动拉黑说明</t>
         </is>
       </c>
-      <c r="H82" s="5" t="n"/>
-      <c r="I82" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J82" s="7" t="inlineStr">
+      <c r="H86" s="5" t="n"/>
+      <c r="I86" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J86" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/peripheral/connection-record-usb-consumer.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="83" ht="28.5" customHeight="1" s="1">
-      <c r="A83" s="4" t="inlineStr">
+    <row r="87" ht="42.75" customHeight="1" s="1">
+      <c r="A87" s="4" t="inlineStr">
         <is>
           <t>PER-029</t>
         </is>
       </c>
-      <c r="B83" s="5" t="inlineStr">
+      <c r="B87" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C83" s="5" t="inlineStr">
+      <c r="C87" s="5" t="inlineStr">
         <is>
           <t>首次连接自动拉黑</t>
         </is>
       </c>
-      <c r="D83" s="5" t="inlineStr">
+      <c r="D87" s="5" t="inlineStr">
         <is>
           <t>验证蓝牙设备首次连接且本地无策略时按 MAC 自动下发禁止接入并写入黑名单</t>
         </is>
       </c>
-      <c r="E83" s="5" t="inlineStr">
+      <c r="E87" s="5" t="inlineStr">
         <is>
           <t>应用已激活企业管理员，蓝牙设备此前未存在本地 allow / deny 策略</t>
         </is>
       </c>
-      <c r="F83" s="5" t="inlineStr">
+      <c r="F87" s="5" t="inlineStr">
         <is>
           <t>1. 进入外设管理页
 2. 连接首次接入的蓝牙设备
 3. 切换到设备连接记录和黑白名单页签</t>
         </is>
       </c>
-      <c r="G83" s="5" t="inlineStr">
+      <c r="G87" s="5" t="inlineStr">
         <is>
           <t>1. 系统按规范化 MAC 同步下发蓝牙禁止接入策略
 2. 下发成功后本地黑白名单新增该设备 deny 策略
 3. 本次连接记录展示禁止接入及首次自动拉黑说明</t>
         </is>
       </c>
-      <c r="H83" s="5" t="n"/>
-      <c r="I83" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J83" s="7" t="inlineStr">
+      <c r="H87" s="5" t="n"/>
+      <c r="I87" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J87" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/peripheral/connection-record-bluetooth-acl-consumer.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="28.5" customHeight="1" s="1">
-      <c r="A84" s="4" t="inlineStr">
+    <row r="88" ht="42.75" customHeight="1" s="1">
+      <c r="A88" s="4" t="inlineStr">
         <is>
           <t>PER-030</t>
         </is>
       </c>
-      <c r="B84" s="5" t="inlineStr">
+      <c r="B88" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C84" s="5" t="inlineStr">
+      <c r="C88" s="5" t="inlineStr">
         <is>
           <t>首次连接自动拉黑</t>
         </is>
       </c>
-      <c r="D84" s="5" t="inlineStr">
+      <c r="D88" s="5" t="inlineStr">
         <is>
           <t>验证已有允许接入策略的设备再次连接时不被自动改回禁止接入</t>
         </is>
       </c>
-      <c r="E84" s="5" t="inlineStr">
+      <c r="E88" s="5" t="inlineStr">
         <is>
           <t>目标 USB 或蓝牙设备已由管理员设置为允许接入</t>
         </is>
       </c>
-      <c r="F84" s="5" t="inlineStr">
+      <c r="F88" s="5" t="inlineStr">
         <is>
           <t>1. 连接目标设备
 2. 查看黑白名单策略和连接记录</t>
         </is>
       </c>
-      <c r="G84" s="5" t="inlineStr">
+      <c r="G88" s="5" t="inlineStr">
         <is>
           <t>1. 运行时不自动覆盖既有 allow 策略
 2. 不重复下发 deny
 3. 设备策略仍显示允许接入</t>
         </is>
       </c>
-      <c r="H84" s="5" t="n"/>
-      <c r="I84" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J84" s="7" t="inlineStr">
+      <c r="H88" s="5" t="n"/>
+      <c r="I88" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J88" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/peripheral/connection-record-usb-consumer.test.ets；entry/src/test/peripheral/connection-record-bluetooth-acl-consumer.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="85" ht="42.75" customHeight="1" s="1">
-      <c r="A85" s="4" t="inlineStr">
+    <row r="89" ht="42.75" customHeight="1" s="1">
+      <c r="A89" s="4" t="inlineStr">
         <is>
           <t>PER-031</t>
         </is>
       </c>
-      <c r="B85" s="5" t="inlineStr">
+      <c r="B89" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C85" s="5" t="inlineStr">
+      <c r="C89" s="5" t="inlineStr">
         <is>
           <t>首次连接自动拉黑</t>
         </is>
       </c>
-      <c r="D85" s="5" t="inlineStr">
+      <c r="D89" s="5" t="inlineStr">
         <is>
           <t>验证已有禁止接入策略的设备再次连接时不重复下发策略</t>
         </is>
       </c>
-      <c r="E85" s="5" t="inlineStr">
+      <c r="E89" s="5" t="inlineStr">
         <is>
           <t>目标 USB 或蓝牙设备已存在禁止接入策略</t>
         </is>
       </c>
-      <c r="F85" s="5" t="inlineStr">
+      <c r="F89" s="5" t="inlineStr">
         <is>
           <t>1. 再次连接目标设备
 2. 查看黑白名单策略和连接记录</t>
         </is>
       </c>
-      <c r="G85" s="5" t="inlineStr">
+      <c r="G89" s="5" t="inlineStr">
         <is>
           <t>1. 运行时识别已有 deny 策略并跳过自动下发
 2. 本地黑白名单不产生重复记录
 3. 连接记录仍展示禁止接入语义</t>
         </is>
       </c>
-      <c r="H85" s="5" t="n"/>
-      <c r="I85" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J85" s="7" t="inlineStr">
+      <c r="H89" s="5" t="n"/>
+      <c r="I89" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J89" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/peripheral/connection-record-usb-consumer.test.ets；entry/src/test/peripheral/connection-record-bluetooth-acl-consumer.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="86" ht="42.75" customHeight="1" s="1">
-      <c r="A86" s="4" t="inlineStr">
+    <row r="90" ht="28.5" customHeight="1" s="1">
+      <c r="A90" s="4" t="inlineStr">
         <is>
           <t>PER-032</t>
         </is>
       </c>
-      <c r="B86" s="5" t="inlineStr">
+      <c r="B90" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C86" s="5" t="inlineStr">
+      <c r="C90" s="5" t="inlineStr">
         <is>
           <t>首次连接自动拉黑</t>
         </is>
       </c>
-      <c r="D86" s="5" t="inlineStr">
+      <c r="D90" s="5" t="inlineStr">
         <is>
           <t>验证自动拉黑系统下发失败时不保存本地黑名单策略，连接记录仍保留失败原因</t>
         </is>
       </c>
-      <c r="E86" s="5" t="inlineStr">
+      <c r="E90" s="5" t="inlineStr">
         <is>
           <t>已构造 USB 或蓝牙自动拉黑系统下发失败场景</t>
         </is>
       </c>
-      <c r="F86" s="5" t="inlineStr">
+      <c r="F90" s="5" t="inlineStr">
         <is>
           <t>1. 连接首次接入设备
 2. 触发系统策略下发失败
 3. 查看黑白名单和连接记录详情</t>
         </is>
       </c>
-      <c r="G86" s="5" t="inlineStr">
+      <c r="G90" s="5" t="inlineStr">
         <is>
           <t>1. 本地黑白名单不保存 deny 策略
 2. 连接记录仍正常落库
 3. 记录详情保留自动拉黑失败原因</t>
         </is>
       </c>
-      <c r="H86" s="5" t="n"/>
-      <c r="I86" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J86" s="7" t="inlineStr">
+      <c r="H90" s="5" t="n"/>
+      <c r="I90" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J90" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/peripheral/connection-record-usb-consumer.test.ets；entry/src/test/peripheral/connection-record-bluetooth-acl-consumer.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="42.75" customHeight="1" s="1">
-      <c r="A87" s="4" t="inlineStr">
+    <row r="91" ht="28.5" customHeight="1" s="1">
+      <c r="A91" s="4" t="inlineStr">
         <is>
           <t>PER-033</t>
         </is>
       </c>
-      <c r="B87" s="5" t="inlineStr">
+      <c r="B91" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C87" s="5" t="inlineStr">
+      <c r="C91" s="5" t="inlineStr">
         <is>
           <t>首次连接自动拉黑</t>
         </is>
       </c>
-      <c r="D87" s="5" t="inlineStr">
+      <c r="D91" s="5" t="inlineStr">
         <is>
           <t>验证 USB 存储总策略为禁止访问时，首次接入 USB 存储设备不自动下发设备级黑名单</t>
         </is>
       </c>
-      <c r="E87" s="5" t="inlineStr">
+      <c r="E91" s="5" t="inlineStr">
         <is>
           <t>应用已激活企业管理员，USB 存储策略当前为 `禁止访问`，目标 U 盘此前未存在本地 allow / deny 策略</t>
         </is>
       </c>
-      <c r="F87" s="5" t="inlineStr">
+      <c r="F91" s="5" t="inlineStr">
         <is>
           <t>1. 进入接口管控页签，将 USB 存储策略设置为 `禁止访问`
 2. 插入首次接入的 USB 存储设备
 3. 查看设备连接记录和黑白名单页签</t>
         </is>
       </c>
-      <c r="G87" s="5" t="inlineStr">
+      <c r="G91" s="5" t="inlineStr">
         <is>
           <t>1. 本次连接记录正常落库并展示 USB 存储已禁用
 2. 不下发设备级 deny
 3. 本地黑白名单不新增该 U 盘 deny 策略</t>
         </is>
       </c>
-      <c r="H87" s="5" t="n"/>
-      <c r="I87" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J87" s="7" t="inlineStr">
+      <c r="H91" s="5" t="n"/>
+      <c r="I91" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J91" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/peripheral/connection-record-usb-consumer.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="88" ht="42.75" customHeight="1" s="1">
-      <c r="A88" s="4" t="inlineStr">
+    <row r="92" ht="42.75" customHeight="1" s="1">
+      <c r="A92" s="4" t="inlineStr">
         <is>
           <t>PER-034</t>
         </is>
       </c>
-      <c r="B88" s="5" t="inlineStr">
+      <c r="B92" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C88" s="5" t="inlineStr">
+      <c r="C92" s="5" t="inlineStr">
         <is>
           <t>设备连接记录</t>
         </is>
       </c>
-      <c r="D88" s="5" t="inlineStr">
+      <c r="D92" s="5" t="inlineStr">
         <is>
           <t>验证 USB 存储只读且本地存在禁止接入策略时，连接记录优先展示禁止接入</t>
         </is>
       </c>
-      <c r="E88" s="5" t="inlineStr">
+      <c r="E92" s="5" t="inlineStr">
         <is>
           <t>USB 存储策略当前为 `只读`，目标 U 盘已存在本地 deny 策略</t>
         </is>
       </c>
-      <c r="F88" s="5" t="inlineStr">
+      <c r="F92" s="5" t="inlineStr">
         <is>
           <t>1. 进入接口管控页签，确认 USB 存储策略为 `只读`
 2. 保持目标 U 盘在黑白名单中为 `禁止接入`
 3. 插入目标 U 盘并查看设备连接记录</t>
         </is>
       </c>
-      <c r="G88" s="5" t="inlineStr">
+      <c r="G92" s="5" t="inlineStr">
         <is>
           <t>1. 本次连接记录正常落库
 2. 记录策略展示为已禁用或禁止接入
 3. 命中类型优先体现单设备禁止接入，不被 USB 存储只读覆盖</t>
         </is>
       </c>
-      <c r="H88" s="5" t="n"/>
-      <c r="I88" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J88" s="7" t="inlineStr">
+      <c r="H92" s="5" t="n"/>
+      <c r="I92" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J92" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/peripheral/connection-record-usb-consumer.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="42.75" customHeight="1" s="1">
-      <c r="A89" s="4" t="inlineStr">
+    <row r="93" ht="42.75" customHeight="1" s="1">
+      <c r="A93" s="4" t="inlineStr">
         <is>
           <t>PER-035</t>
         </is>
       </c>
-      <c r="B89" s="5" t="inlineStr">
+      <c r="B93" s="5" t="inlineStr">
         <is>
           <t>外设管理</t>
         </is>
       </c>
-      <c r="C89" s="5" t="inlineStr">
+      <c r="C93" s="5" t="inlineStr">
         <is>
           <t>单设备策略切换</t>
         </is>
       </c>
-      <c r="D89" s="5" t="inlineStr">
+      <c r="D93" s="5" t="inlineStr">
         <is>
           <t>验证 USB 存储总策略为禁止访问时，黑白名单不允许将 USB 存储设备切换为禁止接入</t>
         </is>
       </c>
-      <c r="E89" s="5" t="inlineStr">
+      <c r="E93" s="5" t="inlineStr">
         <is>
           <t>USB 存储策略当前为 `禁止访问`，黑白名单中存在目标 USB 存储设备</t>
         </is>
       </c>
-      <c r="F89" s="5" t="inlineStr">
+      <c r="F93" s="5" t="inlineStr">
         <is>
           <t>1. 进入接口管控页签，确认 USB 存储策略为 `禁止访问`
 2. 进入黑白名单页签
 3. 将目标 USB 存储设备从 `允许接入` 切换为 `禁止接入`</t>
         </is>
       </c>
-      <c r="G89" s="5" t="inlineStr">
+      <c r="G93" s="5" t="inlineStr">
         <is>
           <t>1. 系统下发被拦截并返回 USB 存储账户级冲突
 2. 本地黑白名单不写入 deny 策略
 3. 页面保持原本单设备策略状态并展示失败提示</t>
         </is>
       </c>
-      <c r="H89" s="5" t="n"/>
-      <c r="I89" s="7" t="inlineStr">
+      <c r="H93" s="5" t="n"/>
+      <c r="I93" s="7" t="inlineStr">
         <is>
           <t>不补UT</t>
         </is>
       </c>
-      <c r="J89" s="7" t="inlineStr">
+      <c r="J93" s="7" t="inlineStr">
         <is>
           <t>该场景依赖系统 MDM USB 存储账户级策略读取与 USB 设备策略下发，当前 UT 环境无法稳定 mock 系统命名空间对象；保留为手工验收场景，相关连接记录行为由 entry/src/test/peripheral/connection-record-usb-consumer.test.ets 覆盖。</t>
         </is>
       </c>
     </row>
-    <row r="90" ht="28.5" customHeight="1" s="1">
-      <c r="A90" s="4" t="inlineStr">
+    <row r="94" ht="28.5" customHeight="1" s="1">
+      <c r="A94" s="4" t="inlineStr">
         <is>
           <t>ID-001</t>
         </is>
       </c>
-      <c r="B90" s="5" t="inlineStr">
+      <c r="B94" s="5" t="inlineStr">
         <is>
           <t>身份鉴别</t>
         </is>
       </c>
-      <c r="C90" s="5" t="inlineStr">
+      <c r="C94" s="5" t="inlineStr">
         <is>
           <t>口令复杂度策略</t>
         </is>
       </c>
-      <c r="D90" s="5" t="inlineStr">
+      <c r="D94" s="5" t="inlineStr">
         <is>
           <t>验证保存口令复杂度策略：最小长度 8，大写/小写/数字开启，特殊字符关闭</t>
         </is>
       </c>
-      <c r="E90" s="5" t="inlineStr">
+      <c r="E94" s="5" t="inlineStr">
         <is>
           <t>应用已激活企业管理员</t>
         </is>
       </c>
-      <c r="F90" s="5" t="inlineStr">
+      <c r="F94" s="5" t="inlineStr">
         <is>
           <t>1. 进入身份鉴别页
 2. 设置最小长度为 `8`
@@ -5682,102 +5889,102 @@
 5. 点击保存身份鉴别配置</t>
         </is>
       </c>
-      <c r="G90" s="5" t="inlineStr">
+      <c r="G94" s="5" t="inlineStr">
         <is>
           <t>1. 页面提示身份鉴别配置已保存
 2. 系统设置中策略显示与配置一致</t>
         </is>
       </c>
-      <c r="H90" s="5" t="n"/>
-      <c r="I90" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J90" s="7" t="inlineStr">
+      <c r="H94" s="5" t="n"/>
+      <c r="I94" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J94" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/identity/settings-viewmodel.test.ets；entry/src/test/identity/service.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="91" ht="28.5" customHeight="1" s="1">
-      <c r="A91" s="4" t="inlineStr">
+    <row r="95" ht="28.5" customHeight="1" s="1">
+      <c r="A95" s="4" t="inlineStr">
         <is>
           <t>ID-002</t>
         </is>
       </c>
-      <c r="B91" s="5" t="inlineStr">
+      <c r="B95" s="5" t="inlineStr">
         <is>
           <t>身份鉴别</t>
         </is>
       </c>
-      <c r="C91" s="5" t="inlineStr">
+      <c r="C95" s="5" t="inlineStr">
         <is>
           <t>密码有效期策略</t>
         </is>
       </c>
-      <c r="D91" s="5" t="inlineStr">
+      <c r="D95" s="5" t="inlineStr">
         <is>
           <t>验证将密码有效期设置为 180 天后保存成功</t>
         </is>
       </c>
-      <c r="E91" s="5" t="inlineStr">
+      <c r="E95" s="5" t="inlineStr">
         <is>
           <t>应用已激活企业管理员</t>
         </is>
       </c>
-      <c r="F91" s="5" t="inlineStr">
+      <c r="F95" s="5" t="inlineStr">
         <is>
           <t>1. 进入身份鉴别页
 2. 选择密码有效期 `180天`
 3. 点击保存</t>
         </is>
       </c>
-      <c r="G91" s="5" t="inlineStr">
+      <c r="G95" s="5" t="inlineStr">
         <is>
           <t>1. 页面提示保存成功
 2. 再次进入页面可回显 `180天`</t>
         </is>
       </c>
-      <c r="H91" s="5" t="n"/>
-      <c r="I91" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J91" s="7" t="inlineStr">
+      <c r="H95" s="5" t="n"/>
+      <c r="I95" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J95" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/identity/settings-viewmodel.test.ets；entry/src/test/identity/service.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="92" ht="42.75" customHeight="1" s="1">
-      <c r="A92" s="4" t="inlineStr">
+    <row r="96" ht="28.5" customHeight="1" s="1">
+      <c r="A96" s="4" t="inlineStr">
         <is>
           <t>ID-003</t>
         </is>
       </c>
-      <c r="B92" s="5" t="inlineStr">
+      <c r="B96" s="5" t="inlineStr">
         <is>
           <t>身份鉴别</t>
         </is>
       </c>
-      <c r="C92" s="5" t="inlineStr">
+      <c r="C96" s="5" t="inlineStr">
         <is>
           <t>密码有效期策略</t>
         </is>
       </c>
-      <c r="D92" s="5" t="inlineStr">
+      <c r="D96" s="5" t="inlineStr">
         <is>
           <t>验证将自定义密码有效期设置为 30 天后保存成功</t>
         </is>
       </c>
-      <c r="E92" s="5" t="inlineStr">
+      <c r="E96" s="5" t="inlineStr">
         <is>
           <t>应用已激活企业管理员</t>
         </is>
       </c>
-      <c r="F92" s="5" t="inlineStr">
+      <c r="F96" s="5" t="inlineStr">
         <is>
           <t>1. 进入身份鉴别页
 2. 选择自定义有效期
@@ -5785,51 +5992,51 @@
 4. 点击保存</t>
         </is>
       </c>
-      <c r="G92" s="5" t="inlineStr">
+      <c r="G96" s="5" t="inlineStr">
         <is>
           <t>1. 页面提示保存成功
 2. 再次进入页面可回显 `30天`</t>
         </is>
       </c>
-      <c r="H92" s="5" t="n"/>
-      <c r="I92" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J92" s="7" t="inlineStr">
+      <c r="H96" s="5" t="n"/>
+      <c r="I96" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J96" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/identity/settings-viewmodel.test.ets；entry/src/test/identity/service.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="93" ht="42.75" customHeight="1" s="1">
-      <c r="A93" s="4" t="inlineStr">
+    <row r="97" ht="28.5" customHeight="1" s="1">
+      <c r="A97" s="4" t="inlineStr">
         <is>
           <t>ID-004</t>
         </is>
       </c>
-      <c r="B93" s="5" t="inlineStr">
+      <c r="B97" s="5" t="inlineStr">
         <is>
           <t>身份鉴别</t>
         </is>
       </c>
-      <c r="C93" s="5" t="inlineStr">
+      <c r="C97" s="5" t="inlineStr">
         <is>
           <t>输入参数校验</t>
         </is>
       </c>
-      <c r="D93" s="5" t="inlineStr">
+      <c r="D97" s="5" t="inlineStr">
         <is>
           <t>验证自定义密码有效期非法字符被过滤，空值保存时被拦截</t>
         </is>
       </c>
-      <c r="E93" s="5" t="inlineStr">
+      <c r="E97" s="5" t="inlineStr">
         <is>
           <t>已选择自定义有效期</t>
         </is>
       </c>
-      <c r="F93" s="5" t="inlineStr">
+      <c r="F97" s="5" t="inlineStr">
         <is>
           <t>1. 选择自定义有效期
 2. 尝试输入 abc、-1 等非法字符
@@ -5837,1077 +6044,1077 @@
 4. 点击保存</t>
         </is>
       </c>
-      <c r="G93" s="5" t="inlineStr">
+      <c r="G97" s="5" t="inlineStr">
         <is>
           <t>1. 非法字符不会保留在输入框中，或仅保留数字字符
 2. 自定义有效期为空时点击保存，页面提示请输入非负整数天数
 3. 未通过校验时不下发策略</t>
         </is>
       </c>
-      <c r="H93" s="5" t="n"/>
-      <c r="I93" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J93" s="7" t="inlineStr">
+      <c r="H97" s="5" t="n"/>
+      <c r="I97" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J97" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/identity/settings-viewmodel.test.ets；entry/src/test/identity/service.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="94" ht="28.5" customHeight="1" s="1">
-      <c r="A94" s="4" t="inlineStr">
+    <row r="98" ht="28.5" customHeight="1" s="1">
+      <c r="A98" s="4" t="inlineStr">
         <is>
           <t>ID-007</t>
         </is>
       </c>
-      <c r="B94" s="5" t="inlineStr">
+      <c r="B98" s="5" t="inlineStr">
         <is>
           <t>身份鉴别</t>
         </is>
       </c>
-      <c r="C94" s="5" t="inlineStr">
+      <c r="C98" s="5" t="inlineStr">
         <is>
           <t>策略保存</t>
         </is>
       </c>
-      <c r="D94" s="5" t="inlineStr">
+      <c r="D98" s="5" t="inlineStr">
         <is>
           <t>验证自定义密码有效期输入 0 天时触发风险提示</t>
         </is>
       </c>
-      <c r="E94" s="5" t="inlineStr">
+      <c r="E98" s="5" t="inlineStr">
         <is>
           <t>应用已激活企业管理员，已选择自定义有效期</t>
         </is>
       </c>
-      <c r="F94" s="5" t="inlineStr">
+      <c r="F98" s="5" t="inlineStr">
         <is>
           <t>1. 输入 `0`
 2. 点击保存</t>
         </is>
       </c>
-      <c r="G94" s="5" t="inlineStr">
+      <c r="G98" s="5" t="inlineStr">
         <is>
           <t>1. 页面弹出风险提示
 2. 用户确认前不直接保存策略</t>
         </is>
       </c>
-      <c r="H94" s="5" t="n"/>
-      <c r="I94" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J94" s="7" t="inlineStr">
+      <c r="H98" s="5" t="n"/>
+      <c r="I98" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J98" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/identity/settings-viewmodel.test.ets；entry/src/test/identity/service.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="95" ht="28.5" customHeight="1" s="1">
-      <c r="A95" s="4" t="inlineStr">
+    <row r="99" ht="28.5" customHeight="1" s="1">
+      <c r="A99" s="4" t="inlineStr">
         <is>
           <t>SET-002</t>
         </is>
       </c>
-      <c r="B95" s="5" t="inlineStr">
+      <c r="B99" s="5" t="inlineStr">
         <is>
           <t>工具设置</t>
         </is>
       </c>
-      <c r="C95" s="5" t="inlineStr">
+      <c r="C99" s="5" t="inlineStr">
         <is>
           <t>启动认证开关</t>
         </is>
       </c>
-      <c r="D95" s="5" t="inlineStr">
+      <c r="D99" s="5" t="inlineStr">
         <is>
           <t>验证关闭启动时身份校验后保存成功</t>
         </is>
       </c>
-      <c r="E95" s="5" t="inlineStr">
+      <c r="E99" s="5" t="inlineStr">
         <is>
           <t>启动时身份校验当前已开启</t>
         </is>
       </c>
-      <c r="F95" s="5" t="inlineStr">
+      <c r="F99" s="5" t="inlineStr">
         <is>
           <t>1. 进入工具设置页
 2. 关闭启动时身份校验
 3. 点击保存设置</t>
         </is>
       </c>
-      <c r="G95" s="5" t="inlineStr">
+      <c r="G99" s="5" t="inlineStr">
         <is>
           <t>1. 页面提示工具设置已保存
 2. 重启应用后不再要求启动认证</t>
         </is>
       </c>
-      <c r="H95" s="5" t="n"/>
-      <c r="I95" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J95" s="7" t="inlineStr">
+      <c r="H99" s="5" t="n"/>
+      <c r="I99" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J99" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/tool-settings/viewmodel.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="96" ht="28.5" customHeight="1" s="1">
-      <c r="A96" s="4" t="inlineStr">
+    <row r="100" ht="42.75" customHeight="1" s="1">
+      <c r="A100" s="4" t="inlineStr">
         <is>
           <t>SET-003</t>
         </is>
       </c>
-      <c r="B96" s="5" t="inlineStr">
+      <c r="B100" s="5" t="inlineStr">
         <is>
           <t>工具设置</t>
         </is>
       </c>
-      <c r="C96" s="5" t="inlineStr">
+      <c r="C100" s="5" t="inlineStr">
         <is>
           <t>认证方式选择</t>
         </is>
       </c>
-      <c r="D96" s="5" t="inlineStr">
+      <c r="D100" s="5" t="inlineStr">
         <is>
           <t>验证选择 PIN 认证方式后保存成功</t>
         </is>
       </c>
-      <c r="E96" s="5" t="inlineStr">
+      <c r="E100" s="5" t="inlineStr">
         <is>
           <t>启动时身份校验已开启，系统 PIN 可用</t>
         </is>
       </c>
-      <c r="F96" s="5" t="inlineStr">
+      <c r="F100" s="5" t="inlineStr">
         <is>
           <t>1. 进入工具设置页
 2. 选择 `PIN` 认证方式
 3. 点击保存设置</t>
         </is>
       </c>
-      <c r="G96" s="5" t="inlineStr">
+      <c r="G100" s="5" t="inlineStr">
         <is>
           <t>1. 页面提示保存成功
 2. 重启应用后按 PIN 方式进行校验</t>
         </is>
       </c>
-      <c r="H96" s="5" t="n"/>
-      <c r="I96" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J96" s="7" t="inlineStr">
+      <c r="H100" s="5" t="n"/>
+      <c r="I100" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J100" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/tool-settings/viewmodel.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="97" ht="28.5" customHeight="1" s="1">
-      <c r="A97" s="4" t="inlineStr">
+    <row r="101" ht="28.5" customHeight="1" s="1">
+      <c r="A101" s="4" t="inlineStr">
         <is>
           <t>SET-004</t>
         </is>
       </c>
-      <c r="B97" s="5" t="inlineStr">
+      <c r="B101" s="5" t="inlineStr">
         <is>
           <t>工具设置</t>
         </is>
       </c>
-      <c r="C97" s="5" t="inlineStr">
+      <c r="C101" s="5" t="inlineStr">
         <is>
           <t>认证方式选择</t>
         </is>
       </c>
-      <c r="D97" s="5" t="inlineStr">
+      <c r="D101" s="5" t="inlineStr">
         <is>
           <t>验证选择指纹认证方式后保存成功</t>
         </is>
       </c>
-      <c r="E97" s="5" t="inlineStr">
+      <c r="E101" s="5" t="inlineStr">
         <is>
           <t>设备已录入指纹且系统指纹认证可用</t>
         </is>
       </c>
-      <c r="F97" s="5" t="inlineStr">
+      <c r="F101" s="5" t="inlineStr">
         <is>
           <t>1. 进入工具设置页
 2. 选择 `指纹` 认证方式
 3. 点击保存设置</t>
         </is>
       </c>
-      <c r="G97" s="5" t="inlineStr">
+      <c r="G101" s="5" t="inlineStr">
         <is>
           <t>1. 页面提示保存成功
 2. 重启应用后按指纹方式进行校验</t>
         </is>
       </c>
-      <c r="H97" s="5" t="n"/>
-      <c r="I97" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J97" s="7" t="inlineStr">
+      <c r="H101" s="5" t="n"/>
+      <c r="I101" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J101" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/tool-settings/viewmodel.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="98" ht="28.5" customHeight="1" s="1">
-      <c r="A98" s="4" t="inlineStr">
+    <row r="102" ht="42.75" customHeight="1" s="1">
+      <c r="A102" s="4" t="inlineStr">
         <is>
           <t>SET-005</t>
         </is>
       </c>
-      <c r="B98" s="5" t="inlineStr">
+      <c r="B102" s="5" t="inlineStr">
         <is>
           <t>工具设置</t>
         </is>
       </c>
-      <c r="C98" s="5" t="inlineStr">
+      <c r="C102" s="5" t="inlineStr">
         <is>
           <t>无变更保存</t>
         </is>
       </c>
-      <c r="D98" s="5" t="inlineStr">
+      <c r="D102" s="5" t="inlineStr">
         <is>
           <t>验证未修改设置时保存按钮不可点击</t>
         </is>
       </c>
-      <c r="E98" s="5" t="inlineStr">
+      <c r="E102" s="5" t="inlineStr">
         <is>
           <t>进入工具设置页且不修改任何配置</t>
         </is>
       </c>
-      <c r="F98" s="5" t="inlineStr">
+      <c r="F102" s="5" t="inlineStr">
         <is>
           <t>1. 进入工具设置页
 2. 不做任何修改
 3. 观察保存按钮状态</t>
         </is>
       </c>
-      <c r="G98" s="5" t="inlineStr">
+      <c r="G102" s="5" t="inlineStr">
         <is>
           <t>1. 保存按钮保持不可点击状态
 2. 页面不触发保存动作</t>
         </is>
       </c>
-      <c r="H98" s="5" t="n"/>
-      <c r="I98" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J98" s="7" t="inlineStr">
+      <c r="H102" s="5" t="n"/>
+      <c r="I102" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J102" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/tool-settings/viewmodel.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="99" ht="28.5" customHeight="1" s="1">
-      <c r="A99" s="4" t="inlineStr">
+    <row r="103" ht="42.75" customHeight="1" s="1">
+      <c r="A103" s="4" t="inlineStr">
         <is>
           <t>SET-006</t>
         </is>
       </c>
-      <c r="B99" s="5" t="inlineStr">
+      <c r="B103" s="5" t="inlineStr">
         <is>
           <t>工具设置</t>
         </is>
       </c>
-      <c r="C99" s="5" t="inlineStr">
+      <c r="C103" s="5" t="inlineStr">
         <is>
           <t>认证方式不可用提示</t>
         </is>
       </c>
-      <c r="D99" s="5" t="inlineStr">
+      <c r="D103" s="5" t="inlineStr">
         <is>
           <t>验证选择当前设备不可用的认证方式时出现不可用确认提示</t>
         </is>
       </c>
-      <c r="E99" s="5" t="inlineStr">
+      <c r="E103" s="5" t="inlineStr">
         <is>
           <t>当前设备存在一种不可用认证方式</t>
         </is>
       </c>
-      <c r="F99" s="5" t="inlineStr">
+      <c r="F103" s="5" t="inlineStr">
         <is>
           <t>1. 进入工具设置页
 2. 选择当前设备不可用的认证方式
 3. 点击保存设置</t>
         </is>
       </c>
-      <c r="G99" s="5" t="inlineStr">
+      <c r="G103" s="5" t="inlineStr">
         <is>
           <t>1. 页面弹出认证方式不可用提示
 2. 用户确认前不直接保存</t>
         </is>
       </c>
-      <c r="H99" s="5" t="n"/>
-      <c r="I99" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J99" s="7" t="inlineStr">
+      <c r="H103" s="5" t="n"/>
+      <c r="I103" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J103" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/tool-settings/viewmodel.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="100" ht="42.75" customHeight="1" s="1">
-      <c r="A100" s="4" t="inlineStr">
+    <row r="104" ht="42.75" customHeight="1" s="1">
+      <c r="A104" s="4" t="inlineStr">
         <is>
           <t>SET-007</t>
         </is>
       </c>
-      <c r="B100" s="5" t="inlineStr">
+      <c r="B104" s="5" t="inlineStr">
         <is>
           <t>工具设置</t>
         </is>
       </c>
-      <c r="C100" s="5" t="inlineStr">
+      <c r="C104" s="5" t="inlineStr">
         <is>
           <t>修改密码入口</t>
         </is>
       </c>
-      <c r="D100" s="5" t="inlineStr">
+      <c r="D104" s="5" t="inlineStr">
         <is>
           <t>验证点击修改密码后拉起系统“生物识别和密码”页面</t>
         </is>
       </c>
-      <c r="E100" s="5" t="inlineStr">
+      <c r="E104" s="5" t="inlineStr">
         <is>
           <t>系统设置能力可用</t>
         </is>
       </c>
-      <c r="F100" s="5" t="inlineStr">
+      <c r="F104" s="5" t="inlineStr">
         <is>
           <t>1. 进入工具设置页
 2. 点击 `修改密码`</t>
         </is>
       </c>
-      <c r="G100" s="5" t="inlineStr">
+      <c r="G104" s="5" t="inlineStr">
         <is>
           <t>1. 成功拉起系统 `生物识别和密码` 页面
 2. 拉起失败时展示明确失败提示</t>
         </is>
       </c>
-      <c r="H100" s="5" t="n"/>
-      <c r="I100" s="7" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J100" s="7" t="inlineStr">
+      <c r="H104" s="5" t="n"/>
+      <c r="I104" s="7" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J104" s="7" t="inlineStr">
         <is>
           <t>entry/src/test/tool-settings/viewmodel.test.ets；entry/src/test/tool-settings/system-settings-service.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="101" ht="28.5" customHeight="1" s="1">
-      <c r="A101" s="4" t="inlineStr">
+    <row r="105">
+      <c r="A105" s="4" t="inlineStr">
         <is>
           <t>HELP-001</t>
         </is>
       </c>
-      <c r="B101" s="5" t="inlineStr">
+      <c r="B105" s="5" t="inlineStr">
         <is>
           <t>帮助与反馈</t>
         </is>
       </c>
-      <c r="C101" s="5" t="inlineStr">
+      <c r="C105" s="5" t="inlineStr">
         <is>
           <t>页面展示</t>
         </is>
       </c>
-      <c r="D101" s="5" t="inlineStr">
+      <c r="D105" s="5" t="inlineStr">
         <is>
           <t>验证帮助与反馈页可正常打开</t>
         </is>
       </c>
-      <c r="E101" s="5" t="inlineStr">
+      <c r="E105" s="5" t="inlineStr">
         <is>
           <t>应用处于任一主页面</t>
         </is>
       </c>
-      <c r="F101" s="5" t="inlineStr">
+      <c r="F105" s="5" t="inlineStr">
         <is>
           <t>1. 打开右上角菜单
 2. 点击帮助与反馈</t>
         </is>
       </c>
-      <c r="G101" s="5" t="inlineStr">
+      <c r="G105" s="5" t="inlineStr">
         <is>
           <t>1. 成功进入帮助与反馈页
 2. 页面标题、说明正常展示</t>
         </is>
       </c>
-      <c r="H101" s="5" t="n"/>
-      <c r="I101" s="7" t="inlineStr">
+      <c r="H105" s="5" t="n"/>
+      <c r="I105" s="7" t="inlineStr">
         <is>
           <t>不补UT</t>
         </is>
       </c>
-      <c r="J101" s="7" t="inlineStr">
+      <c r="J105" s="7" t="inlineStr">
         <is>
           <t>页面打开属于页面渲染/导航场景，不进入本轮 UT 补充范围。</t>
         </is>
       </c>
     </row>
-    <row r="102" ht="42.75" customHeight="1" s="1">
-      <c r="A102" s="4" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="4" t="inlineStr">
         <is>
           <t>HELP-002</t>
         </is>
       </c>
-      <c r="B102" s="5" t="inlineStr">
+      <c r="B106" s="5" t="inlineStr">
         <is>
           <t>帮助与反馈</t>
         </is>
       </c>
-      <c r="C102" s="5" t="inlineStr">
+      <c r="C106" s="5" t="inlineStr">
         <is>
           <t>使用指南展示</t>
         </is>
       </c>
-      <c r="D102" s="5" t="inlineStr">
+      <c r="D106" s="5" t="inlineStr">
         <is>
           <t>验证使用指南内容展示完整</t>
         </is>
       </c>
-      <c r="E102" s="5" t="inlineStr">
+      <c r="E106" s="5" t="inlineStr">
         <is>
           <t>已进入帮助与反馈页</t>
         </is>
       </c>
-      <c r="F102" s="5" t="inlineStr">
+      <c r="F106" s="5" t="inlineStr">
         <is>
           <t>1. 查看使用指南区域</t>
         </is>
       </c>
-      <c r="G102" s="5" t="inlineStr">
+      <c r="G106" s="5" t="inlineStr">
         <is>
           <t>1. 展示防火墙、外设、身份鉴别、工具设置、主题模式等指南项
 2. 文案无截断</t>
         </is>
       </c>
-      <c r="H102" s="5" t="n"/>
-      <c r="I102" s="7" t="inlineStr">
+      <c r="H106" s="5" t="n"/>
+      <c r="I106" s="7" t="inlineStr">
         <is>
           <t>不补UT</t>
         </is>
       </c>
-      <c r="J102" s="7" t="inlineStr">
+      <c r="J106" s="7" t="inlineStr">
         <is>
           <t>使用指南展示属于页面展示场景；文案结构已有基础 UT，不再补。</t>
         </is>
       </c>
     </row>
-    <row r="103" ht="42.75" customHeight="1" s="1">
-      <c r="A103" s="4" t="inlineStr">
+    <row r="107">
+      <c r="A107" s="4" t="inlineStr">
         <is>
           <t>HELP-003</t>
         </is>
       </c>
-      <c r="B103" s="5" t="inlineStr">
+      <c r="B107" s="5" t="inlineStr">
         <is>
           <t>帮助与反馈</t>
         </is>
       </c>
-      <c r="C103" s="5" t="inlineStr">
+      <c r="C107" s="5" t="inlineStr">
         <is>
           <t>FAQ展开收起</t>
         </is>
       </c>
-      <c r="D103" s="5" t="inlineStr">
+      <c r="D107" s="5" t="inlineStr">
         <is>
           <t>验证 FAQ 可以展开和收起</t>
         </is>
       </c>
-      <c r="E103" s="5" t="inlineStr">
+      <c r="E107" s="5" t="inlineStr">
         <is>
           <t>已进入帮助与反馈页</t>
         </is>
       </c>
-      <c r="F103" s="5" t="inlineStr">
+      <c r="F107" s="5" t="inlineStr">
         <is>
           <t>1. 点击任一 FAQ 展开按钮
 2. 再次点击收起按钮</t>
         </is>
       </c>
-      <c r="G103" s="5" t="inlineStr">
+      <c r="G107" s="5" t="inlineStr">
         <is>
           <t>1. 首次点击展示答案
 2. 再次点击隐藏答案
 3. 按钮文案在展开和收起间切换</t>
         </is>
       </c>
-      <c r="H103" s="5" t="n"/>
-      <c r="I103" s="7" t="inlineStr">
+      <c r="H107" s="5" t="n"/>
+      <c r="I107" s="7" t="inlineStr">
         <is>
           <t>不补UT</t>
         </is>
       </c>
-      <c r="J103" s="7" t="inlineStr">
+      <c r="J107" s="7" t="inlineStr">
         <is>
           <t>FAQ 展开收起属于页面交互场景，不进入本轮 UT 补充范围。</t>
         </is>
       </c>
     </row>
-    <row r="104" ht="42.75" customHeight="1" s="1">
-      <c r="A104" s="4" t="inlineStr">
+    <row r="108">
+      <c r="A108" s="4" t="inlineStr">
         <is>
           <t>HELP-004</t>
         </is>
       </c>
-      <c r="B104" s="5" t="inlineStr">
+      <c r="B108" s="5" t="inlineStr">
         <is>
           <t>帮助与反馈</t>
         </is>
       </c>
-      <c r="C104" s="5" t="inlineStr">
+      <c r="C108" s="5" t="inlineStr">
         <is>
           <t>联系方式展示</t>
         </is>
       </c>
-      <c r="D104" s="5" t="inlineStr">
+      <c r="D108" s="5" t="inlineStr">
         <is>
           <t>验证联系与反馈信息展示正确</t>
         </is>
       </c>
-      <c r="E104" s="5" t="inlineStr">
+      <c r="E108" s="5" t="inlineStr">
         <is>
           <t>已进入帮助与反馈页</t>
         </is>
       </c>
-      <c r="F104" s="5" t="inlineStr">
+      <c r="F108" s="5" t="inlineStr">
         <is>
           <t>1. 查看联系与反馈区域</t>
         </is>
       </c>
-      <c r="G104" s="5" t="inlineStr">
+      <c r="G108" s="5" t="inlineStr">
         <is>
           <t>1. 展示反馈邮箱
 2. 邮箱内容为 `consumer@huawei.com`</t>
         </is>
       </c>
-      <c r="H104" s="5" t="n"/>
-      <c r="I104" s="7" t="inlineStr">
+      <c r="H108" s="5" t="n"/>
+      <c r="I108" s="7" t="inlineStr">
         <is>
           <t>不补UT</t>
         </is>
       </c>
-      <c r="J104" s="7" t="inlineStr">
+      <c r="J108" s="7" t="inlineStr">
         <is>
           <t>联系方式展示属于页面展示场景；文案结构已有基础 UT，不再补。</t>
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="4" t="inlineStr">
+    <row r="109">
+      <c r="A109" s="4" t="inlineStr">
         <is>
           <t>NAV-001</t>
         </is>
       </c>
-      <c r="B105" s="5" t="inlineStr">
+      <c r="B109" s="5" t="inlineStr">
         <is>
           <t>全局导航与主题</t>
         </is>
       </c>
-      <c r="C105" s="5" t="inlineStr">
+      <c r="C109" s="5" t="inlineStr">
         <is>
           <t>侧边栏导航</t>
         </is>
       </c>
-      <c r="D105" s="5" t="inlineStr">
+      <c r="D109" s="5" t="inlineStr">
         <is>
           <t>验证侧边栏可以进入所有主模块</t>
         </is>
       </c>
-      <c r="E105" s="5" t="inlineStr">
+      <c r="E109" s="5" t="inlineStr">
         <is>
           <t>应用处于安全总览页</t>
         </is>
       </c>
-      <c r="F105" s="5" t="inlineStr">
+      <c r="F109" s="5" t="inlineStr">
         <is>
           <t>1. 依次点击侧边栏防火墙、日志、外设、身份鉴别、工具设置</t>
         </is>
       </c>
-      <c r="G105" s="5" t="inlineStr">
+      <c r="G109" s="5" t="inlineStr">
         <is>
           <t>1. 每次均进入对应页面
 2. 侧边栏选中态同步更新</t>
         </is>
       </c>
-      <c r="H105" s="5" t="n"/>
-      <c r="I105" s="7" t="inlineStr">
+      <c r="H109" s="5" t="n"/>
+      <c r="I109" s="7" t="inlineStr">
         <is>
           <t>不补UT</t>
         </is>
       </c>
-      <c r="J105" s="7" t="inlineStr">
+      <c r="J109" s="7" t="inlineStr">
         <is>
           <t>导航、弹窗或菜单交互属于 UI/ohosTest 范围，不进入本轮 UT 补充范围。</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="4" t="inlineStr">
+    <row r="110">
+      <c r="A110" s="4" t="inlineStr">
         <is>
           <t>NAV-002</t>
         </is>
       </c>
-      <c r="B106" s="5" t="inlineStr">
+      <c r="B110" s="5" t="inlineStr">
         <is>
           <t>全局导航与主题</t>
         </is>
       </c>
-      <c r="C106" s="5" t="inlineStr">
+      <c r="C110" s="5" t="inlineStr">
         <is>
           <t>返回按钮</t>
         </is>
       </c>
-      <c r="D106" s="5" t="inlineStr">
+      <c r="D110" s="5" t="inlineStr">
         <is>
           <t>验证子页面返回按钮回到安全总览或上级页面</t>
         </is>
       </c>
-      <c r="E106" s="5" t="inlineStr">
+      <c r="E110" s="5" t="inlineStr">
         <is>
           <t>已进入任一子页面</t>
         </is>
       </c>
-      <c r="F106" s="5" t="inlineStr">
+      <c r="F110" s="5" t="inlineStr">
         <is>
           <t>1. 点击页面左上角返回按钮</t>
         </is>
       </c>
-      <c r="G106" s="5" t="inlineStr">
+      <c r="G110" s="5" t="inlineStr">
         <is>
           <t>1. 返回到预期上级页面
 2. 页面不闪退、不空白</t>
         </is>
       </c>
-      <c r="H106" s="5" t="n"/>
-      <c r="I106" s="7" t="inlineStr">
+      <c r="H110" s="5" t="n"/>
+      <c r="I110" s="7" t="inlineStr">
         <is>
           <t>不补UT</t>
         </is>
       </c>
-      <c r="J106" s="7" t="inlineStr">
+      <c r="J110" s="7" t="inlineStr">
         <is>
           <t>导航、弹窗或菜单交互属于 UI/ohosTest 范围，不进入本轮 UT 补充范围。</t>
         </is>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" s="0" t="inlineStr">
+    <row r="111">
+      <c r="A111" s="0" t="inlineStr">
         <is>
           <t>NAV-003</t>
         </is>
       </c>
-      <c r="B107" s="0" t="inlineStr">
+      <c r="B111" s="0" t="inlineStr">
         <is>
           <t>全局导航与主题</t>
         </is>
       </c>
-      <c r="C107" s="0" t="inlineStr">
+      <c r="C111" s="0" t="inlineStr">
         <is>
           <t>主题菜单</t>
         </is>
       </c>
-      <c r="D107" s="0" t="inlineStr">
+      <c r="D111" s="0" t="inlineStr">
         <is>
           <t>验证右上角主题菜单可以打开和关闭</t>
         </is>
       </c>
-      <c r="E107" s="0" t="inlineStr">
+      <c r="E111" s="0" t="inlineStr">
         <is>
           <t>应用处于任一页面</t>
         </is>
       </c>
-      <c r="F107" s="0" t="inlineStr">
+      <c r="F111" s="0" t="inlineStr">
         <is>
           <t>1. 点击右上角菜单按钮
 2. 点击页面空白区域</t>
         </is>
       </c>
-      <c r="G107" s="0" t="inlineStr">
+      <c r="G111" s="0" t="inlineStr">
         <is>
           <t>1. 菜单打开后展示主题、帮助、关于等入口
 2. 点击空白区域后菜单关闭</t>
         </is>
       </c>
-      <c r="H107" s="0" t="n"/>
-      <c r="I107" s="0" t="inlineStr">
+      <c r="H111" s="0" t="n"/>
+      <c r="I111" s="0" t="inlineStr">
         <is>
           <t>不补UT</t>
         </is>
       </c>
-      <c r="J107" s="0" t="inlineStr">
+      <c r="J111" s="0" t="inlineStr">
         <is>
           <t>导航、弹窗或菜单交互属于 UI/ohosTest 范围，不进入本轮 UT 补充范围。</t>
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" s="0" t="inlineStr">
+    <row r="112">
+      <c r="A112" s="0" t="inlineStr">
         <is>
           <t>NAV-004</t>
         </is>
       </c>
-      <c r="B108" s="0" t="inlineStr">
+      <c r="B112" s="0" t="inlineStr">
         <is>
           <t>全局导航与主题</t>
         </is>
       </c>
-      <c r="C108" s="0" t="inlineStr">
+      <c r="C112" s="0" t="inlineStr">
         <is>
           <t>深浅色切换</t>
         </is>
       </c>
-      <c r="D108" s="0" t="inlineStr">
+      <c r="D112" s="0" t="inlineStr">
         <is>
           <t>验证浅色模式切换生效</t>
         </is>
       </c>
-      <c r="E108" s="0" t="inlineStr">
+      <c r="E112" s="0" t="inlineStr">
         <is>
           <t>应用可正常打开</t>
         </is>
       </c>
-      <c r="F108" s="0" t="inlineStr">
+      <c r="F112" s="0" t="inlineStr">
         <is>
           <t>1. 打开右上角菜单
 2. 选择浅色模式</t>
         </is>
       </c>
-      <c r="G108" s="0" t="inlineStr">
+      <c r="G112" s="0" t="inlineStr">
         <is>
           <t>1. 页面切换为浅色主题
 2. 顶部窗口按钮样式同步浅色配置</t>
         </is>
       </c>
-      <c r="H108" s="0" t="n"/>
-      <c r="I108" s="0" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J108" s="0" t="inlineStr">
+      <c r="H112" s="0" t="n"/>
+      <c r="I112" s="0" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J112" s="0" t="inlineStr">
         <is>
           <t>entry/src/test/theme/theme-manager.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="109">
-      <c r="A109" s="0" t="inlineStr">
+    <row r="113">
+      <c r="A113" s="0" t="inlineStr">
         <is>
           <t>NAV-005</t>
         </is>
       </c>
-      <c r="B109" s="0" t="inlineStr">
+      <c r="B113" s="0" t="inlineStr">
         <is>
           <t>全局导航与主题</t>
         </is>
       </c>
-      <c r="C109" s="0" t="inlineStr">
+      <c r="C113" s="0" t="inlineStr">
         <is>
           <t>深浅色切换</t>
         </is>
       </c>
-      <c r="D109" s="0" t="inlineStr">
+      <c r="D113" s="0" t="inlineStr">
         <is>
           <t>验证深色模式切换生效</t>
         </is>
       </c>
-      <c r="E109" s="0" t="inlineStr">
+      <c r="E113" s="0" t="inlineStr">
         <is>
           <t>应用可正常打开</t>
         </is>
       </c>
-      <c r="F109" s="0" t="inlineStr">
+      <c r="F113" s="0" t="inlineStr">
         <is>
           <t>1. 打开右上角菜单
 2. 选择深色模式</t>
         </is>
       </c>
-      <c r="G109" s="0" t="inlineStr">
+      <c r="G113" s="0" t="inlineStr">
         <is>
           <t>1. 页面切换为深色主题
 2. 页面文字、背景、图标对比度正常</t>
         </is>
       </c>
-      <c r="H109" s="0" t="n"/>
-      <c r="I109" s="0" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J109" s="0" t="inlineStr">
+      <c r="H113" s="0" t="n"/>
+      <c r="I113" s="0" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J113" s="0" t="inlineStr">
         <is>
           <t>entry/src/test/theme/theme-manager.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" s="0" t="inlineStr">
+    <row r="114">
+      <c r="A114" s="0" t="inlineStr">
         <is>
           <t>NAV-006</t>
         </is>
       </c>
-      <c r="B110" s="0" t="inlineStr">
+      <c r="B114" s="0" t="inlineStr">
         <is>
           <t>全局导航与主题</t>
         </is>
       </c>
-      <c r="C110" s="0" t="inlineStr">
+      <c r="C114" s="0" t="inlineStr">
         <is>
           <t>深浅色切换</t>
         </is>
       </c>
-      <c r="D110" s="0" t="inlineStr">
+      <c r="D114" s="0" t="inlineStr">
         <is>
           <t>验证跟随系统模式保存和回显</t>
         </is>
       </c>
-      <c r="E110" s="0" t="inlineStr">
+      <c r="E114" s="0" t="inlineStr">
         <is>
           <t>系统主题可切换</t>
         </is>
       </c>
-      <c r="F110" s="0" t="inlineStr">
+      <c r="F114" s="0" t="inlineStr">
         <is>
           <t>1. 打开右上角菜单
 2. 选择跟随系统
 3. 重启应用</t>
         </is>
       </c>
-      <c r="G110" s="0" t="inlineStr">
+      <c r="G114" s="0" t="inlineStr">
         <is>
           <t>1. 应用主题跟随系统当前主题
 2. 菜单中当前选项回显正确</t>
         </is>
       </c>
-      <c r="H110" s="0" t="n"/>
-      <c r="I110" s="0" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J110" s="0" t="inlineStr">
+      <c r="H114" s="0" t="n"/>
+      <c r="I114" s="0" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J114" s="0" t="inlineStr">
         <is>
           <t>entry/src/test/theme/theme-manager.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="111">
-      <c r="A111" s="0" t="inlineStr">
+    <row r="115">
+      <c r="A115" s="0" t="inlineStr">
         <is>
           <t>NAV-007</t>
         </is>
       </c>
-      <c r="B111" s="0" t="inlineStr">
+      <c r="B115" s="0" t="inlineStr">
         <is>
           <t>全局导航与主题</t>
         </is>
       </c>
-      <c r="C111" s="0" t="inlineStr">
+      <c r="C115" s="0" t="inlineStr">
         <is>
           <t>关于弹窗</t>
         </is>
       </c>
-      <c r="D111" s="0" t="inlineStr">
+      <c r="D115" s="0" t="inlineStr">
         <is>
           <t>验证关于弹窗展示应用信息</t>
         </is>
       </c>
-      <c r="E111" s="0" t="inlineStr">
+      <c r="E115" s="0" t="inlineStr">
         <is>
           <t>应用处于任一页面</t>
         </is>
       </c>
-      <c r="F111" s="0" t="inlineStr">
+      <c r="F115" s="0" t="inlineStr">
         <is>
           <t>1. 打开右上角菜单
 2. 点击关于</t>
         </is>
       </c>
-      <c r="G111" s="0" t="inlineStr">
+      <c r="G115" s="0" t="inlineStr">
         <is>
           <t>1. 弹窗展示应用名称、版本和版权信息
 2. 点击确定后弹窗关闭</t>
         </is>
       </c>
-      <c r="H111" s="0" t="n"/>
-      <c r="I111" s="0" t="inlineStr">
+      <c r="H115" s="0" t="n"/>
+      <c r="I115" s="0" t="inlineStr">
         <is>
           <t>不补UT</t>
         </is>
       </c>
-      <c r="J111" s="0" t="inlineStr">
+      <c r="J115" s="0" t="inlineStr">
         <is>
           <t>导航、弹窗或菜单交互属于 UI/ohosTest 范围，不进入本轮 UT 补充范围。</t>
         </is>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" s="0" t="inlineStr">
+    <row r="116">
+      <c r="A116" s="0" t="inlineStr">
         <is>
           <t>SYS-005</t>
         </is>
       </c>
-      <c r="B112" s="0" t="inlineStr">
+      <c r="B116" s="0" t="inlineStr">
         <is>
           <t>系统集成基础</t>
         </is>
       </c>
-      <c r="C112" s="0" t="inlineStr">
+      <c r="C116" s="0" t="inlineStr">
         <is>
           <t>导出文件能力</t>
         </is>
       </c>
-      <c r="D112" s="0" t="inlineStr">
+      <c r="D116" s="0" t="inlineStr">
         <is>
           <t>验证通用 CSV 导出能力正常</t>
         </is>
       </c>
-      <c r="E112" s="0" t="inlineStr">
+      <c r="E116" s="0" t="inlineStr">
         <is>
           <t>日志或外设存在可导出数据</t>
         </is>
       </c>
-      <c r="F112" s="0" t="inlineStr">
+      <c r="F116" s="0" t="inlineStr">
         <is>
           <t>1. 在任一支持导出的页面点击导出
 2. 打开导出文件</t>
         </is>
       </c>
-      <c r="G112" s="0" t="inlineStr">
+      <c r="G116" s="0" t="inlineStr">
         <is>
           <t>1. 文件保存成功
 2. 文件编码和表头正确
 3. 中文内容不乱码</t>
         </is>
       </c>
-      <c r="H112" s="0" t="n"/>
-      <c r="I112" s="0" t="inlineStr">
-        <is>
-          <t>已有UT覆盖</t>
-        </is>
-      </c>
-      <c r="J112" s="0" t="inlineStr">
+      <c r="H116" s="0" t="n"/>
+      <c r="I116" s="0" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J116" s="0" t="inlineStr">
         <is>
           <t>entry/src/test/common/csv-file-export-service.test.ets；entry/src/test/log-manage/export-service.test.ets</t>
         </is>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" s="0" t="inlineStr">
+    <row r="117">
+      <c r="A117" s="0" t="inlineStr">
         <is>
           <t>SYS-006</t>
         </is>
       </c>
-      <c r="B113" s="0" t="inlineStr">
+      <c r="B117" s="0" t="inlineStr">
         <is>
           <t>系统集成基础</t>
         </is>
       </c>
-      <c r="C113" s="0" t="inlineStr">
+      <c r="C117" s="0" t="inlineStr">
         <is>
           <t>本地存储能力</t>
         </is>
       </c>
-      <c r="D113" s="0" t="inlineStr">
+      <c r="D117" s="0" t="inlineStr">
         <is>
           <t>验证设置类配置重启后可恢复</t>
         </is>
       </c>
-      <c r="E113" s="0" t="inlineStr">
+      <c r="E117" s="0" t="inlineStr">
         <is>
           <t>已修改工具设置或日志存储设置</t>
         </is>
       </c>
-      <c r="F113" s="0" t="inlineStr">
+      <c r="F117" s="0" t="inlineStr">
         <is>
           <t>1. 保存配置
 2. 关闭并重启应用
 3. 重新进入对应页面</t>
         </is>
       </c>
-      <c r="G113" s="0" t="inlineStr">
+      <c r="G117" s="0" t="inlineStr">
         <is>
           <t>1. 页面回显上次保存配置
 2. 无默认值覆盖已保存配置</t>
         </is>
       </c>
-      <c r="H113" s="0" t="n"/>
-      <c r="I113" s="0" t="inlineStr">
+      <c r="H117" s="0" t="n"/>
+      <c r="I117" s="0" t="inlineStr">
         <is>
           <t>不补UT</t>
         </is>
       </c>
-      <c r="J113" s="0" t="inlineStr">
+      <c r="J117" s="0" t="inlineStr">
         <is>
           <t>重启后恢复属于集成语义；存储读写已有基础 UT，不再补。</t>
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="0" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="0" t="inlineStr">
         <is>
           <t>SYS-007</t>
         </is>
       </c>
-      <c r="B114" s="0" t="inlineStr">
+      <c r="B118" s="0" t="inlineStr">
         <is>
           <t>系统集成基础</t>
         </is>
       </c>
-      <c r="C114" s="0" t="inlineStr">
+      <c r="C118" s="0" t="inlineStr">
         <is>
           <t>应用恢复</t>
         </is>
       </c>
-      <c r="D114" s="0" t="inlineStr">
+      <c r="D118" s="0" t="inlineStr">
         <is>
           <t>验证应用前后台切换后当前页面状态正常</t>
         </is>
       </c>
-      <c r="E114" s="0" t="inlineStr">
+      <c r="E118" s="0" t="inlineStr">
         <is>
           <t>应用已打开任一业务页面</t>
         </is>
       </c>
-      <c r="F114" s="0" t="inlineStr">
+      <c r="F118" s="0" t="inlineStr">
         <is>
           <t>1. 将应用切到后台
 2. 等待 5 秒
 3. 恢复到前台</t>
         </is>
       </c>
-      <c r="G114" s="0" t="inlineStr">
+      <c r="G118" s="0" t="inlineStr">
         <is>
           <t>1. 当前页面仍可操作
 2. 关键数据自动刷新或保持一致
 3. 无崩溃</t>
         </is>
       </c>
-      <c r="H114" s="0" t="n"/>
-      <c r="I114" s="0" t="inlineStr">
+      <c r="H118" s="0" t="n"/>
+      <c r="I118" s="0" t="inlineStr">
         <is>
           <t>不补UT</t>
         </is>
       </c>
-      <c r="J114" s="0" t="inlineStr">
+      <c r="J118" s="0" t="inlineStr">
         <is>
           <t>前后台切换属于应用生命周期集成场景，不进入本轮 UT 补充范围。</t>
         </is>

</xml_diff>

<commit_message>
test: cover log import exception branches
</commit_message>
<xml_diff>
--- a/docs/04-测试文档/手工测试用例/测试用例基线.xlsx
+++ b/docs/04-测试文档/手工测试用例/测试用例基线.xlsx
@@ -3968,12 +3968,12 @@
       <c r="H56" s="5" t="n"/>
       <c r="I56" s="8" t="inlineStr">
         <is>
-          <t>待补UT</t>
+          <t>已有UT覆盖</t>
         </is>
       </c>
       <c r="J56" s="8" t="inlineStr">
         <is>
-          <t>待补 entry/src/test/log-manage/import-service.test.ets：覆盖 pickZip() 返回 null 与 pickDirectory() 返回 null。</t>
+          <t>entry/src/test/log-manage/import-service.test.ets</t>
         </is>
       </c>
     </row>
@@ -4019,12 +4019,12 @@
       <c r="H57" s="5" t="n"/>
       <c r="I57" s="8" t="inlineStr">
         <is>
-          <t>待补UT</t>
+          <t>已有UT覆盖</t>
         </is>
       </c>
       <c r="J57" s="8" t="inlineStr">
         <is>
-          <t>待补 entry/src/test/log-manage/import-service.test.ets：覆盖规则 parse() 抛异常时 failedEntryCount 增加且流程不中断。</t>
+          <t>entry/src/test/log-manage/import-service.test.ets</t>
         </is>
       </c>
     </row>
@@ -4070,12 +4070,12 @@
       <c r="H58" s="5" t="n"/>
       <c r="I58" s="8" t="inlineStr">
         <is>
-          <t>待补UT</t>
+          <t>已有UT覆盖</t>
         </is>
       </c>
       <c r="J58" s="8" t="inlineStr">
         <is>
-          <t>待补 entry/src/test/log-manage/import-service.test.ets：覆盖 appendEntries() 返回失败时结果为 save_failed。</t>
+          <t>entry/src/test/log-manage/import-service.test.ets</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: sync firewall test baseline cases
</commit_message>
<xml_diff>
--- a/docs/04-测试文档/手工测试用例/测试用例基线.xlsx
+++ b/docs/04-测试文档/手工测试用例/测试用例基线.xlsx
@@ -564,7 +564,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -589,6 +589,9 @@
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1060,7 +1063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J120"/>
+  <dimension ref="A1:J127"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14" defaultRowHeight="13.5"/>
   <cols>
     <col width="9.25" customWidth="1" style="1" min="1" max="1"/>
@@ -7240,6 +7243,392 @@
         </is>
       </c>
     </row>
+    <row r="121">
+      <c r="A121" s="9" t="inlineStr">
+        <is>
+          <t>FW-033</t>
+        </is>
+      </c>
+      <c r="B121" s="9" t="inlineStr">
+        <is>
+          <t>防火墙管理</t>
+        </is>
+      </c>
+      <c r="C121" s="9" t="inlineStr">
+        <is>
+          <t>规则新增失败回滚</t>
+        </is>
+      </c>
+      <c r="D121" s="9" t="inlineStr">
+        <is>
+          <t>验证多用户新增规则时任一用户下发失败会回滚已成功下发的系统规则且不保存本地规则</t>
+        </is>
+      </c>
+      <c r="E121" s="9" t="inlineStr">
+        <is>
+          <t>防火墙开启，当前为自定义模式，至少存在两个可用目标用户，模拟其中一个用户系统规则下发失败</t>
+        </is>
+      </c>
+      <c r="F121" s="9" t="inlineStr">
+        <is>
+          <t>1. 进入防火墙规则详情页
+2. 点击新增规则
+3. 选择 IP 规则并选择多个目标用户
+4. 输入合法规则参数
+5. 点击保存
+6. 触发其中一个目标用户下发失败</t>
+        </is>
+      </c>
+      <c r="G121" s="9" t="inlineStr">
+        <is>
+          <t>1. 页面返回新增失败提示
+2. 已成功下发到系统的规则被删除回滚
+3. 本地不保存该规则 intent/deployment
+4. 刷新规则列表后不展示半成功规则</t>
+        </is>
+      </c>
+      <c r="H121" s="9" t="n"/>
+      <c r="I121" s="9" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J121" s="9" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/service.test.ets</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="9" t="inlineStr">
+        <is>
+          <t>FW-034</t>
+        </is>
+      </c>
+      <c r="B122" s="9" t="inlineStr">
+        <is>
+          <t>防火墙管理</t>
+        </is>
+      </c>
+      <c r="C122" s="9" t="inlineStr">
+        <is>
+          <t>规则编辑差量更新</t>
+        </is>
+      </c>
+      <c r="D122" s="9" t="inlineStr">
+        <is>
+          <t>验证编辑规则变更目标用户时按用户差量执行 update/add/remove 并保存新的 deployment 集合</t>
+        </is>
+      </c>
+      <c r="E122" s="9" t="inlineStr">
+        <is>
+          <t>已存在一条作用于多个用户的自定义规则，防火墙处于自定义模式</t>
+        </is>
+      </c>
+      <c r="F122" s="9" t="inlineStr">
+        <is>
+          <t>1. 进入防火墙规则详情页
+2. 编辑已有规则
+3. 保留一个原目标用户，新增一个目标用户，移除一个原目标用户
+4. 修改合法规则参数后保存</t>
+        </is>
+      </c>
+      <c r="G122" s="9" t="inlineStr">
+        <is>
+          <t>1. 保留用户的系统规则执行 update
+2. 新增用户执行 add
+3. 移除用户执行 remove
+4. 全部成功后保存新的 intent/deployment
+5. 列表展示更新后的目标用户范围</t>
+        </is>
+      </c>
+      <c r="H122" s="9" t="n"/>
+      <c r="I122" s="9" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J122" s="9" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/service.test.ets</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="9" t="inlineStr">
+        <is>
+          <t>FW-035</t>
+        </is>
+      </c>
+      <c r="B123" s="9" t="inlineStr">
+        <is>
+          <t>防火墙管理</t>
+        </is>
+      </c>
+      <c r="C123" s="9" t="inlineStr">
+        <is>
+          <t>规则编辑失败回滚</t>
+        </is>
+      </c>
+      <c r="D123" s="9" t="inlineStr">
+        <is>
+          <t>验证编辑规则时移除旧 deployment 失败会回滚已 update 和已 add 的系统动作并恢复本地 deployment</t>
+        </is>
+      </c>
+      <c r="E123" s="9" t="inlineStr">
+        <is>
+          <t>已存在一条作用于多个用户的自定义规则，模拟编辑过程中移除旧系统规则失败</t>
+        </is>
+      </c>
+      <c r="F123" s="9" t="inlineStr">
+        <is>
+          <t>1. 进入防火墙规则详情页
+2. 编辑已有规则并调整目标用户范围
+3. 触发保留用户 update 成功、新增用户 add 成功、移除用户 remove 失败
+4. 等待保存结果</t>
+        </is>
+      </c>
+      <c r="G123" s="9" t="inlineStr">
+        <is>
+          <t>1. 页面返回编辑失败提示
+2. 已 update 的保留用户规则恢复为旧规则
+3. 已 add 的新用户规则被删除
+4. 本地 intent 不提交新内容
+5. 本地 deployment 恢复为与系统实际状态一致的旧映射</t>
+        </is>
+      </c>
+      <c r="H123" s="9" t="n"/>
+      <c r="I123" s="9" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J123" s="9" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/service.test.ets</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="9" t="inlineStr">
+        <is>
+          <t>FW-036</t>
+        </is>
+      </c>
+      <c r="B124" s="9" t="inlineStr">
+        <is>
+          <t>防火墙管理</t>
+        </is>
+      </c>
+      <c r="C124" s="9" t="inlineStr">
+        <is>
+          <t>规则删除失败恢复</t>
+        </is>
+      </c>
+      <c r="D124" s="9" t="inlineStr">
+        <is>
+          <t>验证删除规则时部分系统规则删除失败会恢复已删除系统规则并保留本地 intent</t>
+        </is>
+      </c>
+      <c r="E124" s="9" t="inlineStr">
+        <is>
+          <t>已存在一条作用于多个用户的自定义规则，模拟其中一个系统规则删除失败</t>
+        </is>
+      </c>
+      <c r="F124" s="9" t="inlineStr">
+        <is>
+          <t>1. 进入防火墙规则详情页
+2. 点击删除已有规则
+3. 在确认弹窗中点击确定
+4. 触发部分目标用户系统规则删除失败</t>
+        </is>
+      </c>
+      <c r="G124" s="9" t="inlineStr">
+        <is>
+          <t>1. 页面返回删除失败提示
+2. 已成功删除的系统规则被 add 回恢复
+3. 本地 intent 保留
+4. 本地 deployment 刷新为恢复后的系统规则 ID
+5. 刷新后仍可追踪该规则</t>
+        </is>
+      </c>
+      <c r="H124" s="9" t="n"/>
+      <c r="I124" s="9" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J124" s="9" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/service.test.ets</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="9" t="inlineStr">
+        <is>
+          <t>FW-037</t>
+        </is>
+      </c>
+      <c r="B125" s="9" t="inlineStr">
+        <is>
+          <t>防火墙管理</t>
+        </is>
+      </c>
+      <c r="C125" s="9" t="inlineStr">
+        <is>
+          <t>DNS规则编辑替换</t>
+        </is>
+      </c>
+      <c r="D125" s="9" t="inlineStr">
+        <is>
+          <t>验证目标类型为 DNS 的编辑不调用系统 update 而是 remove 旧规则后 add 新规则并保存新的 systemRuleId</t>
+        </is>
+      </c>
+      <c r="E125" s="9" t="inlineStr">
+        <is>
+          <t>已存在一条 DNS 或待编辑为 DNS 的自定义规则，防火墙处于自定义模式</t>
+        </is>
+      </c>
+      <c r="F125" s="9" t="inlineStr">
+        <is>
+          <t>1. 进入防火墙规则详情页
+2. 编辑已有规则
+3. 将目标类型保存为 DNS 规则并填写合法主 DNS 和备用 DNS
+4. 点击保存</t>
+        </is>
+      </c>
+      <c r="G125" s="9" t="inlineStr">
+        <is>
+          <t>1. 保留用户不调用 updateNetFirewallRule
+2. 旧系统规则先 remove
+3. 新 DNS 系统规则再 add
+4. 本地 deployment 使用 add 返回的新 systemRuleId
+5. 列表展示 DNS 主地址和备用地址</t>
+        </is>
+      </c>
+      <c r="H125" s="9" t="n"/>
+      <c r="I125" s="9" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J125" s="9" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/service.test.ets</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="9" t="inlineStr">
+        <is>
+          <t>FW-038</t>
+        </is>
+      </c>
+      <c r="B126" s="9" t="inlineStr">
+        <is>
+          <t>防火墙管理</t>
+        </is>
+      </c>
+      <c r="C126" s="9" t="inlineStr">
+        <is>
+          <t>DNS规则替换失败恢复</t>
+        </is>
+      </c>
+      <c r="D126" s="9" t="inlineStr">
+        <is>
+          <t>验证 DNS 编辑 remove 旧规则后 add 新规则失败时会恢复旧 DNS deployment 且不保存新 intent</t>
+        </is>
+      </c>
+      <c r="E126" s="9" t="inlineStr">
+        <is>
+          <t>已存在一条 DNS 自定义规则，模拟 DNS 替换新增时系统返回重复或失败错误</t>
+        </is>
+      </c>
+      <c r="F126" s="9" t="inlineStr">
+        <is>
+          <t>1. 进入防火墙规则详情页
+2. 编辑已有 DNS 规则
+3. 修改 DNS 参数后保存
+4. 触发新 DNS 系统规则 add 失败</t>
+        </is>
+      </c>
+      <c r="G126" s="9" t="inlineStr">
+        <is>
+          <t>1. 页面返回 DNS 编辑失败或重复提示
+2. 已 remove 的旧 DNS 系统规则被 add 回恢复
+3. 本地不保存新 intent
+4. 本地 deployment 记录恢复后的 systemRuleId
+5. 刷新后仍展示旧 DNS 规则</t>
+        </is>
+      </c>
+      <c r="H126" s="9" t="n"/>
+      <c r="I126" s="9" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J126" s="9" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/service.test.ets</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="9" t="inlineStr">
+        <is>
+          <t>FW-039</t>
+        </is>
+      </c>
+      <c r="B127" s="9" t="inlineStr">
+        <is>
+          <t>防火墙管理</t>
+        </is>
+      </c>
+      <c r="C127" s="9" t="inlineStr">
+        <is>
+          <t>DNS转IP编辑</t>
+        </is>
+      </c>
+      <c r="D127" s="9" t="inlineStr">
+        <is>
+          <t>验证已有 DNS 规则编辑为 IP 规则时保留用户可原地 update 且 deployment 的 systemRuleId 保持不变</t>
+        </is>
+      </c>
+      <c r="E127" s="9" t="inlineStr">
+        <is>
+          <t>已存在一条 DNS 自定义规则，防火墙处于自定义模式</t>
+        </is>
+      </c>
+      <c r="F127" s="9" t="inlineStr">
+        <is>
+          <t>1. 进入防火墙规则详情页
+2. 编辑已有 DNS 规则
+3. 将规则类型改为 IP 规则
+4. 输入合法 IP、协议和端口参数
+5. 点击保存</t>
+        </is>
+      </c>
+      <c r="G127" s="9" t="inlineStr">
+        <is>
+          <t>1. 保留用户的系统规则执行 update
+2. 不删除并重建保留用户 deployment
+3. 本地 deployment 的 systemRuleId 保持不变
+4. 规则列表展示为更新后的 IP 规则</t>
+        </is>
+      </c>
+      <c r="H127" s="9" t="n"/>
+      <c r="I127" s="9" t="inlineStr">
+        <is>
+          <t>已有UT覆盖</t>
+        </is>
+      </c>
+      <c r="J127" s="9" t="inlineStr">
+        <is>
+          <t>entry/src/test/firewall/service.test.ets</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>